<commit_message>
Update source Excel spreadsheet for solution training configuration
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="581" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68312DA4-974D-4E7B-B3CC-8CD6D5A4210F}"/>
+  <xr:revisionPtr revIDLastSave="595" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E989119-29C8-4FA7-8930-E0AE81B1D66F}"/>
   <bookViews>
-    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="193">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -687,14 +687,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[내부]CONTRABASS 솔루션 딥다이브 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>신규입사자 온보딩</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>d</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -720,6 +712,26 @@
   </si>
   <si>
     <t>[고객사]VIOLA 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgBl5W8IGDwUTIwFI6v1QhpKAVl_Qdeq1lpOLvM8lgK3-Uw?e=pJejqh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgC6pWckq1-mSKTcy28l6wJPAWSFFsQxH39wxe-7v6r20r8?e=9Jnw5L</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부]CONTRABASS 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부]VIOLA 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[파트너사]VIOLA 소개 및 기능 교육</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1037,7 +1049,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1138,6 +1150,66 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1156,65 +1228,8 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1505,10 +1520,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="44"/>
+      <c r="C4" s="38"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1527,10 +1542,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="45"/>
+      <c r="C8" s="39"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -1576,18 +1591,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="47" t="s">
+      <c r="B3" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
+      <c r="C3" s="42"/>
+      <c r="D3" s="42"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -1748,7 +1763,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="43" t="s">
         <v>155</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -1757,117 +1772,117 @@
       <c r="D3" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="52" t="s">
+      <c r="F3" s="46" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="50"/>
+      <c r="B4" s="44"/>
       <c r="C4" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="F4" s="53"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="47"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="50"/>
+      <c r="B5" s="44"/>
       <c r="C5" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="56"/>
-      <c r="F5" s="53"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="47"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="50"/>
+      <c r="B6" s="44"/>
       <c r="C6" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="53"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="47"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="50"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="56"/>
-      <c r="F7" s="53"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="47"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="50"/>
+      <c r="B8" s="44"/>
       <c r="C8" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="56"/>
-      <c r="F8" s="53"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="47"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="50"/>
+      <c r="B9" s="44"/>
       <c r="C9" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="56"/>
-      <c r="F9" s="53"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="47"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="50"/>
+      <c r="B10" s="44"/>
       <c r="C10" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="56"/>
-      <c r="F10" s="53"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="47"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="50"/>
+      <c r="B11" s="44"/>
       <c r="C11" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="56"/>
-      <c r="F11" s="53"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="47"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="51"/>
+      <c r="B12" s="45"/>
       <c r="C12" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="57"/>
-      <c r="F12" s="54"/>
+      <c r="E12" s="51"/>
+      <c r="F12" s="48"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="52" t="s">
         <v>84</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -1876,114 +1891,114 @@
       <c r="D13" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="52" t="s">
+      <c r="E13" s="46" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="61" t="s">
+      <c r="F13" s="55" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="59"/>
+      <c r="B14" s="53"/>
       <c r="C14" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="53"/>
-      <c r="F14" s="62"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="56"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="59"/>
+      <c r="B15" s="53"/>
       <c r="C15" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="53"/>
-      <c r="F15" s="62"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="56"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="59"/>
+      <c r="B16" s="53"/>
       <c r="C16" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="53"/>
-      <c r="F16" s="62"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="56"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="59"/>
+      <c r="B17" s="53"/>
       <c r="C17" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="53"/>
-      <c r="F17" s="62"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="56"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="59"/>
+      <c r="B18" s="53"/>
       <c r="C18" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="53"/>
-      <c r="F18" s="62"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="56"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="59"/>
+      <c r="B19" s="53"/>
       <c r="C19" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="53"/>
-      <c r="F19" s="62"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="56"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="59"/>
+      <c r="B20" s="53"/>
       <c r="C20" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="53"/>
-      <c r="F20" s="62"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="56"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="59"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="53"/>
-      <c r="F21" s="62"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="56"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="60"/>
+      <c r="B22" s="54"/>
       <c r="C22" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="54"/>
-      <c r="F22" s="63"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="57"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="52" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="30" t="s">
@@ -1992,111 +2007,111 @@
       <c r="D23" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="52" t="s">
+      <c r="E23" s="46" t="s">
         <v>153</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="55" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="59"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E24" s="53"/>
-      <c r="F24" s="62"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="56"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="59"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E25" s="53"/>
-      <c r="F25" s="62"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="56"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="59"/>
+      <c r="B26" s="53"/>
       <c r="C26" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="E26" s="53"/>
-      <c r="F26" s="62"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="56"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="59"/>
+      <c r="B27" s="53"/>
       <c r="C27" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="E27" s="53"/>
-      <c r="F27" s="62"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="56"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="59"/>
+      <c r="B28" s="53"/>
       <c r="C28" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="53"/>
-      <c r="F28" s="62"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="56"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="59"/>
+      <c r="B29" s="53"/>
       <c r="C29" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="E29" s="53"/>
-      <c r="F29" s="62"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="56"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="59"/>
+      <c r="B30" s="53"/>
       <c r="C30" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="E30" s="53"/>
-      <c r="F30" s="62"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="56"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="59"/>
+      <c r="B31" s="53"/>
       <c r="C31" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="53"/>
-      <c r="F31" s="62"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="60"/>
+      <c r="B32" s="54"/>
       <c r="C32" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="54"/>
-      <c r="F32" s="63"/>
+      <c r="E32" s="48"/>
+      <c r="F32" s="57"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="5"/>
@@ -2159,30 +2174,30 @@
         <v>88</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>186</v>
-      </c>
-      <c r="G4" s="42" t="s">
+        <v>184</v>
+      </c>
+      <c r="G4" s="62" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="43"/>
+      <c r="H4" s="63"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="38" t="s">
+      <c r="B5" s="58" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="38" t="s">
+      <c r="C5" s="58" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="38" t="s">
+      <c r="D5" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="38" t="s">
+      <c r="E5" s="58" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="38" t="s">
+      <c r="F5" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2193,11 +2208,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="39"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="39"/>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="59"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2206,19 +2221,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="60" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="60" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="60" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2229,11 +2244,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="61"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2242,19 +2257,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="58" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="58" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="38" t="s">
+      <c r="E9" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="38" t="s">
+      <c r="F9" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2265,11 +2280,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="59"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2278,19 +2293,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="60" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C11" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D11" s="60" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="40" t="s">
+      <c r="E11" s="60" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="40" t="s">
+      <c r="F11" s="60" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2301,11 +2316,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="41"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="41"/>
-      <c r="F12" s="41"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2314,19 +2329,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="58" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="38" t="s">
+      <c r="C13" s="58" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="58" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="38" t="s">
+      <c r="E13" s="58" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="38" t="s">
+      <c r="F13" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2337,11 +2352,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="39"/>
-      <c r="C14" s="39"/>
-      <c r="D14" s="39"/>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
+      <c r="B14" s="59"/>
+      <c r="C14" s="59"/>
+      <c r="D14" s="59"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="59"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2350,19 +2365,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="58" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="58" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="38" t="s">
+      <c r="E15" s="58" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="38" t="s">
+      <c r="F15" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2373,11 +2388,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="39"/>
-      <c r="C16" s="39"/>
-      <c r="D16" s="39"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
+      <c r="B16" s="59"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="59"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2386,19 +2401,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="38" t="s">
+      <c r="B17" s="58" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="58" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="38" t="s">
+      <c r="D17" s="58" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="58" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="38" t="s">
+      <c r="F17" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2409,11 +2424,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="59"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="59"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2422,19 +2437,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="40" t="s">
+      <c r="B19" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="40" t="s">
+      <c r="C19" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="60" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="40" t="s">
+      <c r="E19" s="60" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="40" t="s">
+      <c r="F19" s="60" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2445,11 +2460,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="41"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
+      <c r="B20" s="61"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2458,19 +2473,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="38" t="s">
+      <c r="B21" s="58" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="38" t="s">
+      <c r="C21" s="58" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="38" t="s">
+      <c r="D21" s="58" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="38" t="s">
+      <c r="E21" s="58" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="38" t="s">
+      <c r="F21" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2481,11 +2496,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="39"/>
-      <c r="C22" s="39"/>
-      <c r="D22" s="39"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="39"/>
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="59"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2494,19 +2509,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="40" t="s">
+      <c r="C23" s="60" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="40" t="s">
+      <c r="D23" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="40" t="s">
+      <c r="E23" s="60" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="40" t="s">
+      <c r="F23" s="60" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2517,11 +2532,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="B24" s="61"/>
+      <c r="C24" s="61"/>
+      <c r="D24" s="61"/>
+      <c r="E24" s="61"/>
+      <c r="F24" s="61"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2530,19 +2545,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="38" t="s">
+      <c r="B25" s="58" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="38" t="s">
+      <c r="C25" s="58" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="38" t="s">
+      <c r="D25" s="58" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="38" t="s">
-        <v>184</v>
-      </c>
-      <c r="F25" s="38" t="s">
+      <c r="E25" s="58" t="s">
+        <v>182</v>
+      </c>
+      <c r="F25" s="58" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2553,11 +2568,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="39"/>
-      <c r="C26" s="39"/>
-      <c r="D26" s="39"/>
-      <c r="E26" s="39"/>
-      <c r="F26" s="39"/>
+      <c r="B26" s="59"/>
+      <c r="C26" s="59"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="59"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2660,7 +2675,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -2698,7 +2713,7 @@
         <v>179</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -2706,10 +2721,10 @@
         <v>46218</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -2719,32 +2734,36 @@
       <c r="C6" s="32" t="s">
         <v>180</v>
       </c>
-      <c r="D6" s="20"/>
+      <c r="D6" s="20" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="34">
         <v>46225</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>180</v>
-      </c>
-      <c r="D7" s="20"/>
+        <v>192</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="34">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="D8" s="20"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="34">
-        <v>46232</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>182</v>
+        <v>46231</v>
+      </c>
+      <c r="C9" s="64" t="s">
+        <v>191</v>
       </c>
       <c r="D9" s="20"/>
     </row>
@@ -2893,6 +2912,8 @@
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{AF5D6986-B77A-43EE-9A59-0C954BD679AC}"/>
     <hyperlink ref="D5" r:id="rId2" xr:uid="{EA3C6668-A9D1-49D9-BBE0-36CC722BCCBE}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{F97F2E3D-58D9-4E4D-8FD0-3B240CEE6920}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{3D7AFB71-15BC-4C9D-B6DE-D5462B3EB859}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update education downloads link for 7/27 training from latest Excel
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="595" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E989119-29C8-4FA7-8930-E0AE81B1D66F}"/>
+  <xr:revisionPtr revIDLastSave="596" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D480F483-8929-45B7-8DFD-EBC96C6E5A7C}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="194">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -732,6 +732,10 @@
   </si>
   <si>
     <t>[파트너사]VIOLA 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqAb7wVzwb3lzh10DCNEJTVBA?e=tM8z9K</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1150,6 +1154,9 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1210,26 +1217,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1520,10 +1524,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="38"/>
+      <c r="C4" s="39"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1542,10 +1546,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="39"/>
+      <c r="C8" s="40"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -1591,18 +1595,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -1763,7 +1767,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="44" t="s">
         <v>155</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -1772,117 +1776,117 @@
       <c r="D3" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="49" t="s">
+      <c r="E3" s="50" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="46" t="s">
+      <c r="F3" s="47" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="44"/>
+      <c r="B4" s="45"/>
       <c r="C4" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="F4" s="47"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="48"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="44"/>
+      <c r="B5" s="45"/>
       <c r="C5" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="50"/>
-      <c r="F5" s="47"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="48"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="44"/>
+      <c r="B6" s="45"/>
       <c r="C6" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="50"/>
-      <c r="F6" s="47"/>
+      <c r="E6" s="51"/>
+      <c r="F6" s="48"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="44"/>
+      <c r="B7" s="45"/>
       <c r="C7" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="50"/>
-      <c r="F7" s="47"/>
+      <c r="E7" s="51"/>
+      <c r="F7" s="48"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="44"/>
+      <c r="B8" s="45"/>
       <c r="C8" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="50"/>
-      <c r="F8" s="47"/>
+      <c r="E8" s="51"/>
+      <c r="F8" s="48"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="44"/>
+      <c r="B9" s="45"/>
       <c r="C9" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="50"/>
-      <c r="F9" s="47"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="48"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="44"/>
+      <c r="B10" s="45"/>
       <c r="C10" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="50"/>
-      <c r="F10" s="47"/>
+      <c r="E10" s="51"/>
+      <c r="F10" s="48"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="44"/>
+      <c r="B11" s="45"/>
       <c r="C11" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="50"/>
-      <c r="F11" s="47"/>
+      <c r="E11" s="51"/>
+      <c r="F11" s="48"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="45"/>
+      <c r="B12" s="46"/>
       <c r="C12" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="51"/>
-      <c r="F12" s="48"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="49"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="52" t="s">
+      <c r="B13" s="53" t="s">
         <v>84</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -1891,114 +1895,114 @@
       <c r="D13" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="46" t="s">
+      <c r="E13" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="55" t="s">
+      <c r="F13" s="56" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="53"/>
+      <c r="B14" s="54"/>
       <c r="C14" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="47"/>
-      <c r="F14" s="56"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="57"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="53"/>
+      <c r="B15" s="54"/>
       <c r="C15" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="47"/>
-      <c r="F15" s="56"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="57"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="53"/>
+      <c r="B16" s="54"/>
       <c r="C16" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="47"/>
-      <c r="F16" s="56"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="57"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="53"/>
+      <c r="B17" s="54"/>
       <c r="C17" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="47"/>
-      <c r="F17" s="56"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="57"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="53"/>
+      <c r="B18" s="54"/>
       <c r="C18" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="47"/>
-      <c r="F18" s="56"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="57"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="53"/>
+      <c r="B19" s="54"/>
       <c r="C19" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="47"/>
-      <c r="F19" s="56"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="57"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="53"/>
+      <c r="B20" s="54"/>
       <c r="C20" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="47"/>
-      <c r="F20" s="56"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="57"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="53"/>
+      <c r="B21" s="54"/>
       <c r="C21" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="47"/>
-      <c r="F21" s="56"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="57"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="54"/>
+      <c r="B22" s="55"/>
       <c r="C22" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="48"/>
-      <c r="F22" s="57"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="58"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="52" t="s">
+      <c r="B23" s="53" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="30" t="s">
@@ -2007,111 +2011,111 @@
       <c r="D23" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="47" t="s">
         <v>153</v>
       </c>
-      <c r="F23" s="55" t="s">
+      <c r="F23" s="56" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="53"/>
+      <c r="B24" s="54"/>
       <c r="C24" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E24" s="47"/>
-      <c r="F24" s="56"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="57"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="53"/>
+      <c r="B25" s="54"/>
       <c r="C25" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E25" s="47"/>
-      <c r="F25" s="56"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="57"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="53"/>
+      <c r="B26" s="54"/>
       <c r="C26" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="E26" s="47"/>
-      <c r="F26" s="56"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="57"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="53"/>
+      <c r="B27" s="54"/>
       <c r="C27" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="E27" s="47"/>
-      <c r="F27" s="56"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="57"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="53"/>
+      <c r="B28" s="54"/>
       <c r="C28" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="47"/>
-      <c r="F28" s="56"/>
+      <c r="E28" s="48"/>
+      <c r="F28" s="57"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="53"/>
+      <c r="B29" s="54"/>
       <c r="C29" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="E29" s="47"/>
-      <c r="F29" s="56"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="57"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="53"/>
+      <c r="B30" s="54"/>
       <c r="C30" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="E30" s="47"/>
-      <c r="F30" s="56"/>
+      <c r="E30" s="48"/>
+      <c r="F30" s="57"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="53"/>
+      <c r="B31" s="54"/>
       <c r="C31" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="47"/>
-      <c r="F31" s="56"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="57"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="54"/>
+      <c r="B32" s="55"/>
       <c r="C32" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="48"/>
-      <c r="F32" s="57"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="58"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="5"/>
@@ -2179,25 +2183,25 @@
       <c r="F4" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="G4" s="62" t="s">
+      <c r="G4" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="63"/>
+      <c r="H4" s="62"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="58" t="s">
+      <c r="B5" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="58" t="s">
+      <c r="C5" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="58" t="s">
+      <c r="D5" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="58" t="s">
+      <c r="E5" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2208,11 +2212,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="59"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2221,19 +2225,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="60" t="s">
+      <c r="B7" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="60" t="s">
+      <c r="C7" s="59" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="60" t="s">
+      <c r="D7" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="60" t="s">
+      <c r="E7" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="60" t="s">
+      <c r="F7" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2244,11 +2248,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="61"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2257,19 +2261,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="58" t="s">
+      <c r="B9" s="63" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="58" t="s">
+      <c r="C9" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="58" t="s">
+      <c r="D9" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="58" t="s">
+      <c r="E9" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="58" t="s">
+      <c r="F9" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2280,11 +2284,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
-      <c r="E10" s="59"/>
-      <c r="F10" s="59"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2293,19 +2297,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="60" t="s">
+      <c r="B11" s="59" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="60" t="s">
+      <c r="C11" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="60" t="s">
+      <c r="D11" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="60" t="s">
+      <c r="E11" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="60" t="s">
+      <c r="F11" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2316,11 +2320,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="61"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
-      <c r="F12" s="61"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2329,19 +2333,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="58" t="s">
+      <c r="B13" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="58" t="s">
+      <c r="D13" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="58" t="s">
+      <c r="E13" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="58" t="s">
+      <c r="F13" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2352,11 +2356,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="59"/>
-      <c r="C14" s="59"/>
-      <c r="D14" s="59"/>
-      <c r="E14" s="59"/>
-      <c r="F14" s="59"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2365,19 +2369,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="58" t="s">
+      <c r="D15" s="63" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="58" t="s">
+      <c r="E15" s="63" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="58" t="s">
+      <c r="F15" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2388,11 +2392,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="59"/>
-      <c r="C16" s="59"/>
-      <c r="D16" s="59"/>
-      <c r="E16" s="59"/>
-      <c r="F16" s="59"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2401,19 +2405,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="58" t="s">
+      <c r="D17" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="58" t="s">
+      <c r="E17" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="58" t="s">
+      <c r="F17" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2424,11 +2428,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="59"/>
-      <c r="C18" s="59"/>
-      <c r="D18" s="59"/>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2437,19 +2441,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="60" t="s">
+      <c r="B19" s="59" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="60" t="s">
+      <c r="C19" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="60" t="s">
+      <c r="D19" s="59" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="60" t="s">
+      <c r="E19" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="60" t="s">
+      <c r="F19" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2460,11 +2464,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="61"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2473,19 +2477,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="63" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="58" t="s">
+      <c r="D21" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="58" t="s">
+      <c r="E21" s="63" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="58" t="s">
+      <c r="F21" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2496,11 +2500,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="59"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="59"/>
-      <c r="F22" s="59"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2509,19 +2513,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="60" t="s">
+      <c r="B23" s="59" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="60" t="s">
+      <c r="C23" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="60" t="s">
+      <c r="D23" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="60" t="s">
+      <c r="E23" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="60" t="s">
+      <c r="F23" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2532,11 +2536,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="61"/>
-      <c r="C24" s="61"/>
-      <c r="D24" s="61"/>
-      <c r="E24" s="61"/>
-      <c r="F24" s="61"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2545,19 +2549,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="63" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="58" t="s">
+      <c r="D25" s="63" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="58" t="s">
+      <c r="E25" s="63" t="s">
         <v>182</v>
       </c>
-      <c r="F25" s="58" t="s">
+      <c r="F25" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2568,11 +2572,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="59"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="59"/>
-      <c r="E26" s="59"/>
-      <c r="F26" s="59"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2582,40 +2586,16 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2628,16 +2608,40 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2756,13 +2760,15 @@
       <c r="C8" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="20" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="34">
         <v>46231</v>
       </c>
-      <c r="C9" s="64" t="s">
+      <c r="C9" s="38" t="s">
         <v>191</v>
       </c>
       <c r="D9" s="20"/>
@@ -2914,6 +2920,7 @@
     <hyperlink ref="D5" r:id="rId2" xr:uid="{EA3C6668-A9D1-49D9-BBE0-36CC722BCCBE}"/>
     <hyperlink ref="D6" r:id="rId3" xr:uid="{F97F2E3D-58D9-4E4D-8FD0-3B240CEE6920}"/>
     <hyperlink ref="D7" r:id="rId4" xr:uid="{3D7AFB71-15BC-4C9D-B6DE-D5462B3EB859}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{F360FD24-0F28-4EBB-B4CD-446461DBBD82}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update education downloads link for 7/27 from latest Excel data
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="596" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D480F483-8929-45B7-8DFD-EBC96C6E5A7C}"/>
+  <xr:revisionPtr revIDLastSave="598" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B31CD1C-8582-4B0B-833A-33799F56167C}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -735,7 +735,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqAb7wVzwb3lzh10DCNEJTVBA?e=tM8z9K</t>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqARgbrFbL5rlHoCsHl3GhRH8?e=B0SOs9</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1217,6 +1217,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1227,12 +1233,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -2183,25 +2183,25 @@
       <c r="F4" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="G4" s="63" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2212,11 +2212,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="64"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2225,19 +2225,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="59" t="s">
+      <c r="D7" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="59" t="s">
+      <c r="E7" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="59" t="s">
+      <c r="F7" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2248,11 +2248,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="60"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2261,19 +2261,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="59" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="C9" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="63" t="s">
+      <c r="F9" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2284,11 +2284,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2297,19 +2297,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="61" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="59" t="s">
+      <c r="E11" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="59" t="s">
+      <c r="F11" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2320,11 +2320,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2333,19 +2333,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="59" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="63" t="s">
+      <c r="E13" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="63" t="s">
+      <c r="F13" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2356,11 +2356,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="64"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2369,19 +2369,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" s="59" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="63" t="s">
+      <c r="F15" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2392,11 +2392,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="64"/>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="64"/>
+      <c r="B16" s="60"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2405,19 +2405,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="63" t="s">
+      <c r="C17" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="63" t="s">
+      <c r="E17" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="63" t="s">
+      <c r="F17" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2428,11 +2428,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="64"/>
-      <c r="C18" s="64"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
+      <c r="B18" s="60"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="60"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="60"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2441,19 +2441,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="59" t="s">
+      <c r="C19" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="59" t="s">
+      <c r="E19" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2464,11 +2464,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2477,19 +2477,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="59" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="63" t="s">
+      <c r="C21" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="63" t="s">
+      <c r="E21" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="63" t="s">
+      <c r="F21" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2500,11 +2500,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="64"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2513,19 +2513,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="61" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="59" t="s">
+      <c r="D23" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="59" t="s">
+      <c r="E23" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="F23" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2536,11 +2536,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2549,19 +2549,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="63" t="s">
+      <c r="C25" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="63" t="s">
+      <c r="E25" s="59" t="s">
         <v>182</v>
       </c>
-      <c r="F25" s="63" t="s">
+      <c r="F25" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2572,11 +2572,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="64"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="60"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2586,16 +2586,40 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2608,40 +2632,16 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2920,7 +2920,7 @@
     <hyperlink ref="D5" r:id="rId2" xr:uid="{EA3C6668-A9D1-49D9-BBE0-36CC722BCCBE}"/>
     <hyperlink ref="D6" r:id="rId3" xr:uid="{F97F2E3D-58D9-4E4D-8FD0-3B240CEE6920}"/>
     <hyperlink ref="D7" r:id="rId4" xr:uid="{3D7AFB71-15BC-4C9D-B6DE-D5462B3EB859}"/>
-    <hyperlink ref="D8" r:id="rId5" xr:uid="{F360FD24-0F28-4EBB-B4CD-446461DBBD82}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{CA4DAE9D-A58B-46BE-8CAD-761CC42C8FC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update education downloads link for 7/28 from latest Excel data
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="598" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B31CD1C-8582-4B0B-833A-33799F56167C}"/>
+  <xr:revisionPtr revIDLastSave="601" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A844283-8D6C-428A-95F6-32185EDC38C5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="195">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -736,6 +736,10 @@
   </si>
   <si>
     <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqARgbrFbL5rlHoCsHl3GhRH8?e=B0SOs9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAi2tO545GUTJDNTdOSm_WYAT7yjij8h810lxQSSeuNXyo?e=bgPkqw</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1217,22 +1221,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -2183,25 +2187,25 @@
       <c r="F4" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="G4" s="63" t="s">
+      <c r="G4" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="64"/>
+      <c r="H4" s="62"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="59" t="s">
+      <c r="D5" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="59" t="s">
+      <c r="E5" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="59" t="s">
+      <c r="F5" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2212,11 +2216,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2225,19 +2229,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="59" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2248,11 +2252,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2261,19 +2265,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="63" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="59" t="s">
+      <c r="C9" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="59" t="s">
+      <c r="D9" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="59" t="s">
+      <c r="E9" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="59" t="s">
+      <c r="F9" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2284,11 +2288,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="60"/>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2297,19 +2301,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="59" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="61" t="s">
+      <c r="D11" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2320,11 +2324,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2333,19 +2337,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="59" t="s">
+      <c r="B13" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="59" t="s">
+      <c r="D13" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="59" t="s">
+      <c r="E13" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="59" t="s">
+      <c r="F13" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2356,11 +2360,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2369,19 +2373,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="D15" s="63" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="59" t="s">
+      <c r="E15" s="63" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="59" t="s">
+      <c r="F15" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2392,11 +2396,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2405,19 +2409,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="59" t="s">
+      <c r="C17" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="59" t="s">
+      <c r="D17" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="59" t="s">
+      <c r="E17" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="59" t="s">
+      <c r="F17" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2428,11 +2432,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="60"/>
-      <c r="C18" s="60"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2441,19 +2445,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="59" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="59" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2464,11 +2468,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2477,19 +2481,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="59" t="s">
+      <c r="C21" s="63" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="59" t="s">
+      <c r="E21" s="63" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2500,11 +2504,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2513,19 +2517,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="59" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2536,11 +2540,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2549,19 +2553,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="59" t="s">
+      <c r="B25" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="59" t="s">
+      <c r="C25" s="63" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="59" t="s">
+      <c r="D25" s="63" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="59" t="s">
+      <c r="E25" s="63" t="s">
         <v>182</v>
       </c>
-      <c r="F25" s="59" t="s">
+      <c r="F25" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2572,11 +2576,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2586,40 +2590,16 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2632,16 +2612,40 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2771,7 +2775,9 @@
       <c r="C9" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="D9" s="20"/>
+      <c r="D9" s="20" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="34"/>
@@ -2921,6 +2927,7 @@
     <hyperlink ref="D6" r:id="rId3" xr:uid="{F97F2E3D-58D9-4E4D-8FD0-3B240CEE6920}"/>
     <hyperlink ref="D7" r:id="rId4" xr:uid="{3D7AFB71-15BC-4C9D-B6DE-D5462B3EB859}"/>
     <hyperlink ref="D8" r:id="rId5" xr:uid="{CA4DAE9D-A58B-46BE-8CAD-761CC42C8FC6}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{3F66A6EE-8E9C-4CA9-AC0C-DC07BBAE40E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update education downloads data for 7/29 from latest Excel sheet
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="601" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A844283-8D6C-428A-95F6-32185EDC38C5}"/>
+  <xr:revisionPtr revIDLastSave="605" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7E29A9A-066E-42EF-856C-A0EA949EAACD}"/>
   <bookViews>
     <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="197">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -740,6 +740,14 @@
   </si>
   <si>
     <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAi2tO545GUTJDNTdOSm_WYAT7yjij8h810lxQSSeuNXyo?e=bgPkqw</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부] 온보딩 제품교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgA_IZOLdByoTZ3BxYsPq0TbAYfW-iQugsnPW4SoyythDrk?e=iGX2bh</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1221,6 +1229,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1231,12 +1245,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -2187,25 +2195,25 @@
       <c r="F4" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="G4" s="63" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="59" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="59" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2216,11 +2224,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="64"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
+      <c r="B6" s="60"/>
+      <c r="C6" s="60"/>
+      <c r="D6" s="60"/>
+      <c r="E6" s="60"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2229,19 +2237,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="59" t="s">
+      <c r="D7" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="59" t="s">
+      <c r="E7" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="59" t="s">
+      <c r="F7" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2252,11 +2260,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="60"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2265,19 +2273,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="59" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="C9" s="59" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="59" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="59" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="63" t="s">
+      <c r="F9" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2288,11 +2296,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="60"/>
+      <c r="E10" s="60"/>
+      <c r="F10" s="60"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2301,19 +2309,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="61" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="59" t="s">
+      <c r="E11" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="59" t="s">
+      <c r="F11" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2324,11 +2332,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2337,19 +2345,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="59" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="59" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="59" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="63" t="s">
+      <c r="E13" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="63" t="s">
+      <c r="F13" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2360,11 +2368,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="64"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
+      <c r="B14" s="60"/>
+      <c r="C14" s="60"/>
+      <c r="D14" s="60"/>
+      <c r="E14" s="60"/>
+      <c r="F14" s="60"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2373,19 +2381,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="59" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" s="59" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="63" t="s">
+      <c r="F15" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2396,11 +2404,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="64"/>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="64"/>
+      <c r="B16" s="60"/>
+      <c r="C16" s="60"/>
+      <c r="D16" s="60"/>
+      <c r="E16" s="60"/>
+      <c r="F16" s="60"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2409,19 +2417,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="59" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="63" t="s">
+      <c r="C17" s="59" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="63" t="s">
+      <c r="E17" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="63" t="s">
+      <c r="F17" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2432,11 +2440,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="64"/>
-      <c r="C18" s="64"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
+      <c r="B18" s="60"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="60"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="60"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2445,19 +2453,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="59" t="s">
+      <c r="C19" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="59" t="s">
+      <c r="E19" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2468,11 +2476,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2481,19 +2489,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="59" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="63" t="s">
+      <c r="C21" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="63" t="s">
+      <c r="E21" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="63" t="s">
+      <c r="F21" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2504,11 +2512,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="64"/>
+      <c r="B22" s="60"/>
+      <c r="C22" s="60"/>
+      <c r="D22" s="60"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="60"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2517,19 +2525,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="61" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="59" t="s">
+      <c r="D23" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="59" t="s">
+      <c r="E23" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="F23" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2540,11 +2548,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2553,19 +2561,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="63" t="s">
+      <c r="C25" s="59" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="59" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="63" t="s">
+      <c r="E25" s="59" t="s">
         <v>182</v>
       </c>
-      <c r="F25" s="63" t="s">
+      <c r="F25" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2576,11 +2584,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="64"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
+      <c r="B26" s="60"/>
+      <c r="C26" s="60"/>
+      <c r="D26" s="60"/>
+      <c r="E26" s="60"/>
+      <c r="F26" s="60"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2590,16 +2598,40 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2612,40 +2644,16 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2780,9 +2788,15 @@
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B10" s="34"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="19"/>
+      <c r="B10" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="34"/>
@@ -2928,6 +2942,7 @@
     <hyperlink ref="D7" r:id="rId4" xr:uid="{3D7AFB71-15BC-4C9D-B6DE-D5462B3EB859}"/>
     <hyperlink ref="D8" r:id="rId5" xr:uid="{CA4DAE9D-A58B-46BE-8CAD-761CC42C8FC6}"/>
     <hyperlink ref="D9" r:id="rId6" xr:uid="{3F66A6EE-8E9C-4CA9-AC0C-DC07BBAE40E5}"/>
+    <hyperlink ref="D10" r:id="rId7" xr:uid="{C932FA4E-851E-4F7C-8642-515FA0A83F91}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add instructor admin dashboard page (/admin) and Excel parsing support
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="605" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7E29A9A-066E-42EF-856C-A0EA949EAACD}"/>
+  <xr:revisionPtr revIDLastSave="615" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81A4F222-2767-4264-B070-49F16348B4EA}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="교육자료 다운로드" sheetId="4" r:id="rId6"/>
     <sheet name="실습자료 다운로드" sheetId="8" r:id="rId7"/>
     <sheet name="(관리자)솔루션 접속 정보" sheetId="6" r:id="rId8"/>
-    <sheet name="(관리자)Trombone 미들웨어 접속정보" sheetId="2" r:id="rId9"/>
+    <sheet name="(관리자)아카데미 VPN 계정 목록" sheetId="10" r:id="rId9"/>
+    <sheet name="(관리자)Trombone 미들웨어 접속정보" sheetId="2" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="206">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -687,10 +688,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>d</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EDU11</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -749,6 +746,44 @@
   <si>
     <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgA_IZOLdByoTZ3BxYsPq0TbAYfW-iQugsnPW4SoyythDrk?e=iGX2bh</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오케스트로 아카데미 VPN계정 목록</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>js.park</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>kZsKnumI</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ws.choi</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>bGcISihA</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>hy.shin</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>nmJjGQLL</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>yh.kim</t>
+  </si>
+  <si>
+    <t>Okestro2018!</t>
   </si>
 </sst>
 </file>
@@ -847,7 +882,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Freesentation 4 Regular"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="6"/>
@@ -922,7 +956,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1060,12 +1094,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1229,23 +1289,35 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1596,6 +1668,92 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB534C5F-5069-44F5-BE30-375C8B57A789}">
+  <dimension ref="B2:D7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="17.625" customWidth="1"/>
+    <col min="4" max="4" width="25.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{00A3F4CF-A6BD-4781-B618-D2E727A880EE}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{088482B0-11E1-4715-B3A3-DAFF004D45F8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90A17B8-D559-4179-9BBE-8680B873B9EB}">
   <dimension ref="B2:D14"/>
@@ -2190,30 +2348,30 @@
         <v>88</v>
       </c>
       <c r="E4" s="24" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="F4" s="37" t="s">
-        <v>184</v>
-      </c>
-      <c r="G4" s="63" t="s">
+      <c r="G4" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="64"/>
+      <c r="H4" s="62"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="59" t="s">
+      <c r="C5" s="63" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="59" t="s">
+      <c r="D5" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="59" t="s">
+      <c r="E5" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="59" t="s">
+      <c r="F5" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2224,11 +2382,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="60"/>
-      <c r="C6" s="60"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="60"/>
-      <c r="F6" s="60"/>
+      <c r="B6" s="64"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2237,19 +2395,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="59" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2260,11 +2418,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="60"/>
+      <c r="F8" s="60"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2273,19 +2431,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="59" t="s">
+      <c r="B9" s="63" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="59" t="s">
+      <c r="C9" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="59" t="s">
+      <c r="D9" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="59" t="s">
+      <c r="E9" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="59" t="s">
+      <c r="F9" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2296,11 +2454,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="60"/>
-      <c r="C10" s="60"/>
-      <c r="D10" s="60"/>
-      <c r="E10" s="60"/>
-      <c r="F10" s="60"/>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2309,19 +2467,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="59" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="61" t="s">
+      <c r="D11" s="59" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="59" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2332,11 +2490,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2345,19 +2503,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="59" t="s">
+      <c r="B13" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="59" t="s">
+      <c r="C13" s="63" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="59" t="s">
+      <c r="D13" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="59" t="s">
+      <c r="E13" s="63" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="59" t="s">
+      <c r="F13" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2368,11 +2526,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="60"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="60"/>
-      <c r="E14" s="60"/>
-      <c r="F14" s="60"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="64"/>
+      <c r="F14" s="64"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2381,19 +2539,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="59" t="s">
+      <c r="C15" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="D15" s="63" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="59" t="s">
+      <c r="E15" s="63" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="59" t="s">
+      <c r="F15" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2404,11 +2562,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="60"/>
-      <c r="C16" s="60"/>
-      <c r="D16" s="60"/>
-      <c r="E16" s="60"/>
-      <c r="F16" s="60"/>
+      <c r="B16" s="64"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2417,19 +2575,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="59" t="s">
+      <c r="B17" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="59" t="s">
+      <c r="C17" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="59" t="s">
+      <c r="D17" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="59" t="s">
+      <c r="E17" s="63" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="59" t="s">
+      <c r="F17" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2440,11 +2598,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="60"/>
-      <c r="C18" s="60"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2453,19 +2611,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="59" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="59" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="59" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2476,11 +2634,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
+      <c r="B20" s="60"/>
+      <c r="C20" s="60"/>
+      <c r="D20" s="60"/>
+      <c r="E20" s="60"/>
+      <c r="F20" s="60"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2489,19 +2647,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="59" t="s">
+      <c r="B21" s="63" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="59" t="s">
+      <c r="C21" s="63" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="63" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="59" t="s">
+      <c r="E21" s="63" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2512,11 +2670,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="60"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="60"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="64"/>
+      <c r="E22" s="64"/>
+      <c r="F22" s="64"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2525,19 +2683,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="59" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="59" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2548,11 +2706,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2561,19 +2719,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="59" t="s">
+      <c r="B25" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="59" t="s">
+      <c r="C25" s="63" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="59" t="s">
+      <c r="D25" s="63" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="59" t="s">
-        <v>182</v>
-      </c>
-      <c r="F25" s="59" t="s">
+      <c r="E25" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="F25" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2584,11 +2742,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="60"/>
-      <c r="C26" s="60"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
+      <c r="B26" s="64"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
+      <c r="F26" s="64"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2598,40 +2756,16 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2644,16 +2778,40 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2688,13 +2846,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9750530-01B1-49BC-B5D5-1F192598EBD5}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2729,7 +2881,7 @@
         <v>179</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -2737,10 +2889,10 @@
         <v>46218</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -2751,7 +2903,7 @@
         <v>180</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -2759,10 +2911,10 @@
         <v>46225</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -2770,10 +2922,10 @@
         <v>46230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -2781,10 +2933,10 @@
         <v>46231</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -2792,10 +2944,10 @@
         <v>46232</v>
       </c>
       <c r="C10" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="D10" s="20" t="s">
         <v>195</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -3094,87 +3246,77 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB534C5F-5069-44F5-BE30-375C8B57A789}">
-  <dimension ref="B2:D7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B48416FD-5E79-4C60-87C7-6AAB59A9E3DF}">
+  <dimension ref="B3:D10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.375" customWidth="1"/>
-    <col min="3" max="3" width="17.625" customWidth="1"/>
-    <col min="4" max="4" width="25.25" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="29.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B2" s="13" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>29</v>
-      </c>
+    <row r="3" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="65" t="s">
+        <v>196</v>
+      </c>
+      <c r="C4" s="66"/>
+      <c r="D4" s="67"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="B5" s="67"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>29</v>
-      </c>
+      <c r="B6" s="16" t="s">
+        <v>197</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="67"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>30</v>
-      </c>
+      <c r="B7" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="C7" s="68" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="67"/>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="68" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" s="68" t="s">
+        <v>201</v>
+      </c>
+      <c r="D8" s="67"/>
+    </row>
+    <row r="9" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B9" s="68" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="68" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="67"/>
+    </row>
+    <row r="10" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B10" s="68" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="68" t="s">
+        <v>205</v>
+      </c>
+      <c r="D10" s="67"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="D5" r:id="rId1" xr:uid="{00A3F4CF-A6BD-4781-B618-D2E727A880EE}"/>
-    <hyperlink ref="D7" r:id="rId2" xr:uid="{088482B0-11E1-4715-B3A3-DAFF004D45F8}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync newly added Excel download item ([내부] 온보딩 제품교육222)
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="615" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81A4F222-2767-4264-B070-49F16348B4EA}"/>
+  <xr:revisionPtr revIDLastSave="675" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5F0E4F0-57FC-4690-8D22-736A1F9A6458}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
     <sheet name="실습용 VPN 계정 정보" sheetId="3" r:id="rId2"/>
     <sheet name="솔루션 접속 정보" sheetId="1" r:id="rId3"/>
     <sheet name="TROMBONE 서비스 접속 정보" sheetId="7" r:id="rId4"/>
-    <sheet name="TROMBONE Git 계정" sheetId="9" r:id="rId5"/>
-    <sheet name="교육자료 다운로드" sheetId="4" r:id="rId6"/>
-    <sheet name="실습자료 다운로드" sheetId="8" r:id="rId7"/>
-    <sheet name="(관리자)솔루션 접속 정보" sheetId="6" r:id="rId8"/>
-    <sheet name="(관리자)아카데미 VPN 계정 목록" sheetId="10" r:id="rId9"/>
-    <sheet name="(관리자)Trombone 미들웨어 접속정보" sheetId="2" r:id="rId10"/>
+    <sheet name="교육자료 다운로드" sheetId="4" r:id="rId5"/>
+    <sheet name="실습자료 다운로드" sheetId="8" r:id="rId6"/>
+    <sheet name="(관리자)솔루션 접속 정보" sheetId="6" r:id="rId7"/>
+    <sheet name="(관리자)아카데미 VPN 계정 목록" sheetId="10" r:id="rId8"/>
+    <sheet name="(관리자)Trombone 미들웨어 접속정보" sheetId="2" r:id="rId9"/>
+    <sheet name="(관리자)Trombone Nodeport" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="221">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -784,6 +784,56 @@
   </si>
   <si>
     <t>Okestro2018!</t>
+  </si>
+  <si>
+    <t>User</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>user00</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>user01</t>
+  </si>
+  <si>
+    <t>user02</t>
+  </si>
+  <si>
+    <t>user03</t>
+  </si>
+  <si>
+    <t>user04</t>
+  </si>
+  <si>
+    <t>user05</t>
+  </si>
+  <si>
+    <t>user06</t>
+  </si>
+  <si>
+    <t>user07</t>
+  </si>
+  <si>
+    <t>user08</t>
+  </si>
+  <si>
+    <t>user09</t>
+  </si>
+  <si>
+    <t>user11</t>
+  </si>
+  <si>
+    <t>stg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부] 온보딩 제품교육222</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1229,6 +1279,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1312,12 +1368,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1608,10 +1658,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="39"/>
+      <c r="C4" s="41"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1630,10 +1680,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="42" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="40"/>
+      <c r="C8" s="42"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -1669,87 +1719,160 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB534C5F-5069-44F5-BE30-375C8B57A789}">
-  <dimension ref="B2:D7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E35D4360-58D8-421A-AAC8-02FFBEB8991A}">
+  <dimension ref="B2:D14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="14.375" customWidth="1"/>
-    <col min="3" max="3" width="17.625" customWidth="1"/>
-    <col min="4" max="4" width="25.25" customWidth="1"/>
+    <col min="2" max="2" width="15.625" customWidth="1"/>
+    <col min="3" max="3" width="25.25" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>32</v>
+        <v>206</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>14</v>
+        <v>218</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>15</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>29</v>
+        <v>207</v>
+      </c>
+      <c r="C3" s="14">
+        <v>31300</v>
+      </c>
+      <c r="D3" s="14">
+        <v>31310</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>29</v>
+        <v>208</v>
+      </c>
+      <c r="C4" s="14">
+        <v>31301</v>
+      </c>
+      <c r="D4" s="14">
+        <v>31311</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>30</v>
+        <v>209</v>
+      </c>
+      <c r="C5" s="14">
+        <v>31302</v>
+      </c>
+      <c r="D5" s="8">
+        <v>31312</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>29</v>
+        <v>210</v>
+      </c>
+      <c r="C6" s="14">
+        <v>31303</v>
+      </c>
+      <c r="D6" s="14">
+        <v>31313</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>30</v>
+        <v>211</v>
+      </c>
+      <c r="C7" s="14">
+        <v>31304</v>
+      </c>
+      <c r="D7" s="8">
+        <v>31314</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C8" s="21">
+        <v>31305</v>
+      </c>
+      <c r="D8" s="21">
+        <v>31315</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C9" s="21">
+        <v>31306</v>
+      </c>
+      <c r="D9" s="21">
+        <v>31316</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="21">
+        <v>31307</v>
+      </c>
+      <c r="D10" s="21">
+        <v>31317</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B11" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C11" s="21">
+        <v>31308</v>
+      </c>
+      <c r="D11" s="21">
+        <v>31318</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C12" s="21">
+        <v>31309</v>
+      </c>
+      <c r="D12" s="21">
+        <v>31319</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="21">
+        <v>31320</v>
+      </c>
+      <c r="D13" s="21">
+        <v>31321</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="C14" s="21">
+        <v>31322</v>
+      </c>
+      <c r="D14" s="21">
+        <v>31323</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="D5" r:id="rId1" xr:uid="{00A3F4CF-A6BD-4781-B618-D2E727A880EE}"/>
-    <hyperlink ref="D7" r:id="rId2" xr:uid="{088482B0-11E1-4715-B3A3-DAFF004D45F8}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1765,18 +1888,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -1937,7 +2060,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="46" t="s">
         <v>155</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -1946,117 +2069,117 @@
       <c r="D3" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="47" t="s">
+      <c r="F3" s="49" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="45"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="F4" s="48"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="50"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="45"/>
+      <c r="B5" s="47"/>
       <c r="C5" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="51"/>
-      <c r="F5" s="48"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="50"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="45"/>
+      <c r="B6" s="47"/>
       <c r="C6" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="51"/>
-      <c r="F6" s="48"/>
+      <c r="E6" s="53"/>
+      <c r="F6" s="50"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="45"/>
+      <c r="B7" s="47"/>
       <c r="C7" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="51"/>
-      <c r="F7" s="48"/>
+      <c r="E7" s="53"/>
+      <c r="F7" s="50"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="45"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="51"/>
-      <c r="F8" s="48"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="50"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="45"/>
+      <c r="B9" s="47"/>
       <c r="C9" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="51"/>
-      <c r="F9" s="48"/>
+      <c r="E9" s="53"/>
+      <c r="F9" s="50"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="45"/>
+      <c r="B10" s="47"/>
       <c r="C10" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="51"/>
-      <c r="F10" s="48"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="50"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="45"/>
+      <c r="B11" s="47"/>
       <c r="C11" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="51"/>
-      <c r="F11" s="48"/>
+      <c r="E11" s="53"/>
+      <c r="F11" s="50"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="46"/>
+      <c r="B12" s="48"/>
       <c r="C12" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="52"/>
-      <c r="F12" s="49"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="51"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="55" t="s">
         <v>84</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -2065,114 +2188,114 @@
       <c r="D13" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="47" t="s">
+      <c r="E13" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="56" t="s">
+      <c r="F13" s="58" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="54"/>
+      <c r="B14" s="56"/>
       <c r="C14" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="48"/>
-      <c r="F14" s="57"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="59"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="54"/>
+      <c r="B15" s="56"/>
       <c r="C15" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="48"/>
-      <c r="F15" s="57"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="59"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="54"/>
+      <c r="B16" s="56"/>
       <c r="C16" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="48"/>
-      <c r="F16" s="57"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="59"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="54"/>
+      <c r="B17" s="56"/>
       <c r="C17" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="48"/>
-      <c r="F17" s="57"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="59"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="54"/>
+      <c r="B18" s="56"/>
       <c r="C18" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="48"/>
-      <c r="F18" s="57"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="59"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="54"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="57"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="59"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="54"/>
+      <c r="B20" s="56"/>
       <c r="C20" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="48"/>
-      <c r="F20" s="57"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="59"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="54"/>
+      <c r="B21" s="56"/>
       <c r="C21" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="E21" s="48"/>
-      <c r="F21" s="57"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="59"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="55"/>
+      <c r="B22" s="57"/>
       <c r="C22" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="49"/>
-      <c r="F22" s="58"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="60"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="53" t="s">
+      <c r="B23" s="55" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="30" t="s">
@@ -2181,111 +2304,111 @@
       <c r="D23" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="47" t="s">
+      <c r="E23" s="49" t="s">
         <v>153</v>
       </c>
-      <c r="F23" s="56" t="s">
+      <c r="F23" s="58" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="54"/>
+      <c r="B24" s="56"/>
       <c r="C24" s="30" t="s">
         <v>165</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E24" s="48"/>
-      <c r="F24" s="57"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="59"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="54"/>
+      <c r="B25" s="56"/>
       <c r="C25" s="30" t="s">
         <v>166</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="E25" s="48"/>
-      <c r="F25" s="57"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="59"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="54"/>
+      <c r="B26" s="56"/>
       <c r="C26" s="30" t="s">
         <v>167</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="E26" s="48"/>
-      <c r="F26" s="57"/>
+      <c r="E26" s="50"/>
+      <c r="F26" s="59"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="54"/>
+      <c r="B27" s="56"/>
       <c r="C27" s="30" t="s">
         <v>168</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="E27" s="48"/>
-      <c r="F27" s="57"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="59"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="54"/>
+      <c r="B28" s="56"/>
       <c r="C28" s="30" t="s">
         <v>169</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="48"/>
-      <c r="F28" s="57"/>
+      <c r="E28" s="50"/>
+      <c r="F28" s="59"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="54"/>
+      <c r="B29" s="56"/>
       <c r="C29" s="30" t="s">
         <v>170</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="E29" s="48"/>
-      <c r="F29" s="57"/>
+      <c r="E29" s="50"/>
+      <c r="F29" s="59"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="54"/>
+      <c r="B30" s="56"/>
       <c r="C30" s="30" t="s">
         <v>171</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="E30" s="48"/>
-      <c r="F30" s="57"/>
+      <c r="E30" s="50"/>
+      <c r="F30" s="59"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="54"/>
+      <c r="B31" s="56"/>
       <c r="C31" s="30" t="s">
         <v>172</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="E31" s="48"/>
-      <c r="F31" s="57"/>
+      <c r="E31" s="50"/>
+      <c r="F31" s="59"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="55"/>
+      <c r="B32" s="57"/>
       <c r="C32" s="30" t="s">
         <v>173</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="E32" s="49"/>
-      <c r="F32" s="58"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="60"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" s="5"/>
@@ -2353,25 +2476,25 @@
       <c r="F4" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="G4" s="61" t="s">
+      <c r="G4" s="63" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="62"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="63" t="s">
+      <c r="B5" s="65" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="65" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="63" t="s">
+      <c r="D5" s="65" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="63" t="s">
+      <c r="E5" s="65" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="63" t="s">
+      <c r="F5" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2382,11 +2505,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="64"/>
-      <c r="C6" s="64"/>
-      <c r="D6" s="64"/>
-      <c r="E6" s="64"/>
-      <c r="F6" s="64"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2395,19 +2518,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="59" t="s">
+      <c r="B7" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="59" t="s">
+      <c r="D7" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="59" t="s">
+      <c r="E7" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="59" t="s">
+      <c r="F7" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2418,11 +2541,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="60"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="60"/>
-      <c r="E8" s="60"/>
-      <c r="F8" s="60"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2431,19 +2554,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="65" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="C9" s="65" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="63" t="s">
+      <c r="F9" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2454,11 +2577,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="64"/>
-      <c r="C10" s="64"/>
-      <c r="D10" s="64"/>
-      <c r="E10" s="64"/>
-      <c r="F10" s="64"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2467,19 +2590,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="59" t="s">
+      <c r="B11" s="61" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="59" t="s">
+      <c r="C11" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="61" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="59" t="s">
+      <c r="E11" s="61" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="59" t="s">
+      <c r="F11" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2490,11 +2613,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2503,19 +2626,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="63" t="s">
+      <c r="B13" s="65" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="65" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="63" t="s">
+      <c r="E13" s="65" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="63" t="s">
+      <c r="F13" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2526,11 +2649,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="64"/>
-      <c r="C14" s="64"/>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="66"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2539,19 +2662,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="65" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="65" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" s="65" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="65" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="63" t="s">
+      <c r="F15" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2562,11 +2685,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="64"/>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="64"/>
-      <c r="F16" s="64"/>
+      <c r="B16" s="66"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2575,19 +2698,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="63" t="s">
+      <c r="B17" s="65" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="63" t="s">
+      <c r="C17" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="63" t="s">
+      <c r="D17" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="63" t="s">
+      <c r="E17" s="65" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="63" t="s">
+      <c r="F17" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2598,11 +2721,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="64"/>
-      <c r="C18" s="64"/>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
-      <c r="F18" s="64"/>
+      <c r="B18" s="66"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2611,19 +2734,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="59" t="s">
+      <c r="B19" s="61" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="59" t="s">
+      <c r="C19" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="61" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="59" t="s">
+      <c r="E19" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="59" t="s">
+      <c r="F19" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2634,11 +2757,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="60"/>
-      <c r="C20" s="60"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2647,19 +2770,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="63" t="s">
+      <c r="C21" s="65" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="63" t="s">
+      <c r="E21" s="65" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="63" t="s">
+      <c r="F21" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2670,11 +2793,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="64"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2683,19 +2806,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="61" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="59" t="s">
+      <c r="C23" s="61" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="59" t="s">
+      <c r="D23" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="59" t="s">
+      <c r="E23" s="61" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="59" t="s">
+      <c r="F23" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2706,11 +2829,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2719,19 +2842,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="65" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="63" t="s">
+      <c r="C25" s="65" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="63" t="s">
+      <c r="D25" s="65" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="63" t="s">
+      <c r="E25" s="65" t="s">
         <v>181</v>
       </c>
-      <c r="F25" s="63" t="s">
+      <c r="F25" s="65" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2742,11 +2865,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="64"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2843,16 +2966,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9750530-01B1-49BC-B5D5-1F192598EBD5}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBECAA52-033D-415F-829D-FF1056F6C051}">
   <dimension ref="B3:D37"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -2951,9 +3064,15 @@
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B11" s="34"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="19"/>
+      <c r="B11" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="34"/>
@@ -3095,12 +3214,13 @@
     <hyperlink ref="D8" r:id="rId5" xr:uid="{CA4DAE9D-A58B-46BE-8CAD-761CC42C8FC6}"/>
     <hyperlink ref="D9" r:id="rId6" xr:uid="{3F66A6EE-8E9C-4CA9-AC0C-DC07BBAE40E5}"/>
     <hyperlink ref="D10" r:id="rId7" xr:uid="{C932FA4E-851E-4F7C-8642-515FA0A83F91}"/>
+    <hyperlink ref="D11" r:id="rId8" xr:uid="{A89DFE54-4EDF-432C-A25C-C9AE0B123B32}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76621BB5-2A53-4F2F-BF17-3FF097396935}">
   <dimension ref="B2:C3"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -3134,7 +3254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34ADF6CC-94F5-451C-9969-3AA5686D07AE}">
   <dimension ref="B2:F7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -3245,7 +3365,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B48416FD-5E79-4C60-87C7-6AAB59A9E3DF}">
   <dimension ref="B3:D10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -3256,16 +3376,16 @@
   <sheetData>
     <row r="3" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="65" t="s">
+      <c r="B4" s="67" t="s">
         <v>196</v>
       </c>
-      <c r="C4" s="66"/>
-      <c r="D4" s="67"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="39"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="67"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
+      <c r="B5" s="39"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="39"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
@@ -3274,43 +3394,43 @@
       <c r="C6" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="67"/>
+      <c r="D6" s="39"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B7" s="68" t="s">
+      <c r="B7" s="40" t="s">
         <v>198</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="40" t="s">
         <v>199</v>
       </c>
-      <c r="D7" s="67"/>
+      <c r="D7" s="39"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B8" s="68" t="s">
+      <c r="B8" s="40" t="s">
         <v>200</v>
       </c>
-      <c r="C8" s="68" t="s">
+      <c r="C8" s="40" t="s">
         <v>201</v>
       </c>
-      <c r="D8" s="67"/>
-    </row>
-    <row r="9" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="68" t="s">
+      <c r="D8" s="39"/>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="40" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="68" t="s">
+      <c r="C9" s="40" t="s">
         <v>203</v>
       </c>
-      <c r="D9" s="67"/>
-    </row>
-    <row r="10" spans="2:4" ht="30.75" x14ac:dyDescent="0.3">
-      <c r="B10" s="68" t="s">
+      <c r="D9" s="39"/>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="40" t="s">
         <v>204</v>
       </c>
-      <c r="C10" s="68" t="s">
+      <c r="C10" s="40" t="s">
         <v>205</v>
       </c>
-      <c r="D10" s="67"/>
+      <c r="D10" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3319,4 +3439,90 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB534C5F-5069-44F5-BE30-375C8B57A789}">
+  <dimension ref="B2:D7"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.375" customWidth="1"/>
+    <col min="3" max="3" width="17.625" customWidth="1"/>
+    <col min="4" max="4" width="25.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{00A3F4CF-A6BD-4781-B618-D2E727A880EE}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{088482B0-11E1-4715-B3A3-DAFF004D45F8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refine 기타 접속정보 parser to handle optional site column and sync latest Harbor URL
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="675" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5F0E4F0-57FC-4690-8D22-736A1F9A6458}"/>
+  <xr:revisionPtr revIDLastSave="714" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75BCB98F-3BF1-47AF-8233-33332DCC0386}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="(관리자)아카데미 VPN 계정 목록" sheetId="10" r:id="rId8"/>
     <sheet name="(관리자)Trombone 미들웨어 접속정보" sheetId="2" r:id="rId9"/>
     <sheet name="(관리자)Trombone Nodeport" sheetId="11" r:id="rId10"/>
+    <sheet name="(관리자)기타 접속정보" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="225">
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
   </si>
@@ -833,6 +834,22 @@
   </si>
   <si>
     <t>[내부] 온보딩 제품교육222</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Harvor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://harbor.305edu.console.trombone.okestro.cloud/harbor/projects</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Site</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://harbor.okestro.cloud/harbor/projects</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -932,6 +949,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Freesentation 4 Regular"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="6"/>
@@ -1345,6 +1363,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1355,12 +1379,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1877,6 +1895,130 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F37E8A44-3A61-49CE-B701-EBC3CA86DF07}">
+  <dimension ref="B3:E16"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="24.125" customWidth="1"/>
+    <col min="3" max="3" width="20.25" customWidth="1"/>
+    <col min="4" max="4" width="26.5" customWidth="1"/>
+    <col min="5" max="5" width="64.125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B3" s="31" t="s">
+        <v>223</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="20" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="20"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="E4" r:id="rId1" xr:uid="{FD717C43-9745-40FD-A3C6-8BB7B59E29A8}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{53E36623-C7F4-4CD8-B277-9E68C5830378}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{9010E554-3EF9-4D6E-9BCE-15890DB2D7A6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90A17B8-D559-4179-9BBE-8680B873B9EB}">
   <dimension ref="B2:D14"/>
@@ -2476,25 +2618,25 @@
       <c r="F4" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="G4" s="63" t="s">
+      <c r="G4" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="H4" s="64"/>
+      <c r="H4" s="66"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="65" t="s">
+      <c r="B5" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="C5" s="61" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="65" t="s">
+      <c r="D5" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="E5" s="65" t="s">
+      <c r="E5" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="F5" s="65" t="s">
+      <c r="F5" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2505,11 +2647,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="25" t="s">
         <v>95</v>
       </c>
@@ -2518,19 +2660,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="63" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2541,11 +2683,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
       <c r="G8" s="26" t="s">
         <v>95</v>
       </c>
@@ -2554,19 +2696,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="65" t="s">
+      <c r="B9" s="61" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="65" t="s">
+      <c r="C9" s="61" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="65" t="s">
+      <c r="D9" s="61" t="s">
         <v>101</v>
       </c>
-      <c r="E9" s="65" t="s">
+      <c r="E9" s="61" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="65" t="s">
+      <c r="F9" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2577,11 +2719,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="66"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
       <c r="G10" s="25" t="s">
         <v>95</v>
       </c>
@@ -2590,19 +2732,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="63" t="s">
         <v>103</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="61" t="s">
+      <c r="D11" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="63" t="s">
         <v>105</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2613,11 +2755,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
       <c r="G12" s="26" t="s">
         <v>95</v>
       </c>
@@ -2626,19 +2768,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="65" t="s">
+      <c r="B13" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="C13" s="65" t="s">
+      <c r="C13" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="65" t="s">
+      <c r="D13" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="E13" s="65" t="s">
+      <c r="E13" s="61" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="65" t="s">
+      <c r="F13" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2649,11 +2791,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
       <c r="G14" s="25" t="s">
         <v>95</v>
       </c>
@@ -2662,19 +2804,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="65" t="s">
+      <c r="B15" s="61" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="65" t="s">
+      <c r="C15" s="61" t="s">
         <v>76</v>
       </c>
-      <c r="D15" s="65" t="s">
+      <c r="D15" s="61" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="65" t="s">
+      <c r="E15" s="61" t="s">
         <v>110</v>
       </c>
-      <c r="F15" s="65" t="s">
+      <c r="F15" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2685,11 +2827,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="66"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
       <c r="G16" s="25" t="s">
         <v>95</v>
       </c>
@@ -2698,19 +2840,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="65" t="s">
+      <c r="B17" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="C17" s="65" t="s">
+      <c r="C17" s="61" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="65" t="s">
+      <c r="D17" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="65" t="s">
+      <c r="E17" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="65" t="s">
+      <c r="F17" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2721,11 +2863,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="66"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
       <c r="G18" s="25" t="s">
         <v>95</v>
       </c>
@@ -2734,19 +2876,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="63" t="s">
         <v>114</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="63" t="s">
         <v>115</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="63" t="s">
         <v>116</v>
       </c>
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2757,11 +2899,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="64"/>
+      <c r="E20" s="64"/>
+      <c r="F20" s="64"/>
       <c r="G20" s="26" t="s">
         <v>95</v>
       </c>
@@ -2770,19 +2912,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="65" t="s">
+      <c r="B21" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="C21" s="65" t="s">
+      <c r="C21" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="65" t="s">
+      <c r="D21" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="E21" s="65" t="s">
+      <c r="E21" s="61" t="s">
         <v>119</v>
       </c>
-      <c r="F21" s="65" t="s">
+      <c r="F21" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2793,11 +2935,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
+      <c r="B22" s="62"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
       <c r="G22" s="25" t="s">
         <v>95</v>
       </c>
@@ -2806,19 +2948,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="63" t="s">
         <v>120</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="63" t="s">
         <v>160</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="63" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="63" t="s">
         <v>157</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="63" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -2829,11 +2971,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
       <c r="G24" s="26" t="s">
         <v>95</v>
       </c>
@@ -2842,19 +2984,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="65" t="s">
+      <c r="B25" s="61" t="s">
         <v>122</v>
       </c>
-      <c r="C25" s="65" t="s">
+      <c r="C25" s="61" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="65" t="s">
+      <c r="D25" s="61" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="65" t="s">
+      <c r="E25" s="61" t="s">
         <v>181</v>
       </c>
-      <c r="F25" s="65" t="s">
+      <c r="F25" s="61" t="s">
         <v>29</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -2865,11 +3007,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
       <c r="G26" s="25" t="s">
         <v>95</v>
       </c>
@@ -2879,16 +3021,40 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -2901,40 +3067,16 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -3075,29 +3217,59 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B12" s="34"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="19"/>
+      <c r="B12" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B13" s="34"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="19"/>
+      <c r="B13" s="34">
+        <v>46231</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>190</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B14" s="34"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="19"/>
+      <c r="B14" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B15" s="34"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="19"/>
+      <c r="B15" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B16" s="34"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="19"/>
+      <c r="B16" s="34">
+        <v>46232</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17" s="34"/>
@@ -3215,6 +3387,11 @@
     <hyperlink ref="D9" r:id="rId6" xr:uid="{3F66A6EE-8E9C-4CA9-AC0C-DC07BBAE40E5}"/>
     <hyperlink ref="D10" r:id="rId7" xr:uid="{C932FA4E-851E-4F7C-8642-515FA0A83F91}"/>
     <hyperlink ref="D11" r:id="rId8" xr:uid="{A89DFE54-4EDF-432C-A25C-C9AE0B123B32}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{621A8E08-9256-488D-A70A-C5E1B0F691A4}"/>
+    <hyperlink ref="D13" r:id="rId10" xr:uid="{AA824B36-87E5-42C8-98E9-2D2001208BCF}"/>
+    <hyperlink ref="D14" r:id="rId11" xr:uid="{4470E29F-4FAE-4202-9E25-2704221D7787}"/>
+    <hyperlink ref="D15" r:id="rId12" xr:uid="{91DAAECC-701D-4C77-A047-E0AF9997EE5A}"/>
+    <hyperlink ref="D16" r:id="rId13" xr:uid="{9BE5FAA4-1725-428C-BABE-E69D8B806D1C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync updated Excel data for downloads and admin other info
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="714" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75BCB98F-3BF1-47AF-8233-33332DCC0386}"/>
+  <xr:revisionPtr revIDLastSave="760" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8084B9A5-E89D-4C59-8459-38273DDA84A6}"/>
   <bookViews>
-    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="(관리자)Trombone Nodeport" sheetId="11" r:id="rId10"/>
     <sheet name="(관리자)기타 접속정보" sheetId="12" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,12 +46,605 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="236">
+  <si>
+    <t>교육장 WiFi 정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>okestro_guest</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okguest!@</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>일일 출석체크</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>URL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://forms.cloud.microsoft/r/dJWEycjbkL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QR code</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAyAAAAMgCAYAAADbcAZoAAAQAElEQVR4AezbgVbjTK4uUGve/509nW74ISYJiVOyS1X7rHGDQ6KStgwz37rr/m/1fwQIECBAgAABAgQIEDhI4H+L/yNA4CQBxxIgQIAAAQIE5hMQQObbuYkJECBAgAABAgQInCYggJxG72ACBAgQIECAwHwCJiYggHgGCBAgQIAAAQIECBA4TEAAOYx6e5B7AgQIECBAgAABAvMJCCDz7dzEBAgQIECAAAECBE4TEEBOo3cwAQIECBCYT8DEBAgQEEA8AwQIECBAgAABAgTGF+hmQgGkm1VohAABAgQIECBAgMD4AgLI+Ds24VbAPQECBAgQIECAwGkCAshp9A4mQIDAfAImJkCAAAECAohngAABAgQIECAwvoAJCXQjIIB0swqNECBAgAABAgQIEBhfYL4AMv5OTUiAAAECBAgQIECgWwEBpNvVaIzAeAImIkCAAAECBAgIIJ4BAgQIECAwvoAJCRAg0I2AANLNKjRCgAABAgQIECAwnoCJtgICyFbEPQECBAgQIECAAAECaQICSBqtwlsB9wQIECBAgAABAgQEEM8AAQIExhcwIQECBAgQ6EZAAOlmFRohQIAAAQIExhMwEQECWwEBZCvingABAgQIECBAgACBNIHUABIRS8S/K8LXCAYRxxmk/dYkF47IM0puXfmDBCLynpEItSMYRNw3yHzMI+6fG/HezzL7zqwd8d7cET4fwSBin0HWs50aQLKaVpcAgZcEvJkAAQIECBAg0I2AANLNKjRCgAABAuMJmIgAAQIEtgICyFbEPQECBAgQIECAQH0BE3QrIIB0uxqNESBAgAABAgQIEBhPQAAZb6fbidwTIECAAAECBAgQ6EZAAOlmFRohQGA8ARMRIECAAAECWwEBZCvingABAgQIEKgvYAICBLoVEEC6XY3GCBAgQIAAAQIECNQT+K1jAeQ3IT8nQIAAAQIECBAgQKCZgADSjFIhAlsB9wQIECBAgAABAlsBAWQr4p4AAQIE6guYgAABAgS6FRBAul2NxggQIECAAAEC9QR0TOA3AQHkNyE/J0CAAAECBAgQIECgmYAA0oxyW8g9AQIECBAgQIAAAQJbAQFkK+KeAIH6AiYgQIAAAQIEuhUQQLpdjcYIECBAgEA9AR0TIEDgNwEB5DchPydAgAABAgQIECDQv0CZDgWQMqvSKAECBAgQIECAAIH6AgJI/R2aYCvgngABAgQIECBAoFsBAaTb1WiMAAEC9QR0TIAAAQIEfhMQQH4T8nMCBAgQIECAQP8COiRQRkAAKbMqjRIgQIAAAQIECBCoL1A2gKzruty8vF7KpeqvUEQsETkXkxzXiJ91q1pX/duX6V3RpKpHxM/fpYg2r2XuMdO7au1Mb7WP+9+pFZ+/sgGkIraeCYwuYD4CBAgQIECAwG8CAshvQn5OgAABAgT6F9AhAQIEyggIIGVWpVECBAgQIECAAIH+BHT0qoAA8qqY9xMgQIAAAQIECBAgsFtAANlN54NbAfcECBAgQIAAAQIEfhMQQH4T8nMCBAj0L6BDAgQIECBQRkAAKbMqjRIgQIAAAQL9CeiIAIFXBQSQV8W8nwABAgQIECBAgACB3QLNAsjuDnyQAAECBAgQIECAAIFpBASQaVZt0IEFjEaAAAECBAgQKCMggJRZlUYJECBAoD8BHREgQIDAqwICyKti3k+AAAECBAgQIHC+gA7KCgggZVencQIECBAgQIAAAQL1BASQejvbduyeAAECBAgQIECAQBkBAaTMqjRKgEB/AjoiQIAAAQIEXhUQQF4V834CBAgQIEDgfAEdECBQVkAAKbs6jRMgQIAAAQIECBA4XuDdEwWQdwV9ngABAgQIECBAgACBpwUEkKepvJHAVsA9AQIECBAgQIDAqwICyKti3k+AAAEC5wvogAABAgTKCgggZVencQIECBAgQIDA8QJOJPCugADyrqDPEyBAgAABAgQIECDwtIAAcoMqIpaI3665fn6DaeqX1nVdsq5M2Ii85zazb9bXe8u0jrg+K6LdfdYeL3UrmlTsOSLS/vZd9hjR7nmLuK6V6a32tUDEtX2E+2shdwKIZ4AAgXoCOiZAgAABAgTKCgggZVencQIECBAgcLyAEwkQIPCugADyrqDPEyBAgAABAgQIEMgXGOYEAWSYVRqEAAECBAgQIECAQP8CAkj/O9LhVsA9AQIECBAgQIBAWQEBpOzqNE6AAIHjBZxIgAABAgTeFRBA3hX0eQIECBAgQIBAvoATCAwjIIAMs0qDECBAgAABAgQIEOhfoF4A6d9UhwQIECBAgAABAgQI3BEQQO7AeJkAgZ8CXiFAgAABAgQIvCsggLwr6PMECBAgQCBfwAkECBAYRkAAGWaVBiFAgAABAgQIEGgvoGJrAQGktah6BAgQIECAAAECBAjcFRBA7tL4wVbAPQECBAgQIECAAIF3BQSQdwV9ngABAvkCTiBAgAABAsMICCDDrNIgBAgQIECAQHsBFQkQaC0ggLQWVY8AAQIECBAgQIAAgbsCTweQuxX8gAABAgQIECBAgAABAk8KCCBPQnkbgRMFHE2AAAECBAgQGEZAABlmlQYhQIAAgfYCKhIgQIBAawEBpLWoegQIECBAgAABAu8LqDCsgAAy7GoNRoAAAQIECBAgQKA/AQGkv51sO3LfoUBELBE5V+a467ouWVdm3xVrZzlf6lb0uPQckfM7ExGX8q5vApfnJOuKiJJ//yJq9v1trb4lMIyAADLMKg1CgEB7ARUJECBAgACB1gICSGtR9QgQIECAAIH3BVQgQGBYAQFk2NUajAABAgQIECBAgMDrAtmfEECyhdUnQIAAAQIECBAgQOA/AQHkPwrfENgKuCdAgAABAgQIEGgtIIC0FlWPAAECBN4XUIEAAQIEhhUQQIZdrcEIECBAgAABAq8L+ASBbAEBJFtYfQIECBAgQIAAAQIE/hMQQP6j2H7jngABAgQIECBAgACB1gICSGtR9QgQeF9ABQIECBAgQGBYAQFk2NUajAABAgQIvC7gEwQIEMgWEECyhdUnQIAAAQIECBAg8LvANO8QQKZZtUEJECBAgAABAgQInC8ggJy/Ax1sBdwTIECAAAECBAgMKyCADLtagxEgQOB1AZ8gQIAAAQLZAgJItrD6BAgQIECAAIHfBbyDwDQCAsg0qzYoAQIECBAgQIAAgfMF+gsg55vogAABAgQIECBAgACBJAEBJAlWWQIVBfRMgAABAgQIEMgWEECyhdUnQIAAAQK/C3gHAQIEphEQQKZZtUEJECBAgAABAgR+CnjlaAEB5Ghx5xEgQIAAAQIECBCYWEAAmXj529HdPy+wrutS8YqIJSLnyvSIyOk5Qt2Ia4PMPWbWfv63t593ZnpEXO81ot19P4KvdZLp/Von3k2AgADiGSBAgMD5AjogQIAAAQLTCAgg06zaoAQIECBAgMBPAa8QIHC0gABytLjzCBAgQIAAAQIECEws8F8AmdjA6AQIECBAgAABAgQIHCQggBwE7RgCDwT8iAABAgQIECAwjYAAMs2qDUqAAAECPwW8QoAAAQJHCwggR4s7jwABAgQIECBAYFkYTCsggEy7eoMTIECAAAECBAgQOF5AADnefHuiewIECBAgQIAAAQLTCAgg06zaoAQI/BTwCgECBAgQIHC0gABytLjzCBAgQIAAgWVhQIDAtAICyLSrNzgBAgQIECBAgMCMAmfPLICcvQHnEyBAgAABAgQIEJhIQACZaNlG3Qq4J0CAAAECBAgQOFpAADla3HkECBAgsCwMCBAgQGBaAQFk2tUbnAABAgQIEJhRwMwEzhYQQM7egPMJECBAgAABAgQITCQwcQCZaMtGJUCAAAECBAgQINCJgADSySK0QWAqAcMSIECAAAEC0woIINOu3uAECBAgMKOAmQkQIHC2gABy9gacT4AAAQIECBAgMIOAGT8EBJAPCF8IECBAgAABAgQIEMgXEEBuGK/ruriuDW4w7X9pgE9GxBKRcw3A03yErN/H5o0OUDAi57mOqFvX83fcg51lfal73BROuni7/O+oR78JAsgjHT8jQIDAYALGIUCAAAECZwsIIGdvwPkECBAgQIDADAJmJEDgQ0AA+YDwhQABAgQIECBAgACBfIHjA0j+TE4gQIAAAQIECBAgQKBTAQGk08Voi0CGgJoECBAgQIAAgbMFBJCzN+B8AgQIEJhBwIwECBAg8CEggHxA+EKAAAECBAgQIDCigJl6ExBAetuIfggQIECAAAECBAgMLCCADLzc7WjuCRAgQIAAAQIECJwtIICcvQHnEyAwg4AZCRAgQIAAgQ8BAeQDwhcCBAgQIEBgRAEzESDQm4AA0ttG9EOAAAECBAgQIEBgBIE7Mwggd2C8TIAAAQIECBAgQIBAewEBpL2pigS2Au4JECBAgAABAgQ+BASQDwhfCBAgQGBEATMRIECAQG8CAkhvG9EPAQIECBAgQGAEATMQuCMggNyB8TIBAgQIECBAgAABAu0FBJD2ptuK7gkQIECAAAECBAgQ+BAQQD4gfCFAYEQBMxEgQIAAAQK9CQggvW1EPwQIECBAYAQBMxAgQOCOgAByB8bLBAgQIECAAAECBCoK9N5z2QASEUuEK6K2Qe+/IPrrQyAi5zlf13XJujLlsnq+1NV3psB17Yic5zoi0p7r7GfkWqjtXUSed9tOj6sWkWcSoXbEMQbHPTHtTiobQNoRqDSugMkIECBAgAABAgR6ExBAetuIfggQIDCCgBkIECBAgMAdAQHkDoyXCRAgQIAAAQIVBfRMoHcBAaT3DemPAAECBAgQIECAwEACAweQgbZkFAIECBAgQIAAAQKDCAgggyzSGAS6EtAMAQIECBAgQOCOgAByB8bLBAgQIECgooCeCRAg0LuAANL7hvRHgAABAgQIECBQQUCPTwoIIE9CeRsBAgQIECBAgAABAu8LCCDvG6qwFXBPgAABAgQIECBA4I6AAHIHxssECBCoKKBnAgQIECDQu4AA0vuG9EeAAAECBAhUENAjAQJPCgggT0J5GwECBAgQIECAAAEC7wu0DyDv96QCAQIECBAgQIAAAQKDCggggy7WWHMKmJoAAQIECBAg0LuAANL7hvRHgAABAhUE9EiAAAECTwoIIE9CeRsBAgQIECBAgECPAnqqJiCAVNuYfgkQIECAAAECBAgUFhBACi9v27p7AgQIECBAgAABAr0LCCC9b0h/BAhUENAjAQIECBAg8KSAAPIklLcRIECAAAECPQroiQCBagICSLWN6ZcAAQIECBAgQIBADwI7e0gNIOu6Li4GZz0DO38nnvpY5kxPNbDzTVX73jnurx+LiCUi58q0jsjpOSJS/2b/uhBvaCYQUfMZicjruxnuwYUy/5ao7X+j/fYMZD3uqQEkq2l1CXQmoB0CBAgQIECAAIEnBQSQJ6G8jQABAgR6FNATAQIECFQTEECqbUy/BAgQIECAAIEelyNvwQAAEABJREFUBPRAYKeAALITzscIECBAgAABAgQIEHhdQAB53Wz7CfcECBAgQIAAAQIECDwpIIA8CeVtBAj0KKAnAgQIECBAoJqAAFJtY/olQIAAAQI9COiBAAECOwUEkJ1wPkaAAAECBAgQIEDgDIHqZwog1TeofwIECBAgQIAAAQKFBASQQsvS6lbAPQECBAgQIECAQDUBAaTaxvRLgACBHgT0QIAAAQIEdgoIIDvhfIwAAQIECBAgcIaAMwlUFxBAqm9Q/wQIECBAgAABAgQKCRQOIIWUtUqAAAECBAgQIECAwF8BAeQvg38IEHhJwJsJECBAgAABAjsFBJCdcD5GgAABAgTOEHAmAQIEqgsIINU3qH8CBAgQIECAAIEjBJzRSEAAaQSpDAECBAgQIECAAAECvwsIIL8becdWwD0BAgQIECBAgACBnQICyE44HyNAgMAZAs4kQIAAAQLVBQSQ6hvUPwECBAgQIHCEgDMIEGgkIIA0glSGAAECBAgQIECAAIHfBV4PIL/X/O8dEbFEuCLqG/y31MbfRNS3iTBDRDR+Mo4pt67rknVFRNrfv2N02p8SkWeStcdL3Yicvi+1K17tn4yvihU9Lj1H5DwjEfGFk/BdRKT8nUpo9b+SETk9R8R/Z2R8ExEp1hGR0W56zdQAkt69AwhMJmBcAgQIECBAgEB1AQGk+gb1T4AAAQJHCDiDAAECBBoJCCCNIJUhQIAAAQIECBDIEFBzNAEBZLSNmocAAQIECBAgQIBAxwICSMfL2bbmngABAgQIECBAgEB1AQGk+gb1T4DAEQLOIECAAAECBBoJCCCNIJUhQIAAAQIEMgTUJEBgNAEBZLSNmocAAQIECBAgQIBAC4GkGgJIEqyyBAgQIECAAAECBAj8FBBAfpp4hcBWwD0BAgQIECBAgEAjAQGkEaQyBAgQIJAhoCYBAgQIjCYggIy2UfMQIECAAAECBFoIqEEgSUAASYJVlgABAgQIECBAgACBnwICyE+T7SvuCRAgQIAAAQIECBBoJCCANIJUhgCBDAE1CRAgQIAAgdEEBJDRNmoeAgQIECDQQkANAgQIJAkIIEmwyhIgQIAAAQIECBDYIzD6ZwSQ0TdsPgIECBAgQIAAAQIdCQggHS1DK1sB9wQIECBAgAABAqMJCCCjbdQ8BAgQaCGgBgECBAgQSBIQQJJglSVAgAABAgQI7BHwGQKjCwggo2/YfAQIECBAgAABAgQ6Eug4gDxWWtd1yboen+ynLQWydli5bkvfba1Ml+1ZLe+z+m7Z47ZWVs+XutuzWt5HxBKRc7Xsc1srIqfniEj775qIvJ63PlXuI2qaXH4vs66IPJOsnjOft6yeL3Uj8qwzTSLq9V02gGQuUm0C0wsAIECAAAECBAgkCQggSbDKEiBAgACBPQI+Q4AAgdEFBJDRN2w+AgQIECBAgACBZwS85yABAeQgaMcQIECAAAECBAgQILAsAoin4KeAVwgQIECAAAECBAgkCQggSbDKEiBAYI+AzxAgQIAAgdEFBJDRN2w+AgQIECBA4BkB7yFA4CABAeQgaMcQIECAAAECBAgQIHDr/w8IFQIECBAgQIAAAQIECCQJ+H8BSYJVlsAeAZ8hQIAAAQIECIwuIICMvmHzESBAgMAzAt5DgAABAgcJCCAHQTuGAAECBAgQIEDgloDXZhMQQGbbuHkJECBAgAABAgQInCgggJyIvz3aPQECBAgQIECAAIHRBQSQ0TdsPgIEnhHwHgIECBAgQOAgAQHkIGjHECBAgAABArcEvEaAwGwCAshsGzcvAQIECBAgQIAAgYvASZcAchK8YwkQIECAAAECBAjMKCCAzLh1M28F3BMgQIAAAQIECBwkIIAcBO0YAgQIELgl4DUCBAgQmE1AAJlt4+YlQIAAAQIECFwEXAROEhBAToJ3LAECBAgQIECAAIEZBVIDyLquS9bVcFk/SmX1fKn747DJX4iIJaLeNfnabo4fYY83YRJevPwtcV3/90sCs5J3BCLyftczn+s74zR5OSLPpEmDBxeJyPOIyKtd9fmr2HdqADn4eXccAQLlBDRMgAABAgQIzCYggMy2cfMSIECAAIGLgIsAAQInCQggJ8E7lgABAgQIECBAYE6B2acWQGZ/AsxPgAABAgQIECBA4EABAeRAbEdtBdwTIECAAAECBAjMJiCAzLZx8xIgQOAi4CJAgAABAicJCCAnwTuWAAECBAgQmFPA1ARmFxBAZn8CzE+AAAECBAgQIEDgQIETA8iBUzqKAAECBAgQIECAAIEuBASQLtagCQIHCziOAAECBAgQIHCSgAByErxjCRAgQGBOAVMTIEBgdgEBZPYnwPwECBAgQIAAgTkETNmJgADSySK0QYAAAQIECBAgQGAGAQFkhi1vZ3RPgAABAgQIECBA4CQBAeQkeMcSIDCngKkJECBAgMDsAgLI7E+A+QkQIECAwBwCpiRAoBMBAaSTRWiDAAECBAgQIECAwJgC11MJINce7ggQIECAAAECBAgQSBQQQBJxlSawFXBPgAABAgQIEJhdQACZ/QkwPwECBOYQMCUBAgQIdCIggHSyCG0QIECAAAECBMYUMBWBawEB5NrDHQECBAgQIECAAAECiQKpASQiloicK9EkreeIWNZ1LXlleWd6ZPVcuW5Ezu9jRKSyZD0nmU1HRNrfEn3/FMh6Ri51I3J2eamddUXk9BwRP/EbvhIRJX9vsvaYXTcixzu776z6ETkeEbn/+6/hr+BhpVIDyGFTOIgAAQKPBfyUAAECBAgQ6ERAAOlkEdogQIAAAQJjCpiKAAEC1wICyLWHOwIECBAgQIAAAQJjCHQ6hQDS6WK0RYAAAQIECBAgQGBEAQFkxK2aaSvgngABAgQIECBAoBMBAaSTRWiDAAECYwqYigABAgQIXAsIINce7ggQIECAAAECYwiYgkCnAgJIp4vRFgECBAgQIECAAIERBWYIICPuzUwECBAgQIAAAQIESgoIICXXpmkCVQT0SYAAAQIECBC4FhBArj3cESBAgACBMQRMQYAAgU4FBJBOF6MtAgQIECBAgACBmgK6fiwggDz28VMCBAgQIECAAAECBBoKCCANMZXaCrgnQIAAAQIECBAgcC0ggFx7uCNAgMAYAqYgQIAAAQKdCgggnS5GWwQIECBAgEBNAV0TIPBYQAB57OOnBAgQIECAAAECBAg0FEgMIA27VIoAAQIECBAgQIAAgSEEBJAh1mgIAhsBtwQIECBAgACBTgUEkE4Xoy0CBAgQqCmgawIECBB4LCCAPPbxUwIECBAgQIAAgRoCuiwiIIAUWZQ2CRAgQIAAAQIECIwgIIAcvMWIWCKSL/X/GmeuNiJvh5l9r+u6ZF2ZfVesneV8qZvpcamfdUXU/L3J9M6qnbXDS92snrPrRuQ9fxF5tbNdMupH5HlE5NW+PN9ZV4Zz5ZoCSOXt6Z0Age4ENESAAAECBAg8FhBAHvv4KQECBAgQIFBDQJcECBQREECKLEqbBAgQIECAAAECBPoUeK0rAeQ1L+8mQIAAAQIECBAgQOANAQHkDTwfJbAVcE+AAAECBAgQIPBYQAB57OOnBAgQIFBDQJcECBAgUERAACmyKG0SIECAAAECBPoU0BWB1wQEkNe8vJsAAQIECBAgQIAAgTcEBJA38LYfdU+AAAECBAgQIECAwGMBAeSxj58SIFBDQJcECBAgQIBAEQEBpMiitEmAAAECBPoU0BUBAgReExBAXvPybgIECBAgQIAAAQJ9CBTtQgApujhtEyBAgAABAgQIEKgoIIBU3JqetwLuCRAgQIAAAQIEiggIIEUWpU0CBAj0KaArAgQIECDwmoAA8pqXdxMgQIAAAQIE+hDQBYGiAgJI0cVpmwABAgQIECBAgEBFgRECSEV3PRMgQIAAAQIECBCYUkAAmXLthibQSkAdAgQIECBAgMBrAgLIa17eTYAAAQIE+hDQBQECBIoKCCBFF6dtAgQIECBAgACBcwSc+p5AagBZ13XJut4b+7xPZ3mo+/NZy9xyVe+IWCJyrkyTiJyeI9SNuDao+nsTcT1HRLv7LJOIdj1GHFcryyO7bubfqMzaEXm7zey7Yu3MZzAib48RebWzTFIDSFbT6vYioA8CBAgQIECAAAECrwkIIK95eTcBAgT6ENAFAQIECBAoKiCAFF2ctgkQIECAAIFzBJxKgMB7AgLIe34+TYAAAQIECBAgQIDACwJvBJAXTvFWAgQIECBAgAABAgQI/BEQQP4g+A+BcgIaJkCAAAECBAgUFRBAii5O2wQIECBwjoBTCRAgQOA9AQHkPT+fJkCAAAECBAgQOEbAKYMICCCDLNIYBAgQIECAAAECBCoICCAVtrTt0T0BAgQIECBAgACBogICSNHFaZsAgXMEnEqAAAECBAi8JyCAvOfn0wQIECBAgMAxAk4hQGAQAQFkkEUagwABAgQIECBAgECOQNuqAkhbT9UIECBAgAABAgQIEHggIIA8wPEjAlsB9wQIECBAgAABAu8JCCDv+fk0AQIECBwj4BQCBAgQGERAABlkkcYgQIAAAQIECOQIqEqgrYAA0tZTNQIECBAgQIAAAQIEHggIIA9wtj9yT4AAAQIECBAgQIDAewICyHt+Pk2AwDECTiFAgAABAgQGERBABlmkMQgQIECAQI6AqgQIEGgrIIC09VSNAAECBAgQIECAQBuBQaukBpCIWCLqXeu6LllX5nMUUc86Iq/nrB1e6lbd46X3rCvTpGLPmR6ZtSPyficj8mpnPSPq5v334dG2EXnPX0Rebb/v17aZHlVrZ/4uZZmkBpCsptWdTsDABAgQIECAAAECgwgIIIMs0hgECBDIEVCVAAECBAi0FRBA2nqqRoAAAQIECBBoI6AKgUEFBJBBF2ssAgQIECBAgAABAj0KVAggPbrpiQABAgQIECBAgACBHQICyA40HyEwj4BJCRAgQIAAAQJtBQSQtp6qESBAgACBNgKqECBAYFABAWTQxRqLAAECBAgQIEBgn4BP5QoIILm+qhMgQIAAAQIECBAg8E1AAPmG4dutgHsCBAgQIECAAAECbQUEkLaeqhEgQKCNgCoECBAgQGBQAQFk0MUaiwABAgQIENgn4FMECOQKCCC5vqoTIECAAAECBAgQIPBN4EEA+fYu3xIgQIAAAQIECBAgQKCBgADSAFEJAs0FFCRAgAABAgQIDCoggAy6WGMRIECAwD4BnyJAgACBXAEBJNdXdQIECBAgQIAAgecEvGsSAQFkkkUbkwABAgQIECBAgEAPAgJID1vY9uCeAAECBAgQIECAwKACAsigizUWAQL7BHyKAAECBAgQyBUQQHJ9VSdAgAABAgSeE/AuAgQmERBAJlm0MQkQIECAAAECBAjcFjj21dQAsq7rknVlMkXEElHvyrK+1M3yvtTOuiLydpjlkV03oqZJRE7fmd5Zz/WlbmbfmbUvvWddmX1H1NxITmMAABAASURBVHv+InJ6johM6tT/7k1tvGjxir+PmdQRkfYMZllf6maaZNVODSBZTatLIEtAXQIECBAgQIAAgVwBASTXV3UCBAgQeE7AuwgQIEBgEgEBZJJFG5MAAQIECBAgcFvAqwSOFRBAjvV2GgECBAgQIECAAIGpBQSQb+v3LQECBAgQIECAAAECuQICSK6v6gQIPCfgXQQIECBAgMAkAgLIJIs2JgECBAgQuC3gVQIECBwrIIAc6+00AgQIECBAgAABAv8EJv1XAJl08cYmQIAAAQIECBAgcIaAAHKGujO3Au4JECBAgAABAgQmERBAJlm0MQkQIHBbwKsECBAgQOBYAQHkWG+nESBAgAABAgT+CfiXwKQCAsikizc2AQIECBAgQIAAgTMEegggZ8ztTAIECBAgQIAAAQIEThAQQE5AdySBfgR0QoAAAQIECBA4VkAAOdbbaQQIECBA4J+AfwkQIDCpgAAy6eKNTYAAAQIECBCYVcDc5woIIOf6O50AAQIECBAgQIDAVAICyFTr3g7rngABAgQIECBAgMCxAgLIsd5OI0CAwD8B/xIgQIAAgUkFBJBJF29sAgQIECAwq4C5CRA4V0AAOdff6QQIECBAgAABAgRmEfg7Z9kAsq7rUvH6q570T0QsETlXUstp/UZE6vMRkeMcEVnU6t4QyPwbEhFpz/eNUZq9xOQnZZbJz5PavZLV86Vuuy5/VrrUr3j9nKTdK5keETl/p9pNf2ylitYRcSxSo9PKBpBG8ytD4BwBpxIgQIAAAQIEJhUQQCZdvLEJECAwq4C5CRAgQOBcAQHkXH+nEyBAgAABAgRmETAngb8CAshfBv8QIECAAAECBAgQIHCEgAByhPL2DPcECBAgQIAAAQIEJhUQQCZdvLEJzCpgbgIECBAgQOBcAQHkXH+nEyBAgACBWQTMSYAAgb8CAshfBv8QIECAAAECBAgQGFWgr7kEkL72oRsCBAgQIECAAAECQwsIIEOv13BbAfcECBAgQIAAAQLnCggg5/o7nQABArMImJMAAQIECPwVEED+MviHAAECBAgQIDCqgLkI9CUggPS1D90QIECAAAECBAgQGFpgqgAy9CYNR4AAAQIECBAgQKCAgABSYElaJDCAgBEIECBAgAABAn8FBJC/DP4hQIAAAQKjCpiLAAECfQkIIH3tQzcECBAgQIAAAQKjCJjjpoAAcpPFiwQIECBAgAABAgQIZAgIIBmqam4F3BMgQIAAAQIECBD4KyCA/GXwDwECBEYVMBcBAgQIEOhLQADpax+6IUCAAAECBEYRMAcBAjcFBJCbLF4kQIAAAQIECBAgQCBD4IgAktH3EhFpV0rDBxRd13VxfRkcQO6IgwSynuvM9rN6zq4bUfNva0Re3xH1amc+25m1I/KsM/vOrB1RzyTz71REPY/M5+NSO6KeSdkAcgF3ESDwm4CfEyBAgAABAgT6EhBA+tqHbggQIEBgFAFzECBAgMBNAQHkJosXCRAgQIAAAQIEqgrou28BAaTv/eiOAAECBAgQIECAwFACAshQ69wO454AAQIECBAgQIBAXwICSF/70A0BAqMImIMAAQIECBC4KSCA3GTxIgECBAgQIFBVQN8ECPQtIID0vR/dESBAgAABAgQIEKgi8FSfAshTTN5EgAABAgQIECBAgEALAQGkhaIaBLYC7gkQIECAAAECBG4KCCA3WbxIgAABAlUF9E2AAAECfQsIIH3vR3cECBAgQIAAgSoC+iTwlIAA8hSTNxEgQIAAAQIECBAg0EJAAGmhuK3hngABAgQIECBAgACBmwICyE0WLxIgUFVA3wQIECBAgEDfAgJI3/vRHQECBAgQqCKgTwIECDwlIIA8xeRNBAgQIECAAAECBHoVqNWXAFJrX7olQIAAAQIECBAgUFpAACm9Ps1vBdwTIECAAAECBAj0LSCA9L0f3REgQKCKgD4JECBAgMBTAgLIU0zeRIAAAQIECBDoVUBfBGoJCCC19qVbAgQIECBAgAABAqUFUgNIRCwROdct9VavReT0HBHLuq5pV0Re361st3Ui6vW8naHSfdXnLyLnOam0u++9RuR4ROT+jcp8/r77tP4+s++s2q0NvteLqPn8fZ+h0vdZz0hm3Yi8Z6TS7o7qNXOXWTOkBpCsptUlQKA7AQ0RIECAAAECBJ4SEECeYvImAgQIECDQq4C+CBAgUEtAAKm1L90SIECAAAECBAj0IqCPXQICyC42HyJAgAABAgQIECBAYI+AALJHzWe2Au4JECBAgAABAgQIPCUggDzF5E0ECBDoVUBfBAgQIECgloAAUmtfuiVAgAABAgR6EdAHAQK7BASQXWw+RIAAAQIECBAgQIDAHoEWAWTPuT5DgAABAgQIECBAgMCEAgLIhEs38kgCZiFAgAABAgQI1BIQQGrtS7cECBAg0IuAPggQIEBgl4AAsovNhwgQIECAAAECBM4ScG5tAQGk9v50T4AAAQIECBAgQKCUgABSal3bZt0TIECAAAECBAgQqCUggNTal24JEOhFQB8ECBAgQIDALgEBZBebDxEgQIAAAQJnCTiXAIHaAgJI7f3pngABAgQIECBAgMBRAk3OEUCaMCpCgAABAgQIECBAgMAzAgLIM0reQ2Ar4J4AAQIECBAgQGCXgACyi82HCBAgQOAsAecSIECAQG0BAaT2/nRPgAABAgQIEDhKwDkEmggIIE0YFSFAgAABAgQIECBA4BmBsgFkXdcl6/oV7o03RMQSkXO90davH43I6Tlrh5e6vw7lDWUELvvMuDIBInJ+ZyIis+20v08RuX1nPB+fNSMixSVzkRE5PUdEZtspzhGRXjcVJbF4RI7N5+9Ota8ROR4Rkfa/WS/GiY9IWumyASRNRGECBLoW0BwBAgQIECBQW0AAqb0/3RMgQIAAgaMEnEOAAIEmAgJIE0ZFCBAgQIAAAQIECGQJjFVXABlrn6YhQIAAAQIECBAg0LWAANL1ejS3FXBPgAABAgQIECBQW0AAqb0/3RMgQOAoAecQIECAAIEmAgJIE0ZFCBAgQIAAAQJZAuoSGEtAABlrn6YhQIAAAQIECBAg0LVAqQDStaTmCBAgQIAAAQIECBD4VUAA+ZXIGwgQWJYFAgECBAgQIECgiYAA0oRREQIECBAgkCWgLgECBMYSEEDG2qdpCBAgQIAAAQIEWgmokyIggKSwKkqAAAECBAgQIECAwC0BAeSWite2Au4JECBAgAABAgQINBEQQJowKkKAAIEsAXUJECBAgMBYAgLIWPs0DQECBAgQINBKQB0CBFIEBJAUVkUJECBAgAABAgQIELgl8EwAufU5rxEgQIAAAQIECBAgQOBlAQHkZTIfIHCkgLMIECBAgAABAmMJCCBj7dM0BAgQINBKQB0CBAgQSBEQQFJYFSVAgAABAgQIENgr4HNjC5QNIBGxRORcVVe+rutS7YrI2WFEpK6xmvNnvxHh9yb1yfgq/mme8fXrlPbfZfT7WTPC89d+Y7crfppnfL19YptXM/r9rNmmw7GqfNq0/hpR83e9tcP3ehE1TbKe+LIBJAukr7q6IUCAAAECBAgQIDCWgAAy1j5NQ4BAKwF1CBAgQIAAgRQBASSFVVECBAgQIEBgr4DPESAwtoAAMvZ+TUeAAAECBAgQIEDgWYFD3ieAHMLsEAIECBAgQIAAAQIELgICyEXBRWAr4J4AAQIECBAgQCBFQABJYVWUAAECBPYK+BwBAgQIjC0ggIy9X9MRIECAAAECBJ4V8D4ChwgIIIcwO4QAAQIECBAgQIAAgYuAAHJR2F7uCRAgQIAAAQIECBBIERBAUlgVJUBgr4DPESBAgAABAmMLCCBj79d0BAgQIEDgWQHvI0CAwCECAsghzA4hQIAAAQIECBAgcE9grtcFkLn2bVoCBAgQIECAAAECpwoIIKfyO3wr4J4AAQIECBAgQGBsAQFk7P2ajgABAs8KeB8BAgQIEDhEQAA5hNkhBAgQIECAAIF7Al4nMJeAADLXvk1LgAABAgQIECBA4FSBrgLIqRIOJ0CAAAECBAgQIEAgXUAASSd2AIESApokQIAAAQIECBwiIIAcwuwQAgQIECBwT8DrBAgQmEtAAJlr36YlQIAAAQIECBD4FPD1FIGyAWRd18V1bZD5BEXEEtH+ytxhRY+IyGw7tXbmLiMi5fmLqFm3qnXmAxiRt8usviPyeo7Iq131+cvsO7N2RN4us55tHlmyt+tG1HtGygaQ2yvw6k4BHyNAgAABAgQIECBwiIAAcgizQwgQIHBPwOsECBAgQGAuAQFkrn2blgABAgQIEPgU8JUAgVMEBJBT2B1KgAABAgQIECBAYE6BSwCZc3JTEyBAgAABAgQIECBwuIAAcji5Awl8F/A9AQIECBAgQGAuAQFkrn2blgABAgQ+BXwlQIAAgVMEBJBT2B1KgAABAgQIEJhXwORzCwggc+/f9AQIECBAgAABAgQOFRBADuXeHuaeAAECBAgQIECAwFwCAshc+zYtAQKfAr4SIECAAAECpwgIIKewO5QAAQIECMwrYHICBOYWEEDm3r/pCRAgQIAAAQIE5hHoYlIBpIs1aIIAAQIECBAgQIDAHAICyBx7NuVWwD0BAgQIECBAgMApAgLIKewOJUCAwLwCJidAgACBuQUEkLn3b3oCBAgQIEBgHgGTEuhCQADpYg2aIECAAAECBAgQIDCHwJwBZI7dmpIAAQIECBAgQIBAdwICSHcr0RCBsQVMR4AAAQIECMwtIIDMvX/TEyBAgMA8AiYlQIBAFwICSBdr0AQBAgQIECBAgMC4Aib7LiCAfNf4+D4iloic6+OIlC8ROT1HxLKua8oVkddzRF7tLI9L3ZSH46PopX7W9XFEypeKPadAfBSNyHu2P44o9yXrGcmsWw75o+GIvOevqncEk4/Hw5cTBCr+3gggJzwoMx9pdgIECBAgQIAAgbkFBJC59296AgTmETApAQIECBDoQkAA6WINmiBAgAABAgTGFTAZAQLfBQSQ7xq+J0CAAAECBAgQIEAgVeDQAJI6ieIECBAgQIAAAQIECHQvIIB0vyINEmgioAgBAgQIECBAoAsBAaSLNWiCAAECBMYVMBkBAgQIfBcQQL5r+J4AAQIECBAgQGAcAZN0KSCAdLkWTREgQIAAAQIECBAYU0AAGXOv26ncEyBAgAABAgQIEOhCQADpYg2aIEBgXAGTESBAgAABAt8FBJDvGr4nQIAAAQIExhEwCQECXQoIIF2uRVMECBAgQIAAAQIE6go86lwAeaTjZwQIECBAgAABAgQINBUQQJpyKkZgK+CeAAECBAgQIEDgu4AA8l3D9wQIECAwjoBJCBAgQKBLAQGky7VoigABAgQIECBQV0DnBB4JCCCPdPyMAAECBAgQIECAAIGmAgJIU85tMfcECBAgQIAAAQIECHwXEEC+a/ieAIFxBExCgAABAgQIdCkggHS5Fk2mI1kgAAAQAElEQVQRIECAAIG6AjonQIDAIwEB5JGOnxEgQIAAAQIECBCoI1CiUwGkxJrObzIiloj217quS9Z1vtq+DiLaO0f8q7mvo/M/FfGv/4i2XzMny3qus+tWNYlo+2xE5NfL3GXVPWb2HZG306q7zPKOyLPO6vlSNyKvb8/IRfjrEkC+LHw3koBZCBAgQIAAAQIEuhQQQLpci6YIECBQV0DnBAgQIEDgkYAA8kjHzwgQIECAAAECdQR0SqCEgABSYk2aJECAAAECBAgQIDCGwJgBZIzdmIIAAQIECBAgQIDAcAICyHArNRCBcwWcToAAAQIECBB4JCCAPNLxMwIECBAgUEdApwQIECghIICUWJMmCRAgQIAAAQIE+hXQ2SsCAsgrWt5LgAABAgQIECBAgMBbAgLIW3w+vBVwT4AAAQIECBAgQOCRgADySMfPCBAgUEdApwQIECBAoISAAFJiTZokQIAAAQIE+hXQGQECrwgIIK9oeS8BAgQIECBAgAABAm8JNA0gb3XiwwQIECBAgAABAgQIDC8ggAy/YgNOImBMAgQIECBAgEAJAQGkxJo0SYAAAQL9CuiMAAECBF4REEBe0fJeAgQIECBAgACBfgR0UlJAACm5Nk0TIECAAAECBAgQqCkggNTc27Zr9wQIECBAgAABAgRKCAggJdakSQIE+hXQGQECBAgQIPCKgADyipb3EiBAgAABAv0I6IQAgZICAkjJtWmaAAECBAgQIECAwHkC75wsgNzQW9d1yboiYonIubJ6zqwbkWMREWk7vHjceGyavXSpn3VF5Hk3AziwUJbzpW5ETetL71lXBJPvtgc+6k2PisjbY0Re7aYIm2IReX1H1Ku94Wl6+/13qNL3TRE2xSLynpHNUc1uBZBmlArNKWBqAgQIECBAgACBVwQEkFe0vJcAAQIE+hHQCQECBAiUFBBASq5N0wQIECBAgACB8wScTOAdAQHkHT2fJUCAAAECBAgQIEDgJQEB5CWu7ZvdEyBAgAABAgQIECDwioAA8oqW9xIg0I+ATggQIECAAIGSAgJIybVpmgABAgQInCfgZAIECLwjIIC8o+ezBAgQIECAAAECBI4TGOIkAWSINRqCAAECBAgQIECAQA0BAaTGnnS5FXBPgAABAgQIECBQUkAAKbk2TRMgQOA8AScTIECAAIF3BASQd/R8lgABAgQIECBwnICTCAwhIIAMsUZDECBAgAABAgQIEKghUDOA1LDVJQECBAgQIECAAAECGwEBZAPilgCBxwJ+SoAAAQIECBB4R0AAeUfPZwkQIECAwHECTiJAgMAQAgLIEGs0BAECBAgQIECAQJ6Ayi0FBJCWmmoRIECAAAECBAgQIPBQQAB5yOOHWwH3BAgQIECAAAECBN4REEDe0fNZAgQIHCfgJAIECBAgMISAADLEGg1BgAABAgQI5AmoTIBASwEBpKWmWgQIECBAgAABAgQIPBR4KYA8rHTjh+u6LlnXjeNKvJTlcalbAmDT5KXvrGtzVNPbiFgicq6mjW6KZVlf6m6Oanp7qZ9xNW1yUyyj38+am6Oa3kbkPNcR0bTPbbFPm4yvEZH2+x6RUzvDoXrN7TPT8r66Tev+W9pua0Xk/M5E5NbdzjH7fWoAmR3X/AQaCihFgAABAgQIEBhCQAAZYo2GIECAAIE8AZUJECBAoKWAANJSUy0CBAgQIECAAIF2AioNKSCADLlWQxEgQIAAAQIECBDoU0AA6XMv267cEyBAgAABAgQIEBhCQAAZYo2GIEAgT0BlAgQIECBAoKWAANJSUy0CBAgQIECgnYBKBAgMKSCADLlWQxEgQIAAAQIECBDYL5D5SQEkU1dtAgQIECBAgAABAgSuBASQKw43BLYC7gkQIECAAAECBFoKCCAtNdUiQIAAgXYCKhEgQIDAkAICyJBrNRQBAgQIECBAYL+ATxLIFBBAMnXVJkCAAAECBAgQIEDgSkAAueLY3rgnQIAAAQIECBAgQKClgADSUlMtAgTaCahEgAABAgQIDCkggAy5VkMRIECAAIH9Aj5JgACBTAEBJFNXbQIECBAgQIAAAQLPC0zxTgFkijUbkgABAgQIECBAgEAfAgJIH3vQxVbAPQECBAgQIECAwJACAsiQazUUAQIE9gv4JAECBAgQyBQQQDJ11SZAgAABAgQIPC/gnQSmEBBAplizIQkQIECAAAECBAj0IZAaQCJiidhx+Qy3Bs9AH79ir3cR4Xcm4hiD17fTxyci8nwyJ1zXdcm6Kvad2XPV2hE1n+1M7wgm332z/oZk143I22Nm79/tW36fGkBaNqoWAQLHCDiFAAECBAgQIJApIIBk6qpNgAABAgSeF/BOAgQITCEggEyxZkMSIECAAAECBAjcF/CTIwUEkCO1nUWAAAECBAgQIEBgcgEBZPIHYDu+ewIECBAgQIAAAQKZAgJIpq7aBAgQeF7AOwkQIECAwBQCAsgUazYkAQIECBAgcF/ATwgQOFJAADlS21kECBAgQIAAAQIEJhe4CiCTWxifAAECBAgQIECAAIFkAQEkGVh5Ak8KeBsBAgQIECBAYAoBAWSKNRuSAAECBO4L+AkBAgQIHCkggByp7SwCBAgQIECAAIEvAd9NKSCATLl2QxMgQIAAAQIECBA4R0AAOcd9e6p7AgQIECBAgAABAlMICCBTrNmQBAjcF/ATAgQIECBA4EgBAeRIbWcRIECAAAECXwK+I0BgSgEBZMq1G5oAAQIECBAgQGBmgTNnF0DO1Hc2AQIECBAgQIAAgckEBJDJFm7crYB7AgQIECBAgACBIwUEkCO1nUWAAAECXwK+I0CAAIEpBQSQKdduaAIECBAgQGBmAbMTOFNAADlT39kECBAgQIAAAQIEJhMoG0DWdV3ev9Q427Dq71umW6aJvq9/5zOtI2KJyLky95hZO9O7Yu1M64icZy8iKlKX7jnzOakIExFpf1sj8mrb4/XTVjaAXI/hjgCBcgIaJkCAAAECBKYUEECmXLuhCRAgQGBmAbMTIEDgTAEB5Ex9ZxMgQIAAAQIECMwkYNY/AgLIHwT/IUCAAAECBAgQIEDgGAEB5Bhnp2wF3BMgQIAAAQIECEwpIIBMuXZDEyAws4DZCRAgQIDAmQICyJn6ziZAgAABAgRmEjArAQJ/BASQPwj+Q4AAAQIECBAgQIDAMQLnBJBjZnMKAQIECBAgQIAAAQKdCQggnS1EOwSyBdQnQIAAAQIECJwpIICcqe9sAgQIEJhJwKwECBAg8EdAAPmD4D8ECBAgQIAAAQIjC5itJwEBpKdt6IUAAQIECBAgQIDA4AICyOAL3o7nngABAgQIECBAgMCZAgLImfrOJkBgJgGzEiBAgAABAn8EBJA/CP5DgAABAgQIjCxgNgIEehIQQHrahl4IECBAgAABAgQIjCRwYxYB5AaKlwgQIECAAAECBAgQyBEQQHJcVSWwFXBPgAABAgQIECDwR0AA+YPgPwQIECAwsoDZCBAgQKAnAQGkp23ohQABAgQIECAwkoBZCNwQEEBuoETEEuGK+DK4wTT1SxFfNhFtv8+EjWjba8RXvcy+K9Ze13XJuiK+3CPafl/ROrvniLbGEfn1Mk0i8vrP+p251K1qEpHnHZFTO9P6ssuKV6ZJRM4eIyKtbQEkjfaqsBsCBAgQIECAAAECBP4ICCB/EPyHAIGRBcxGgAABAgQI9CQggPS0Db0QIECAAIGRBMxCgACBGwICyA0ULxEgQIAAAQIECBCoLNBz7wJIz9vRGwECBAgQIECAAIHBBASQwRZqnK2AewIECBAgQIAAgZ4EBJCetqEXAgQIjCRgFgIECBAgcENAALmB4iUCBAgQIECAQGUBvRPoWUAA6Xk7eiNAgAABAgQIECAwmMDgAWSwbRmHAAECBAgQIECAQHEBAaT4ArVPoFsBjREgQIAAAQIEbggIIDdQvESAAAECBCoL6J0AAQI9CwggPW9HbwQIECBAgAABApUE9PqEgADyBJK3ECBAgAABAgQIECDQRkAAaeOoylbAPQECBAgQIECAAIEbAgLIDRQvESBAoLKA3gkQIECAQM8CAkjP29EbAQIECBAgUElArwQIPCEggDyB5C0ECBAgQIAAAQIECLQRyAkgbXpThQABAgQIECBAgACBwQQEkMEWahwCBAgQIECAAAECPQsIID1vR28ECBAgUElArwQIECDwhIAA8gSStxAgQIAAAQIECPQsoLdKAgJIpW3pdQqBdV2XrCsTMKvnS92IWCJcEf8MMvcY8e+MiPZfM/tWewyBiPbPXcS/mplCl79TFa9Mk6zaEf/2GdH+a1bPl7oR7fuN+FfzUr/aJYBU29gv/foxAQIECBAgQIAAgZ4FBJCet6M3AgQqCeiVAAECBAgQeEJAAHkCyVsIECBAgACBngX0RoBAJQEBpNK29EqAAAECBAgQIECgJ4EdvQggO9B8hAABAgQIECBAgACBfQICyD43nyKwFXBPgAABAgQIECDwhIAA8gSStxAgQIBAzwJ6I0CAAIFKAgJIpW3plQABAgQIECDQk4BeCOwQEEB2oPkIAQIECBAgQIAAAQL7BASQfW7bT7knQIAAAQIECBAgQOAJAQHkCSRvIUCgZwG9ESBAgAABApUEBJBK29IrAQIECBDoSUAvBAgQ2CEggOxA8xECBAgQIECAAAECZwpUPlsAqbw9vRMgQIAAAQIECBAoJiCAFFuYdrcC7gkQIECAAAECBCoJCCCVtqVXAgQI9CSgFwIECBAgsENAANmB5iMECBAgQIAAgTMFnE2gsoAAUnl7eidAgAABAgQIECBQTKB4ACmmrV0CBAgQIECAAAECkwsIIJM/AMYnsFvABwkQIECAAAECOwQEkB1oPkKAAAECBM4UcDYBAgQqCwgglbendwIECBAgQIAAgSMFnNVAQABpgKgEAQK5Auu6LhlXbtc1q2c4f9bMFImIJSLn+uy/9ddMj9a9fq+X2Xdm7e8ztP4+s++InOc6IlL+rra23dbLtM6svZ2jyn2WiQCSJTt6XfMRIECAAAECBAgQ2CEggOxA8xECBAicKeBsAgQIECBQWUAAqbw9vRMgQIAAAQJHCjiLAIEGAgJIA0QlCBAgQIAAAQIECBB4TmBfAHmutncRIECAAAECBAgQIEDgSkAAueJwQ6B/AR0SIECAAAECBCoLCCCVt6d3AgQIEDhSwFkECBAg0EBAAGmAqAQBAgQIECBAgECmgNojCQggI23TLAQIECBAgAABAgQ6FxBAOl/Qtj33BAgQIECAAAECBCoLCCCVt6d3AgSOFHAWAQIECBAg0EBAAGmAqAQBAgQIECCQKaA2AQIjCQggI23TLAQIECBAgAABAgRaCiTUEkASUJUkQIAAAQIECBAgQOC2gABy28WrBLYC7gkQIECAAAECBBoICCANEJUgQIAAgUwBtQkQIEBgJAEBZKRtmoUAAQIECBAg0FJALQIJAgJIKDdmWgAABlVJREFUAqqSBAgQIECAAAECBAjcFhBAbrtsX3VPgAABAgQIECBAgEADAQGkAaISBAhkCqhNgAABAgQIjCQggIy0TbMQIECAAIGWAmoRIEAgQUAASUBVkgABAgQIECBAgMA7AiN/VgC5sd11XRfXtcENJi8lCUTEEpFzZT7XSRx/y0bkePwtnvRPpnVm7SSO9LJMrokjcn5nIuL6oMZ3VfcYEWl/txsTX5WLyOs7Iqf21QCNbyJyeo6Ixp3WLyeA1N/h4BMYjwABAgQIECBAYCQBAWSkbZqFAAECLQXUIkCAAAECCQICSAKqkgQIECBAgACBdwR8lsDIAgLIyNs1GwECBAgQIECAAIHOBDoPIJ1paYcAAQIECBAgQIAAgbcEBJC3+HyYwMACRiNAgAABAgQIJAgIIAmoShIgQIAAgXcEfJYAAQIjCwggI2/XbAQIECBAgAABAq8IeO8BAgLIAciOIECAAAECBAgQIEDgn4AA8s/Bv1sB9wQIECBAgAABAgQSBASQBFQlCRAg8I6AzxIgQIAAgZEFBJCRt2s2AgQIECBA4BUB7yVA4AABAeQAZEcQIECAAAECBAgQIPBP4HYA+fcz/xIgQIAAAQIECBAgQKCpgADSlFMxAu8LqECAAAECBAgQGFlAABl5u2YjQIAAgVcEvJcAAQIEDhAQQA5AdgQBAgQIECBAgMAjAT+bSUAAmWnbZiVAgAABAgQIECBwsoAAcvICtse7J0CAAAECBAgQIDCygAAy8nbNRoDAKwLeS4AAAQIECBwgIIAcgOwIAgQIECBA4JGAnxEgMJOAADLTts1KgAABAgQIECBA4LvACd+XDSARsUS4ImobnPDMT31kRN7zUhF2Xdcl64rIs46oWbviM5LZc9azd6mb2Xdm7Yiaz/bFPOvK9M6qnWVxqZvV86XupX7WFZH3bF96r3aVDSDVoPXbvYAGCRAgQIAAAQIEDhAQQA5AdgQBAgQIPBLwMwIECBCYSUAAmWnbZiVAgAABAgQIfBfwPYETBASQE9AdSYAAAQIECBAgQGBWAQHk3+b9S4AAAQIECBAgQIDAAQICyAHIjiBA4JGAnxEgQIAAAQIzCQggM23brAQIECBA4LuA7wkQIHCCgAByArojCRAgQIAAAQIE5haYeXoBZObtm50AAQIECBAgQIDAwQICyMHgjtsKuCdAgAABAgQIEJhJQACZadtmJUCAwHcB3xMgQIAAgRMEBJAT0B1JgAABAgQIzC1gegIzCwggM2/f7AQIECBAgAABAgQOFjg5gBw8reMIECBAgAABAgQIEDhVQAA5ld/hBE4UcDQBAgQIECBA4AQBAeQEdEcSIECAwNwCpidAgMDMAgLIzNs3OwECBAgQIEBgLgHTdiAggHSwBC0QIECAAAECBAgQmEVAAJll09s53RMgQIAAAQIECBA4QUAAOQHdkQQIzC1gegIECBAgMLOAADLz9s1OgAABAgTmEjAtAQIdCAggHSxBCwQIECBAgAABAgTGFviaLjWArOu6uBic9Qx8Pebtvztrpp7Pba/8VTFr7q8T2n+X1XPluu2VVbwnUPk5qdj7vT20eJ3HtWKmx/VJbe+q9t1W4ataagD5OsZ3BAh8CvhKgAABAgQIEJhZQACZeftmJ0CAwFwCpiVAgACBDgQEkA6WoAUCBAgQIECAwNgCpiPwJSCAfFn4jgABAgQIECBAgACBZAEBJBl4W949AQIECBAgQIAAgZkFBJCZt292AnMJmJYAAQIECBDoQEAA6WAJWiBAgAABAmMLmI4AAQJfAgLIl4XvCBAgQIAAAQIECIwl0OE0AkiHS9ESAQIECBAgQIAAgVEFBJBRN2uurYB7AgQIECBAgACBDgQEkA6WoAUCBAiMLWA6AgQIECDwJSCAfFn4jgABAgQIECAwloBpCHQoIIB0uBQtESBAgAABAgQIEBhVYJYAMur+zEWAAAECBAgQIECglIAAUmpdmiVQUUDPBAgQIECAAIEvAQHky8J3BAgQIEBgLAHTECBAoEMBAaTDpWiJAAECBAgQIECgtoDu7wsIIPdt/IQAAQIECBAgQIAAgcYCAkhjUOW2Au4JECBAgAABAgQIfAkIIF8WviNAgMBYAqYhQIAAAQIdCgggHS5FSwQIECBAgEBtAd0TIHBf4P8AAAD//197aM0AAAAGSURBVAMAI43gJfhyxMYAAAAASUVORK5CYII=</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>오케스트로 아카데미 솔루션 실습용 VPN계정 목록</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>실습용 노트북 번호를 확인 후 Password로 로그인하세요.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>no.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>VPN ID</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Password</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>rydbr2o26-1</t>
+  </si>
+  <si>
+    <t>EB7TPP7wSqpx</t>
+  </si>
+  <si>
+    <t>rydbr2o26-2</t>
+  </si>
+  <si>
+    <t>nMBFCxkWVak3</t>
+  </si>
+  <si>
+    <t>rydbr2o26-3</t>
+  </si>
+  <si>
+    <t>z9rmYSbbkfvv</t>
+  </si>
+  <si>
+    <t>rydbr2o26-4</t>
+  </si>
+  <si>
+    <t>Kb3cK2H1Fy97</t>
+  </si>
+  <si>
+    <t>rydbr2o26-5</t>
+  </si>
+  <si>
+    <t>il1F98mduykO</t>
+  </si>
+  <si>
+    <t>rydbr2o26-6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0EpB9mbdEIQS</t>
+  </si>
+  <si>
+    <t>rydbr2o26-7</t>
+  </si>
+  <si>
+    <t>91DDYymVM7jz</t>
+  </si>
+  <si>
+    <t>rydbr2o26-8</t>
+  </si>
+  <si>
+    <t>Be6WoeM4w13H</t>
+  </si>
+  <si>
+    <t>rydbr2o26-9</t>
+  </si>
+  <si>
+    <t>D9C373lsNy6F</t>
+  </si>
+  <si>
+    <t>rydbr2o26-10</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>vw1W7i48l47Y</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>솔루션</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노트북 번호</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>교육생 ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>교육생 PW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>접속주소</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
   <si>
     <t>CONTRABASS/VIOLA 3.0.4</t>
-  </si>
-  <si>
-    <t>솔루션</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노트북 1번</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>user1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okestro2026!</t>
+  </si>
+  <si>
+    <t>https://edu.console.304bf.okestro.cloud</t>
+  </si>
+  <si>
+    <t>노트북 2번</t>
+  </si>
+  <si>
+    <t>user2</t>
+  </si>
+  <si>
+    <t>노트북 3번</t>
+  </si>
+  <si>
+    <t>user3</t>
+  </si>
+  <si>
+    <t>i</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노트북 4번</t>
+  </si>
+  <si>
+    <t>user4</t>
+  </si>
+  <si>
+    <t>노트북 5번</t>
+  </si>
+  <si>
+    <t>user5</t>
+  </si>
+  <si>
+    <t>노트북 6번</t>
+  </si>
+  <si>
+    <t>user6</t>
+  </si>
+  <si>
+    <t>노트북 7번</t>
+  </si>
+  <si>
+    <t>user7</t>
+  </si>
+  <si>
+    <t>노트북 8번</t>
+  </si>
+  <si>
+    <t>user8</t>
+  </si>
+  <si>
+    <t>노트북 9번</t>
+  </si>
+  <si>
+    <t>user9</t>
+  </si>
+  <si>
+    <t>노트북 10번</t>
+  </si>
+  <si>
+    <t>user10</t>
+  </si>
+  <si>
+    <t>CONTRABASS/VIOLA 3.0.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okestro2026@</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://edu.console.bf.okestro.cloud/login</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TROMBONE 3.0.5</t>
+  </si>
+  <si>
+    <t>edu01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okestro2026!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://305edu.console.trombone.okestro.cloud/</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>edu02</t>
+  </si>
+  <si>
+    <t>edu03</t>
+  </si>
+  <si>
+    <t>edu04</t>
+  </si>
+  <si>
+    <t>edu05</t>
+  </si>
+  <si>
+    <t>edu06</t>
+  </si>
+  <si>
+    <t>edu07</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>edu08</t>
+  </si>
+  <si>
+    <t>edu10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>edu11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VPN ID</t>
+  </si>
+  <si>
+    <t>user ID</t>
+  </si>
+  <si>
+    <t>업무 코드</t>
+  </si>
+  <si>
+    <t>Git저장소(ID)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Git저장소PW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서비스 접속 주소</t>
+  </si>
+  <si>
+    <t>강사</t>
+  </si>
+  <si>
+    <t>user00</t>
+  </si>
+  <si>
+    <t>USER99</t>
+  </si>
+  <si>
+    <t>EDU99</t>
+  </si>
+  <si>
+    <t>cloud1234</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STG</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31300/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PRD</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31310/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-1</t>
+  </si>
+  <si>
+    <t>user1</t>
+  </si>
+  <si>
+    <t>USER01</t>
+  </si>
+  <si>
+    <t>EDU01</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31301/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31311/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-2</t>
+  </si>
+  <si>
+    <t>USER02</t>
+  </si>
+  <si>
+    <t>EDU02</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31302/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31312/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-3</t>
+  </si>
+  <si>
+    <t>USER03</t>
+  </si>
+  <si>
+    <t>EDU03</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31303/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31313/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-4</t>
+  </si>
+  <si>
+    <t>USER04</t>
+  </si>
+  <si>
+    <t>EDU04</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31304/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31314/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-5</t>
+  </si>
+  <si>
+    <t>USER05</t>
+  </si>
+  <si>
+    <t>EDU05</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31305/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31315/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-6</t>
+  </si>
+  <si>
+    <t>USER06</t>
+  </si>
+  <si>
+    <t>EDU06</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31306/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31316/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-7</t>
+  </si>
+  <si>
+    <t>USER07</t>
+  </si>
+  <si>
+    <t>EDU07</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31307/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31317/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-8</t>
+  </si>
+  <si>
+    <t>USER08</t>
+  </si>
+  <si>
+    <t>EDU08</t>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31308/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31318/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-9</t>
+  </si>
+  <si>
+    <t>user10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER09</t>
+  </si>
+  <si>
+    <t>EDU10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31309/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31319/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>handson-10</t>
+  </si>
+  <si>
+    <t>user11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EDU11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31320/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>http://10.255.62.49:31321/members</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>날짜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[고객사]CONTRABASS 소개 및 기능 교육</t>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgCBIBPxuolZQLyZDp4QQrZmATV-9i46e6T0jsQM4IySD6Q?e=geqmdX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[고객사]VIOLA 소개 및 기능 교육</t>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgBMiVC-RUCOTadlCoEtbrkHAUnfYjbMtLp8HxPN0kwRRYA?e=cxGPtg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[파트너사]CONTRABASS 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgBl5W8IGDwUTIwFI6v1QhpKAVl_Qdeq1lpOLvM8lgK3-Uw?e=pJejqh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[파트너사]VIOLA 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgC6pWckq1-mSKTcy28l6wJPAWSFFsQxH39wxe-7v6r20r8?e=9Jnw5L</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부]CONTRABASS 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqARgbrFbL5rlHoCsHl3GhRH8?e=B0SOs9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부]VIOLA 소개 및 기능 교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAi2tO545GUTJDNTdOSm_WYAT7yjij8h810lxQSSeuNXyo?e=bgPkqw</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부] 온보딩 제품교육</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgA_IZOLdByoTZ3BxYsPq0TbAYfW-iQugsnPW4SoyythDrk?e=iGX2bh</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[내부] 온보딩 제품교육222</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>[고객사]TROMBONE 소개 및 기능 교육</t>
+  </si>
+  <si>
+    <t>다운로드 링크</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CONTRABASS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:u:/g/personal/ws_choi_okekr_onmicrosoft_com/IQDvfs5bsBxIQI9mz5hSAogxAT1VljI4jPHipTx4Woj0a8Q?e=4STXbE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>계정(ID)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>계정(PW)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -63,20 +656,61 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>CONTRABASS/VIOLA 3.0.4</t>
+  </si>
+  <si>
+    <t>admin</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>okestro2018@</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>10.255.62.225 edu.console.304bf.okestro.cloud harbor.okestro.cloud</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://edu.console.304bf.okestro.cloud</t>
-  </si>
-  <si>
     <t>CONTRABASS/VIOLA 3.0.5</t>
   </si>
   <si>
-    <t>TROMBONE 3.0.5</t>
+    <t>bootfactory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okestro2018@</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>10.255.62.69 edu.console.bf.okestro.cloud</t>
+  </si>
+  <si>
+    <t>305edu.console.trombone.okestro.cloud</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sysadmin</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cloud1234!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>10.255.62.49 minio-console.305edu.console.trombone.okestro.cloud alertmanager.305edu.console.trombone.okestro.cloud argocd.305edu.console.trombone.okestro.cloud gitlab.305edu.console.trombone.okestro.cloud grafana.305edu.console.trombone.okestro.cloud harbor.305edu.console.trombone.okestro.cloud jenkins.305edu.console.trombone.okestro.cloud 305edu.console.trombone.okestro.cloud minio-console.305edu.console.trombone.okestro.cloud nexus.305edu.console.trombone.okestro.cloud prometheus.305edu.console.trombone.okestro.cloud sonarqube.305edu.console.trombone.okestro.cloud</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OKESTRO CMP 3.0.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>maestro</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Okestro2018!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>10.255.62.57 edu.console.cmp.okestro.cloud edu.cmp.okestro.cloud</t>
@@ -88,667 +722,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://305edu.console.trombone.okestro.cloud/</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>305edu.console.trombone.okestro.cloud</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>OKESTRO CMP 3.0.5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>계정(ID)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>계정(PW)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>okestro2018@</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Okestro2018@</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Cloud1234!</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Okestro2018!</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>maestro</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>sysadmin</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>bootfactory</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>admin</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>gitlab</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>jenkins</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>argocd</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>nexus</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>harbor</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>cloud1234</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Cloud1234!@</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>root</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>미들웨어</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>10.255.62.49 minio-console.305edu.console.trombone.okestro.cloud alertmanager.305edu.console.trombone.okestro.cloud argocd.305edu.console.trombone.okestro.cloud gitlab.305edu.console.trombone.okestro.cloud grafana.305edu.console.trombone.okestro.cloud harbor.305edu.console.trombone.okestro.cloud jenkins.305edu.console.trombone.okestro.cloud 305edu.console.trombone.okestro.cloud minio-console.305edu.console.trombone.okestro.cloud nexus.305edu.console.trombone.okestro.cloud prometheus.305edu.console.trombone.okestro.cloud sonarqube.305edu.console.trombone.okestro.cloud</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>오케스트로 아카데미 솔루션 실습용 VPN계정 목록</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>실습용 노트북 번호를 확인 후 Password로 로그인하세요.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>Password</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>rydbr2o26-1</t>
-  </si>
-  <si>
-    <t>EB7TPP7wSqpx</t>
-  </si>
-  <si>
-    <t>rydbr2o26-2</t>
-  </si>
-  <si>
-    <t>nMBFCxkWVak3</t>
-  </si>
-  <si>
-    <t>rydbr2o26-3</t>
-  </si>
-  <si>
-    <t>z9rmYSbbkfvv</t>
-  </si>
-  <si>
-    <t>rydbr2o26-4</t>
-  </si>
-  <si>
-    <t>Kb3cK2H1Fy97</t>
-  </si>
-  <si>
-    <t>rydbr2o26-5</t>
-  </si>
-  <si>
-    <t>il1F98mduykO</t>
-  </si>
-  <si>
-    <t>0EpB9mbdEIQS</t>
-  </si>
-  <si>
-    <t>rydbr2o26-7</t>
-  </si>
-  <si>
-    <t>91DDYymVM7jz</t>
-  </si>
-  <si>
-    <t>rydbr2o26-8</t>
-  </si>
-  <si>
-    <t>Be6WoeM4w13H</t>
-  </si>
-  <si>
-    <t>rydbr2o26-9</t>
-  </si>
-  <si>
-    <t>D9C373lsNy6F</t>
-  </si>
-  <si>
-    <t>rydbr2o26-10</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>vw1W7i48l47Y</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>rydbr2o26-6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>no.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>VPN ID</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>교육장 WiFi 정보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PW</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://forms.cloud.microsoft/r/dJWEycjbkL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>URL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>QR code</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAyAAAAMgCAYAAADbcAZoAAAQAElEQVR4AezbgVbjTK4uUGve/509nW74ISYJiVOyS1X7rHGDQ6KStgwz37rr/m/1fwQIECBAgAABAgQIEDhI4H+L/yNA4CQBxxIgQIAAAQIE5hMQQObbuYkJECBAgAABAgQInCYggJxG72ACBAgQIECAwHwCJiYggHgGCBAgQIAAAQIECBA4TEAAOYx6e5B7AgQIECBAgAABAvMJCCDz7dzEBAgQIECAAAECBE4TEEBOo3cwAQIECBCYT8DEBAgQEEA8AwQIECBAgAABAgTGF+hmQgGkm1VohAABAgQIECBAgMD4AgLI+Ds24VbAPQECBAgQIECAwGkCAshp9A4mQIDAfAImJkCAAAECAohngAABAgQIECAwvoAJCXQjIIB0swqNECBAgAABAgQIEBhfYL4AMv5OTUiAAAECBAgQIECgWwEBpNvVaIzAeAImIkCAAAECBAgIIJ4BAgQIECAwvoAJCRAg0I2AANLNKjRCgAABAgQIECAwnoCJtgICyFbEPQECBAgQIECAAAECaQICSBqtwlsB9wQIECBAgAABAgQEEM8AAQIExhcwIQECBAgQ6EZAAOlmFRohQIAAAQIExhMwEQECWwEBZCvingABAgQIECBAgACBNIHUABIRS8S/K8LXCAYRxxmk/dYkF47IM0puXfmDBCLynpEItSMYRNw3yHzMI+6fG/HezzL7zqwd8d7cET4fwSBin0HWs50aQLKaVpcAgZcEvJkAAQIECBAg0I2AANLNKjRCgAABAuMJmIgAAQIEtgICyFbEPQECBAgQIECAQH0BE3QrIIB0uxqNESBAgAABAgQIEBhPQAAZb6fbidwTIECAAAECBAgQ6EZAAOlmFRohQGA8ARMRIECAAAECWwEBZCvingABAgQIEKgvYAICBLoVEEC6XY3GCBAgQIAAAQIECNQT+K1jAeQ3IT8nQIAAAQIECBAgQKCZgADSjFIhAlsB9wQIECBAgAABAlsBAWQr4p4AAQIE6guYgAABAgS6FRBAul2NxggQIECAAAEC9QR0TOA3AQHkNyE/J0CAAAECBAgQIECgmYAA0oxyW8g9AQIECBAgQIAAAQJbAQFkK+KeAIH6AiYgQIAAAQIEuhUQQLpdjcYIECBAgEA9AR0TIEDgNwEB5DchPydAgAABAgQIECDQv0CZDgWQMqvSKAECBAgQIECAAIH6AgJI/R2aYCvgngABAgQIECBAoFsBAaTb1WiMAAEC9QR0TIAAAQIEfhMQQH4T8nMCBAgQIECAQP8COiRQRkAAKbMqjRIgQIAAAQIECBCoL1A2gKzruty8vF7KpeqvUEQsETkXkxzXiJ91q1pX/duX6V3RpKpHxM/fpYg2r2XuMdO7au1Mb7WP+9+pFZ+/sgGkIraeCYwuYD4CBAgQIECAwG8CAshvQn5OgAABAgT6F9AhAQIEyggIIGVWpVECBAgQIECAAIH+BHT0qoAA8qqY9xMgQIAAAQIECBAgsFtAANlN54NbAfcECBAgQIAAAQIEfhMQQH4T8nMCBAj0L6BDAgQIECBQRkAAKbMqjRIgQIAAAQL9CeiIAIFXBQSQV8W8nwABAgQIECBAgACB3QLNAsjuDnyQAAECBAgQIECAAIFpBASQaVZt0IEFjEaAAAECBAgQKCMggJRZlUYJECBAoD8BHREgQIDAqwICyKti3k+AAAECBAgQIHC+gA7KCgggZVencQIECBAgQIAAAQL1BASQejvbduyeAAECBAgQIECAQBkBAaTMqjRKgEB/AjoiQIAAAQIEXhUQQF4V834CBAgQIEDgfAEdECBQVkAAKbs6jRMgQIAAAQIECBA4XuDdEwWQdwV9ngABAgQIECBAgACBpwUEkKepvJHAVsA9AQIECBAgQIDAqwICyKti3k+AAAEC5wvogAABAgTKCgggZVencQIECBAgQIDA8QJOJPCugADyrqDPEyBAgAABAgQIECDwtIAAcoMqIpaI3665fn6DaeqX1nVdsq5M2Ii85zazb9bXe8u0jrg+K6LdfdYeL3UrmlTsOSLS/vZd9hjR7nmLuK6V6a32tUDEtX2E+2shdwKIZ4AAgXoCOiZAgAABAgTKCgggZVencQIECBAgcLyAEwkQIPCugADyrqDPEyBAgAABAgQIEMgXGOYEAWSYVRqEAAECBAgQIECAQP8CAkj/O9LhVsA9AQIECBAgQIBAWQEBpOzqNE6AAIHjBZxIgAABAgTeFRBA3hX0eQIECBAgQIBAvoATCAwjIIAMs0qDECBAgAABAgQIEOhfoF4A6d9UhwQIECBAgAABAgQI3BEQQO7AeJkAgZ8CXiFAgAABAgQIvCsggLwr6PMECBAgQCBfwAkECBAYRkAAGWaVBiFAgAABAgQIEGgvoGJrAQGktah6BAgQIECAAAECBAjcFRBA7tL4wVbAPQECBAgQIECAAIF3BQSQdwV9ngABAvkCTiBAgAABAsMICCDDrNIgBAgQIECAQHsBFQkQaC0ggLQWVY8AAQIECBAgQIAAgbsCTweQuxX8gAABAgQIECBAgAABAk8KCCBPQnkbgRMFHE2AAAECBAgQGEZAABlmlQYhQIAAgfYCKhIgQIBAawEBpLWoegQIECBAgAABAu8LqDCsgAAy7GoNRoAAAQIECBAgQKA/AQGkv51sO3LfoUBELBE5V+a467ouWVdm3xVrZzlf6lb0uPQckfM7ExGX8q5vApfnJOuKiJJ//yJq9v1trb4lMIyAADLMKg1CgEB7ARUJECBAgACB1gICSGtR9QgQIECAAIH3BVQgQGBYAQFk2NUajAABAgQIECBAgMDrAtmfEECyhdUnQIAAAQIECBAgQOA/AQHkPwrfENgKuCdAgAABAgQIEGgtIIC0FlWPAAECBN4XUIEAAQIEhhUQQIZdrcEIECBAgAABAq8L+ASBbAEBJFtYfQIECBAgQIAAAQIE/hMQQP6j2H7jngABAgQIECBAgACB1gICSGtR9QgQeF9ABQIECBAgQGBYAQFk2NUajAABAgQIvC7gEwQIEMgWEECyhdUnQIAAAQIECBAg8LvANO8QQKZZtUEJECBAgAABAgQInC8ggJy/Ax1sBdwTIECAAAECBAgMKyCADLtagxEgQOB1AZ8gQIAAAQLZAgJItrD6BAgQIECAAIHfBbyDwDQCAsg0qzYoAQIECBAgQIAAgfMF+gsg55vogAABAgQIECBAgACBJAEBJAlWWQIVBfRMgAABAgQIEMgWEECyhdUnQIAAAQK/C3gHAQIEphEQQKZZtUEJECBAgAABAgR+CnjlaAEB5Ghx5xEgQIAAAQIECBCYWEAAmXj529HdPy+wrutS8YqIJSLnyvSIyOk5Qt2Ia4PMPWbWfv63t593ZnpEXO81ot19P4KvdZLp/Von3k2AgADiGSBAgMD5AjogQIAAAQLTCAgg06zaoAQIECBAgMBPAa8QIHC0gABytLjzCBAgQIAAAQIECEws8F8AmdjA6AQIECBAgAABAgQIHCQggBwE7RgCDwT8iAABAgQIECAwjYAAMs2qDUqAAAECPwW8QoAAAQJHCwggR4s7jwABAgQIECBAYFkYTCsggEy7eoMTIECAAAECBAgQOF5AADnefHuiewIECBAgQIAAAQLTCAgg06zaoAQI/BTwCgECBAgQIHC0gABytLjzCBAgQIAAgWVhQIDAtAICyLSrNzgBAgQIECBAgMCMAmfPLICcvQHnEyBAgAABAgQIEJhIQACZaNlG3Qq4J0CAAAECBAgQOFpAADla3HkECBAgsCwMCBAgQGBaAQFk2tUbnAABAgQIEJhRwMwEzhYQQM7egPMJECBAgAABAgQITCQwcQCZaMtGJUCAAAECBAgQINCJgADSySK0QWAqAcMSIECAAAEC0woIINOu3uAECBAgMKOAmQkQIHC2gABy9gacT4AAAQIECBAgMIOAGT8EBJAPCF8IECBAgAABAgQIEMgXEEBuGK/ruriuDW4w7X9pgE9GxBKRcw3A03yErN/H5o0OUDAi57mOqFvX83fcg51lfal73BROuni7/O+oR78JAsgjHT8jQIDAYALGIUCAAAECZwsIIGdvwPkECBAgQIDADAJmJEDgQ0AA+YDwhQABAgQIECBAgACBfIHjA0j+TE4gQIAAAQIECBAgQKBTAQGk08Voi0CGgJoECBAgQIAAgbMFBJCzN+B8AgQIEJhBwIwECBAg8CEggHxA+EKAAAECBAgQIDCigJl6ExBAetuIfggQIECAAAECBAgMLCCADLzc7WjuCRAgQIAAAQIECJwtIICcvQHnEyAwg4AZCRAgQIAAgQ8BAeQDwhcCBAgQIEBgRAEzESDQm4AA0ttG9EOAAAECBAgQIEBgBIE7Mwggd2C8TIAAAQIECBAgQIBAewEBpL2pigS2Au4JECBAgAABAgQ+BASQDwhfCBAgQGBEATMRIECAQG8CAkhvG9EPAQIECBAgQGAEATMQuCMggNyB8TIBAgQIECBAgAABAu0FBJD2ptuK7gkQIECAAAECBAgQ+BAQQD4gfCFAYEQBMxEgQIAAAQK9CQggvW1EPwQIECBAYAQBMxAgQOCOgAByB8bLBAgQIECAAAECBCoK9N5z2QASEUuEK6K2Qe+/IPrrQyAi5zlf13XJujLlsnq+1NV3psB17Yic5zoi0p7r7GfkWqjtXUSed9tOj6sWkWcSoXbEMQbHPTHtTiobQNoRqDSugMkIECBAgAABAgR6ExBAetuIfggQIDCCgBkIECBAgMAdAQHkDoyXCRAgQIAAAQIVBfRMoHcBAaT3DemPAAECBAgQIECAwEACAweQgbZkFAIECBAgQIAAAQKDCAgggyzSGAS6EtAMAQIECBAgQOCOgAByB8bLBAgQIECgooCeCRAg0LuAANL7hvRHgAABAgQIECBQQUCPTwoIIE9CeRsBAgQIECBAgAABAu8LCCDvG6qwFXBPgAABAgQIECBA4I6AAHIHxssECBCoKKBnAgQIECDQu4AA0vuG9EeAAAECBAhUENAjAQJPCgggT0J5GwECBAgQIECAAAEC7wu0DyDv96QCAQIECBAgQIAAAQKDCggggy7WWHMKmJoAAQIECBAg0LuAANL7hvRHgAABAhUE9EiAAAECTwoIIE9CeRsBAgQIECBAgECPAnqqJiCAVNuYfgkQIECAAAECBAgUFhBACi9v27p7AgQIECBAgAABAr0LCCC9b0h/BAhUENAjAQIECBAg8KSAAPIklLcRIECAAAECPQroiQCBagICSLWN6ZcAAQIECBAgQIBADwI7e0gNIOu6Li4GZz0DO38nnvpY5kxPNbDzTVX73jnurx+LiCUi58q0jsjpOSJS/2b/uhBvaCYQUfMZicjruxnuwYUy/5ao7X+j/fYMZD3uqQEkq2l1CXQmoB0CBAgQIECAAIEnBQSQJ6G8jQABAgR6FNATAQIECFQTEECqbUy/BAgQIECAAIEelyNvwQAAEABJREFUBPRAYKeAALITzscIECBAgAABAgQIEHhdQAB53Wz7CfcECBAgQIAAAQIECDwpIIA8CeVtBAj0KKAnAgQIECBAoJqAAFJtY/olQIAAAQI9COiBAAECOwUEkJ1wPkaAAAECBAgQIEDgDIHqZwog1TeofwIECBAgQIAAAQKFBASQQsvS6lbAPQECBAgQIECAQDUBAaTaxvRLgACBHgT0QIAAAQIEdgoIIDvhfIwAAQIECBAgcIaAMwlUFxBAqm9Q/wQIECBAgAABAgQKCRQOIIWUtUqAAAECBAgQIECAwF8BAeQvg38IEHhJwJsJECBAgAABAjsFBJCdcD5GgAABAgTOEHAmAQIEqgsIINU3qH8CBAgQIECAAIEjBJzRSEAAaQSpDAECBAgQIECAAAECvwsIIL8becdWwD0BAgQIECBAgACBnQICyE44HyNAgMAZAs4kQIAAAQLVBQSQ6hvUPwECBAgQIHCEgDMIEGgkIIA0glSGAAECBAgQIECAAIHfBV4PIL/X/O8dEbFEuCLqG/y31MbfRNS3iTBDRDR+Mo4pt67rknVFRNrfv2N02p8SkWeStcdL3Yicvi+1K17tn4yvihU9Lj1H5DwjEfGFk/BdRKT8nUpo9b+SETk9R8R/Z2R8ExEp1hGR0W56zdQAkt69AwhMJmBcAgQIECBAgEB1AQGk+gb1T4AAAQJHCDiDAAECBBoJCCCNIJUhQIAAAQIECBDIEFBzNAEBZLSNmocAAQIECBAgQIBAxwICSMfL2bbmngABAgQIECBAgEB1AQGk+gb1T4DAEQLOIECAAAECBBoJCCCNIJUhQIAAAQIEMgTUJEBgNAEBZLSNmocAAQIECBAgQIBAC4GkGgJIEqyyBAgQIECAAAECBAj8FBBAfpp4hcBWwD0BAgQIECBAgEAjAQGkEaQyBAgQIJAhoCYBAgQIjCYggIy2UfMQIECAAAECBFoIqEEgSUAASYJVlgABAgQIECBAgACBnwICyE+T7SvuCRAgQIAAAQIECBBoJCCANIJUhgCBDAE1CRAgQIAAgdEEBJDRNmoeAgQIECDQQkANAgQIJAkIIEmwyhIgQIAAAQIECBDYIzD6ZwSQ0TdsPgIECBAgQIAAAQIdCQggHS1DK1sB9wQIECBAgAABAqMJCCCjbdQ8BAgQaCGgBgECBAgQSBIQQJJglSVAgAABAgQI7BHwGQKjCwggo2/YfAQIECBAgAABAgQ6Eug4gDxWWtd1yboen+ynLQWydli5bkvfba1Ml+1ZLe+z+m7Z47ZWVs+XutuzWt5HxBKRc7Xsc1srIqfniEj775qIvJ63PlXuI2qaXH4vs66IPJOsnjOft6yeL3Uj8qwzTSLq9V02gGQuUm0C0wsAIECAAAECBAgkCQggSbDKEiBAgACBPQI+Q4AAgdEFBJDRN2w+AgQIECBAgACBZwS85yABAeQgaMcQIECAAAECBAgQILAsAoin4KeAVwgQIECAAAECBAgkCQggSbDKEiBAYI+AzxAgQIAAgdEFBJDRN2w+AgQIECBA4BkB7yFA4CABAeQgaMcQIECAAAECBAgQIHDr/w8IFQIECBAgQIAAAQIECCQJ+H8BSYJVlsAeAZ8hQIAAAQIECIwuIICMvmHzESBAgMAzAt5DgAABAgcJCCAHQTuGAAECBAgQIEDgloDXZhMQQGbbuHkJECBAgAABAgQInCgggJyIvz3aPQECBAgQIECAAIHRBQSQ0TdsPgIEnhHwHgIECBAgQOAgAQHkIGjHECBAgAABArcEvEaAwGwCAshsGzcvAQIECBAgQIAAgYvASZcAchK8YwkQIECAAAECBAjMKCCAzLh1M28F3BMgQIAAAQIECBwkIIAcBO0YAgQIELgl4DUCBAgQmE1AAJlt4+YlQIAAAQIECFwEXAROEhBAToJ3LAECBAgQIECAAIEZBVIDyLquS9bVcFk/SmX1fKn747DJX4iIJaLeNfnabo4fYY83YRJevPwtcV3/90sCs5J3BCLyftczn+s74zR5OSLPpEmDBxeJyPOIyKtd9fmr2HdqADn4eXccAQLlBDRMgAABAgQIzCYggMy2cfMSIECAAIGLgIsAAQInCQggJ8E7lgABAgQIECBAYE6B2acWQGZ/AsxPgAABAgQIECBA4EABAeRAbEdtBdwTIECAAAECBAjMJiCAzLZx8xIgQOAi4CJAgAABAicJCCAnwTuWAAECBAgQmFPA1ARmFxBAZn8CzE+AAAECBAgQIEDgQIETA8iBUzqKAAECBAgQIECAAIEuBASQLtagCQIHCziOAAECBAgQIHCSgAByErxjCRAgQGBOAVMTIEBgdgEBZPYnwPwECBAgQIAAgTkETNmJgADSySK0QYAAAQIECBAgQGAGAQFkhi1vZ3RPgAABAgQIECBA4CQBAeQkeMcSIDCngKkJECBAgMDsAgLI7E+A+QkQIECAwBwCpiRAoBMBAaSTRWiDAAECBAgQIECAwJgC11MJINce7ggQIECAAAECBAgQSBQQQBJxlSawFXBPgAABAgQIEJhdQACZ/QkwPwECBOYQMCUBAgQIdCIggHSyCG0QIECAAAECBMYUMBWBawEB5NrDHQECBAgQIECAAAECiQKpASQiloicK9EkreeIWNZ1LXlleWd6ZPVcuW5Ezu9jRKSyZD0nmU1HRNrfEn3/FMh6Ri51I3J2eamddUXk9BwRP/EbvhIRJX9vsvaYXTcixzu776z6ETkeEbn/+6/hr+BhpVIDyGFTOIgAAQKPBfyUAAECBAgQ6ERAAOlkEdogQIAAAQJjCpiKAAEC1wICyLWHOwIECBAgQIAAAQJjCHQ6hQDS6WK0RYAAAQIECBAgQGBEAQFkxK2aaSvgngABAgQIECBAoBMBAaSTRWiDAAECYwqYigABAgQIXAsIINce7ggQIECAAAECYwiYgkCnAgJIp4vRFgECBAgQIECAAIERBWYIICPuzUwECBAgQIAAAQIESgoIICXXpmkCVQT0SYAAAQIECBC4FhBArj3cESBAgACBMQRMQYAAgU4FBJBOF6MtAgQIECBAgACBmgK6fiwggDz28VMCBAgQIECAAAECBBoKCCANMZXaCrgnQIAAAQIECBAgcC0ggFx7uCNAgMAYAqYgQIAAAQKdCgggnS5GWwQIECBAgEBNAV0TIPBYQAB57OOnBAgQIECAAAECBAg0FEgMIA27VIoAAQIECBAgQIAAgSEEBJAh1mgIAhsBtwQIECBAgACBTgUEkE4Xoy0CBAgQqCmgawIECBB4LCCAPPbxUwIECBAgQIAAgRoCuiwiIIAUWZQ2CRAgQIAAAQIECIwgIIAcvMWIWCKSL/X/GmeuNiJvh5l9r+u6ZF2ZfVesneV8qZvpcamfdUXU/L3J9M6qnbXDS92snrPrRuQ9fxF5tbNdMupH5HlE5NW+PN9ZV4Zz5ZoCSOXt6Z0Age4ENESAAAECBAg8FhBAHvv4KQECBAgQIFBDQJcECBQREECKLEqbBAgQIECAAAECBPoUeK0rAeQ1L+8mQIAAAQIECBAgQOANAQHkDTwfJbAVcE+AAAECBAgQIPBYQAB57OOnBAgQIFBDQJcECBAgUERAACmyKG0SIECAAAECBPoU0BWB1wQEkNe8vJsAAQIECBAgQIAAgTcEBJA38LYfdU+AAAECBAgQIECAwGMBAeSxj58SIFBDQJcECBAgQIBAEQEBpMiitEmAAAECBPoU0BUBAgReExBAXvPybgIECBAgQIAAAQJ9CBTtQgApujhtEyBAgAABAgQIEKgoIIBU3JqetwLuCRAgQIAAAQIEiggIIEUWpU0CBAj0KaArAgQIECDwmoAA8pqXdxMgQIAAAQIE+hDQBYGiAgJI0cVpmwABAgQIECBAgEBFgRECSEV3PRMgQIAAAQIECBCYUkAAmXLthibQSkAdAgQIECBAgMBrAgLIa17eTYAAAQIE+hDQBQECBIoKCCBFF6dtAgQIECBAgACBcwSc+p5AagBZ13XJut4b+7xPZ3mo+/NZy9xyVe+IWCJyrkyTiJyeI9SNuDao+nsTcT1HRLv7LJOIdj1GHFcryyO7bubfqMzaEXm7zey7Yu3MZzAib48RebWzTFIDSFbT6vYioA8CBAgQIECAAAECrwkIIK95eTcBAgT6ENAFAQIECBAoKiCAFF2ctgkQIECAAIFzBJxKgMB7AgLIe34+TYAAAQIECBAgQIDACwJvBJAXTvFWAgQIECBAgAABAgQI/BEQQP4g+A+BcgIaJkCAAAECBAgUFRBAii5O2wQIECBwjoBTCRAgQOA9AQHkPT+fJkCAAAECBAgQOEbAKYMICCCDLNIYBAgQIECAAAECBCoICCAVtrTt0T0BAgQIECBAgACBogICSNHFaZsAgXMEnEqAAAECBAi8JyCAvOfn0wQIECBAgMAxAk4hQGAQAQFkkEUagwABAgQIECBAgECOQNuqAkhbT9UIECBAgAABAgQIEHggIIA8wPEjAlsB9wQIECBAgAABAu8JCCDv+fk0AQIECBwj4BQCBAgQGERAABlkkcYgQIAAAQIECOQIqEqgrYAA0tZTNQIECBAgQIAAAQIEHggIIA9wtj9yT4AAAQIECBAgQIDAewICyHt+Pk2AwDECTiFAgAABAgQGERBABlmkMQgQIECAQI6AqgQIEGgrIIC09VSNAAECBAgQIECAQBuBQaukBpCIWCLqXeu6LllX5nMUUc86Iq/nrB1e6lbd46X3rCvTpGLPmR6ZtSPyficj8mpnPSPq5v334dG2EXnPX0Rebb/v17aZHlVrZ/4uZZmkBpCsptWdTsDABAgQIECAAAECgwgIIIMs0hgECBDIEVCVAAECBAi0FRBA2nqqRoAAAQIECBBoI6AKgUEFBJBBF2ssAgQIECBAgAABAj0KVAggPbrpiQABAgQIECBAgACBHQICyA40HyEwj4BJCRAgQIAAAQJtBQSQtp6qESBAgACBNgKqECBAYFABAWTQxRqLAAECBAgQIEBgn4BP5QoIILm+qhMgQIAAAQIECBAg8E1AAPmG4dutgHsCBAgQIECAAAECbQUEkLaeqhEgQKCNgCoECBAgQGBQAQFk0MUaiwABAgQIENgn4FMECOQKCCC5vqoTIECAAAECBAgQIPBN4EEA+fYu3xIgQIAAAQIECBAgQKCBgADSAFEJAs0FFCRAgAABAgQIDCoggAy6WGMRIECAwD4BnyJAgACBXAEBJNdXdQIECBAgQIAAgecEvGsSAQFkkkUbkwABAgQIECBAgEAPAgJID1vY9uCeAAECBAgQIECAwKACAsigizUWAQL7BHyKAAECBAgQyBUQQHJ9VSdAgAABAgSeE/AuAgQmERBAJlm0MQkQIECAAAECBAjcFjj21dQAsq7rknVlMkXEElHvyrK+1M3yvtTOuiLydpjlkV03oqZJRE7fmd5Zz/WlbmbfmbUvvWddmX1H1NxITmMAABAASURBVHv+InJ6johM6tT/7k1tvGjxir+PmdQRkfYMZllf6maaZNVODSBZTatLIEtAXQIECBAgQIAAgVwBASTXV3UCBAgQeE7AuwgQIEBgEgEBZJJFG5MAAQIECBAgcFvAqwSOFRBAjvV2GgECBAgQIECAAIGpBQSQb+v3LQECBAgQIECAAAECuQICSK6v6gQIPCfgXQQIECBAgMAkAgLIJIs2JgECBAgQuC3gVQIECBwrIIAc6+00AgQIECBAgAABAv8EJv1XAJl08cYmQIAAAQIECBAgcIaAAHKGujO3Au4JECBAgAABAgQmERBAJlm0MQkQIHBbwKsECBAgQOBYAQHkWG+nESBAgAABAgT+CfiXwKQCAsikizc2AQIECBAgQIAAgTMEegggZ8ztTAIECBAgQIAAAQIEThAQQE5AdySBfgR0QoAAAQIECBA4VkAAOdbbaQQIECBA4J+AfwkQIDCpgAAy6eKNTYAAAQIECBCYVcDc5woIIOf6O50AAQIECBAgQIDAVAICyFTr3g7rngABAgQIECBAgMCxAgLIsd5OI0CAwD8B/xIgQIAAgUkFBJBJF29sAgQIECAwq4C5CRA4V0AAOdff6QQIECBAgAABAgRmEfg7Z9kAsq7rUvH6q570T0QsETlXUstp/UZE6vMRkeMcEVnU6t4QyPwbEhFpz/eNUZq9xOQnZZbJz5PavZLV86Vuuy5/VrrUr3j9nKTdK5keETl/p9pNf2ylitYRcSxSo9PKBpBG8ytD4BwBpxIgQIAAAQIEJhUQQCZdvLEJECAwq4C5CRAgQOBcAQHkXH+nEyBAgAABAgRmETAngb8CAshfBv8QIECAAAECBAgQIHCEgAByhPL2DPcECBAgQIAAAQIEJhUQQCZdvLEJzCpgbgIECBAgQOBcAQHkXH+nEyBAgACBWQTMSYAAgb8CAshfBv8QIECAAAECBAgQGFWgr7kEkL72oRsCBAgQIECAAAECQwsIIEOv13BbAfcECBAgQIAAAQLnCggg5/o7nQABArMImJMAAQIECPwVEED+MviHAAECBAgQIDCqgLkI9CUggPS1D90QIECAAAECBAgQGFpgqgAy9CYNR4AAAQIECBAgQKCAgABSYElaJDCAgBEIECBAgAABAn8FBJC/DP4hQIAAAQKjCpiLAAECfQkIIH3tQzcECBAgQIAAAQKjCJjjpoAAcpPFiwQIECBAgAABAgQIZAgIIBmqam4F3BMgQIAAAQIECBD4KyCA/GXwDwECBEYVMBcBAgQIEOhLQADpax+6IUCAAAECBEYRMAcBAjcFBJCbLF4kQIAAAQIECBAgQCBD4IgAktH3EhFpV0rDBxRd13VxfRkcQO6IgwSynuvM9rN6zq4bUfNva0Re3xH1amc+25m1I/KsM/vOrB1RzyTz71REPY/M5+NSO6KeSdkAcgF3ESDwm4CfEyBAgAABAgT6EhBA+tqHbggQIEBgFAFzECBAgMBNAQHkJosXCRAgQIAAAQIEqgrou28BAaTv/eiOAAECBAgQIECAwFACAshQ69wO454AAQIECBAgQIBAXwICSF/70A0BAqMImIMAAQIECBC4KSCA3GTxIgECBAgQIFBVQN8ECPQtIID0vR/dESBAgAABAgQIEKgi8FSfAshTTN5EgAABAgQIECBAgEALAQGkhaIaBLYC7gkQIECAAAECBG4KCCA3WbxIgAABAlUF9E2AAAECfQsIIH3vR3cECBAgQIAAgSoC+iTwlIAA8hSTNxEgQIAAAQIECBAg0EJAAGmhuK3hngABAgQIECBAgACBmwICyE0WLxIgUFVA3wQIECBAgEDfAgJI3/vRHQECBAgQqCKgTwIECDwlIIA8xeRNBAgQIECAAAECBHoVqNWXAFJrX7olQIAAAQIECBAgUFpAACm9Ps1vBdwTIECAAAECBAj0LSCA9L0f3REgQKCKgD4JECBAgMBTAgLIU0zeRIAAAQIECBDoVUBfBGoJCCC19qVbAgQIECBAgAABAqUFUgNIRCwROdct9VavReT0HBHLuq5pV0Re361st3Ui6vW8naHSfdXnLyLnOam0u++9RuR4ROT+jcp8/r77tP4+s++s2q0NvteLqPn8fZ+h0vdZz0hm3Yi8Z6TS7o7qNXOXWTOkBpCsptUlQKA7AQ0RIECAAAECBJ4SEECeYvImAgQIECDQq4C+CBAgUEtAAKm1L90SIECAAAECBAj0IqCPXQICyC42HyJAgAABAgQIECBAYI+AALJHzWe2Au4JECBAgAABAgQIPCUggDzF5E0ECBDoVUBfBAgQIECgloAAUmtfuiVAgAABAgR6EdAHAQK7BASQXWw+RIAAAQIECBAgQIDAHoEWAWTPuT5DgAABAgQIECBAgMCEAgLIhEs38kgCZiFAgAABAgQI1BIQQGrtS7cECBAg0IuAPggQIEBgl4AAsovNhwgQIECAAAECBM4ScG5tAQGk9v50T4AAAQIECBAgQKCUgABSal3bZt0TIECAAAECBAgQqCUggNTal24JEOhFQB8ECBAgQIDALgEBZBebDxEgQIAAAQJnCTiXAIHaAgJI7f3pngABAgQIECBAgMBRAk3OEUCaMCpCgAABAgQIECBAgMAzAgLIM0reQ2Ar4J4AAQIECBAgQGCXgACyi82HCBAgQOAsAecSIECAQG0BAaT2/nRPgAABAgQIEDhKwDkEmggIIE0YFSFAgAABAgQIECBA4BmBsgFkXdcl6/oV7o03RMQSkXO90davH43I6Tlrh5e6vw7lDWUELvvMuDIBInJ+ZyIis+20v08RuX1nPB+fNSMixSVzkRE5PUdEZtspzhGRXjcVJbF4RI7N5+9Ota8ROR4Rkfa/WS/GiY9IWumyASRNRGECBLoW0BwBAgQIECBQW0AAqb0/3RMgQIAAgaMEnEOAAIEmAgJIE0ZFCBAgQIAAAQIECGQJjFVXABlrn6YhQIAAAQIECBAg0LWAANL1ejS3FXBPgAABAgQIECBQW0AAqb0/3RMgQOAoAecQIECAAIEmAgJIE0ZFCBAgQIAAAQJZAuoSGEtAABlrn6YhQIAAAQIECBAg0LVAqQDStaTmCBAgQIAAAQIECBD4VUAA+ZXIGwgQWJYFAgECBAgQIECgiYAA0oRREQIECBAgkCWgLgECBMYSEEDG2qdpCBAgQIAAAQIEWgmokyIggKSwKkqAAAECBAgQIECAwC0BAeSWite2Au4JECBAgAABAgQINBEQQJowKkKAAIEsAXUJECBAgMBYAgLIWPs0DQECBAgQINBKQB0CBFIEBJAUVkUJECBAgAABAgQIELgl8EwAufU5rxEgQIAAAQIECBAgQOBlAQHkZTIfIHCkgLMIECBAgAABAmMJCCBj7dM0BAgQINBKQB0CBAgQSBEQQFJYFSVAgAABAgQIENgr4HNjC5QNIBGxRORcVVe+rutS7YrI2WFEpK6xmvNnvxHh9yb1yfgq/mme8fXrlPbfZfT7WTPC89d+Y7crfppnfL19YptXM/r9rNmmw7GqfNq0/hpR83e9tcP3ehE1TbKe+LIBJAukr7q6IUCAAAECBAgQIDCWgAAy1j5NQ4BAKwF1CBAgQIAAgRQBASSFVVECBAgQIEBgr4DPESAwtoAAMvZ+TUeAAAECBAgQIEDgWYFD3ieAHMLsEAIECBAgQIAAAQIELgICyEXBRWAr4J4AAQIECBAgQCBFQABJYVWUAAECBPYK+BwBAgQIjC0ggIy9X9MRIECAAAECBJ4V8D4ChwgIIIcwO4QAAQIECBAgQIAAgYuAAHJR2F7uCRAgQIAAAQIECBBIERBAUlgVJUBgr4DPESBAgAABAmMLCCBj79d0BAgQIEDgWQHvI0CAwCECAsghzA4hQIAAAQIECBAgcE9grtcFkLn2bVoCBAgQIECAAAECpwoIIKfyO3wr4J4AAQIECBAgQGBsAQFk7P2ajgABAs8KeB8BAgQIEDhEQAA5hNkhBAgQIECAAIF7Al4nMJeAADLXvk1LgAABAgQIECBA4FSBrgLIqRIOJ0CAAAECBAgQIEAgXUAASSd2AIESApokQIAAAQIECBwiIIAcwuwQAgQIECBwT8DrBAgQmEtAAJlr36YlQIAAAQIECBD4FPD1FIGyAWRd18V1bZD5BEXEEtH+ytxhRY+IyGw7tXbmLiMi5fmLqFm3qnXmAxiRt8usviPyeo7Iq131+cvsO7N2RN4us55tHlmyt+tG1HtGygaQ2yvw6k4BHyNAgAABAgQIECBwiIAAcgizQwgQIHBPwOsECBAgQGAuAQFkrn2blgABAgQIEPgU8JUAgVMEBJBT2B1KgAABAgQIECBAYE6BSwCZc3JTEyBAgAABAgQIECBwuIAAcji5Awl8F/A9AQIECBAgQGAuAQFkrn2blgABAgQ+BXwlQIAAgVMEBJBT2B1KgAABAgQIEJhXwORzCwggc+/f9AQIECBAgAABAgQOFRBADuXeHuaeAAECBAgQIECAwFwCAshc+zYtAQKfAr4SIECAAAECpwgIIKewO5QAAQIECMwrYHICBOYWEEDm3r/pCRAgQIAAAQIE5hHoYlIBpIs1aIIAAQIECBAgQIDAHAICyBx7NuVWwD0BAgQIECBAgMApAgLIKewOJUCAwLwCJidAgACBuQUEkLn3b3oCBAgQIEBgHgGTEuhCQADpYg2aIECAAAECBAgQIDCHwJwBZI7dmpIAAQIECBAgQIBAdwICSHcr0RCBsQVMR4AAAQIECMwtIIDMvX/TEyBAgMA8AiYlQIBAFwICSBdr0AQBAgQIECBAgMC4Aib7LiCAfNf4+D4iloic6+OIlC8ROT1HxLKua8oVkddzRF7tLI9L3ZSH46PopX7W9XFEypeKPadAfBSNyHu2P44o9yXrGcmsWw75o+GIvOevqncEk4/Hw5cTBCr+3gggJzwoMx9pdgIECBAgQIAAgbkFBJC59296AgTmETApAQIECBDoQkAA6WINmiBAgAABAgTGFTAZAQLfBQSQ7xq+J0CAAAECBAgQIEAgVeDQAJI6ieIECBAgQIAAAQIECHQvIIB0vyINEmgioAgBAgQIECBAoAsBAaSLNWiCAAECBMYVMBkBAgQIfBcQQL5r+J4AAQIECBAgQGAcAZN0KSCAdLkWTREgQIAAAQIECBAYU0AAGXOv26ncEyBAgAABAgQIEOhCQADpYg2aIEBgXAGTESBAgAABAt8FBJDvGr4nQIAAAQIExhEwCQECXQoIIF2uRVMECBAgQIAAAQIE6go86lwAeaTjZwQIECBAgAABAgQINBUQQJpyKkZgK+CeAAECBAgQIEDgu4AA8l3D9wQIECAwjoBJCBAgQKBLAQGky7VoigABAgQIECBQV0DnBB4JCCCPdPyMAAECBAgQIECAAIGmAgJIU85tMfcECBAgQIAAAQIECHwXEEC+a/ieAIFxBExCgAABAgQIdCkggHS5Fk2mI1kgAAAQAElEQVQRIECAAIG6AjonQIDAIwEB5JGOnxEgQIAAAQIECBCoI1CiUwGkxJrObzIiloj217quS9Z1vtq+DiLaO0f8q7mvo/M/FfGv/4i2XzMny3qus+tWNYlo+2xE5NfL3GXVPWb2HZG306q7zPKOyLPO6vlSNyKvb8/IRfjrEkC+LHw3koBZCBAgQIAAAQIEuhQQQLpci6YIECBQV0DnBAgQIEDgkYAA8kjHzwgQIECAAAECdQR0SqCEgABSYk2aJECAAAECBAgQIDCGwJgBZIzdmIIAAQIECBAgQIDAcAICyHArNRCBcwWcToAAAQIECBB4JCCAPNLxMwIECBAgUEdApwQIECghIICUWJMmCRAgQIAAAQIE+hXQ2SsCAsgrWt5LgAABAgQIECBAgMBbAgLIW3w+vBVwT4AAAQIECBAgQOCRgADySMfPCBAgUEdApwQIECBAoISAAFJiTZokQIAAAQIE+hXQGQECrwgIIK9oeS8BAgQIECBAgAABAm8JNA0gb3XiwwQIECBAgAABAgQIDC8ggAy/YgNOImBMAgQIECBAgEAJAQGkxJo0SYAAAQL9CuiMAAECBF4REEBe0fJeAgQIECBAgACBfgR0UlJAACm5Nk0TIECAAAECBAgQqCkggNTc27Zr9wQIECBAgAABAgRKCAggJdakSQIE+hXQGQECBAgQIPCKgADyipb3EiBAgAABAv0I6IQAgZICAkjJtWmaAAECBAgQIECAwHkC75wsgNzQW9d1yboiYonIubJ6zqwbkWMREWk7vHjceGyavXSpn3VF5Hk3AziwUJbzpW5ETetL71lXBJPvtgc+6k2PisjbY0Re7aYIm2IReX1H1Ku94Wl6+/13qNL3TRE2xSLynpHNUc1uBZBmlArNKWBqAgQIECBAgACBVwQEkFe0vJcAAQIE+hHQCQECBAiUFBBASq5N0wQIECBAgACB8wScTOAdAQHkHT2fJUCAAAECBAgQIEDgJQEB5CWu7ZvdEyBAgAABAgQIECDwioAA8oqW9xIg0I+ATggQIECAAIGSAgJIybVpmgABAgQInCfgZAIECLwjIIC8o+ezBAgQIECAAAECBI4TGOIkAWSINRqCAAECBAgQIECAQA0BAaTGnnS5FXBPgAABAgQIECBQUkAAKbk2TRMgQOA8AScTIECAAIF3BASQd/R8lgABAgQIECBwnICTCAwhIIAMsUZDECBAgAABAgQIEKghUDOA1LDVJQECBAgQIECAAAECGwEBZAPilgCBxwJ+SoAAAQIECBB4R0AAeUfPZwkQIECAwHECTiJAgMAQAgLIEGs0BAECBAgQIECAQJ6Ayi0FBJCWmmoRIECAAAECBAgQIPBQQAB5yOOHWwH3BAgQIECAAAECBN4REEDe0fNZAgQIHCfgJAIECBAgMISAADLEGg1BgAABAgQI5AmoTIBASwEBpKWmWgQIECBAgAABAgQIPBR4KYA8rHTjh+u6LlnXjeNKvJTlcalbAmDT5KXvrGtzVNPbiFgicq6mjW6KZVlf6m6Oanp7qZ9xNW1yUyyj38+am6Oa3kbkPNcR0bTPbbFPm4yvEZH2+x6RUzvDoXrN7TPT8r66Tev+W9pua0Xk/M5E5NbdzjH7fWoAmR3X/AQaCihFgAABAgQIEBhCQAAZYo2GIECAAIE8AZUJECBAoKWAANJSUy0CBAgQIECAAIF2AioNKSCADLlWQxEgQIAAAQIECBDoU0AA6XMv267cEyBAgAABAgQIEBhCQAAZYo2GIEAgT0BlAgQIECBAoKWAANJSUy0CBAgQIECgnYBKBAgMKSCADLlWQxEgQIAAAQIECBDYL5D5SQEkU1dtAgQIECBAgAABAgSuBASQKw43BLYC7gkQIECAAAECBFoKCCAtNdUiQIAAgXYCKhEgQIDAkAICyJBrNRQBAgQIECBAYL+ATxLIFBBAMnXVJkCAAAECBAgQIEDgSkAAueLY3rgnQIAAAQIECBAgQKClgADSUlMtAgTaCahEgAABAgQIDCkggAy5VkMRIECAAIH9Aj5JgACBTAEBJFNXbQIECBAgQIAAAQLPC0zxTgFkijUbkgABAgQIECBAgEAfAgJIH3vQxVbAPQECBAgQIECAwJACAsiQazUUAQIE9gv4JAECBAgQyBQQQDJ11SZAgAABAgQIPC/gnQSmEBBAplizIQkQIECAAAECBAj0IZAaQCJiidhx+Qy3Bs9AH79ir3cR4Xcm4hiD17fTxyci8nwyJ1zXdcm6Kvad2XPV2hE1n+1M7wgm332z/oZk143I22Nm79/tW36fGkBaNqoWAQLHCDiFAAECBAgQIJApIIBk6qpNgAABAgSeF/BOAgQITCEggEyxZkMSIECAAAECBAjcF/CTIwUEkCO1nUWAAAECBAgQIEBgcgEBZPIHYDu+ewIECBAgQIAAAQKZAgJIpq7aBAgQeF7AOwkQIECAwBQCAsgUazYkAQIECBAgcF/ATwgQOFJAADlS21kECBAgQIAAAQIEJhe4CiCTWxifAAECBAgQIECAAIFkAQEkGVh5Ak8KeBsBAgQIECBAYAoBAWSKNRuSAAECBO4L+AkBAgQIHCkggByp7SwCBAgQIECAAIEvAd9NKSCATLl2QxMgQIAAAQIECBA4R0AAOcd9e6p7AgQIECBAgAABAlMICCBTrNmQBAjcF/ATAgQIECBA4EgBAeRIbWcRIECAAAECXwK+I0BgSgEBZMq1G5oAAQIECBAgQGBmgTNnF0DO1Hc2AQIECBAgQIAAgckEBJDJFm7crYB7AgQIECBAgACBIwUEkCO1nUWAAAECXwK+I0CAAIEpBQSQKdduaAIECBAgQGBmAbMTOFNAADlT39kECBAgQIAAAQIEJhMoG0DWdV3ev9Q427Dq71umW6aJvq9/5zOtI2KJyLky95hZO9O7Yu1M64icZy8iKlKX7jnzOakIExFpf1sj8mrb4/XTVjaAXI/hjgCBcgIaJkCAAAECBKYUEECmXLuhCRAgQGBmAbMTIEDgTAEB5Ex9ZxMgQIAAAQIECMwkYNY/AgLIHwT/IUCAAAECBAgQIEDgGAEB5Bhnp2wF3BMgQIAAAQIECEwpIIBMuXZDEyAws4DZCRAgQIDAmQICyJn6ziZAgAABAgRmEjArAQJ/BASQPwj+Q4AAAQIECBAgQIDAMQLnBJBjZnMKAQIECBAgQIAAAQKdCQggnS1EOwSyBdQnQIAAAQIECJwpIICcqe9sAgQIEJhJwKwECBAg8EdAAPmD4D8ECBAgQIAAAQIjC5itJwEBpKdt6IUAAQIECBAgQIDA4AICyOAL3o7nngABAgQIECBAgMCZAgLImfrOJkBgJgGzEiBAgAABAn8EBJA/CP5DgAABAgQIjCxgNgIEehIQQHrahl4IECBAgAABAgQIjCRwYxYB5AaKlwgQIECAAAECBAgQyBEQQHJcVSWwFXBPgAABAgQIECDwR0AA+YPgPwQIECAwsoDZCBAgQKAnAQGkp23ohQABAgQIECAwkoBZCNwQEEBuoETEEuGK+DK4wTT1SxFfNhFtv8+EjWjba8RXvcy+K9Ze13XJuiK+3CPafl/ROrvniLbGEfn1Mk0i8vrP+p251K1qEpHnHZFTO9P6ssuKV6ZJRM4eIyKtbQEkjfaqsBsCBAgQIECAAAECBP4ICCB/EPyHAIGRBcxGgAABAgQI9CQggPS0Db0QIECAAIGRBMxCgACBGwICyA0ULxEgQIAAAQIECBCoLNBz7wJIz9vRGwECBAgQIECAAIHBBASQwRZqnK2AewIECBAgQIAAgZ4EBJCetqEXAgQIjCRgFgIECBAgcENAALmB4iUCBAgQIECAQGUBvRPoWUAA6Xk7eiNAgAABAgQIECAwmMDgAWSwbRmHAAECBAgQIECAQHEBAaT4ArVPoFsBjREgQIAAAQIEbggIIDdQvESAAAECBCoL6J0AAQI9CwggPW9HbwQIECBAgAABApUE9PqEgADyBJK3ECBAgAABAgQIECDQRkAAaeOoylbAPQECBAgQIECAAIEbAgLIDRQvESBAoLKA3gkQIECAQM8CAkjP29EbAQIECBAgUElArwQIPCEggDyB5C0ECBAgQIAAAQIECLQRyAkgbXpThQABAgQIECBAgACBwQQEkMEWahwCBAgQIECAAAECPQsIID1vR28ECBAgUElArwQIECDwhIAA8gSStxAgQIAAAQIECPQsoLdKAgJIpW3pdQqBdV2XrCsTMKvnS92IWCJcEf8MMvcY8e+MiPZfM/tWewyBiPbPXcS/mplCl79TFa9Mk6zaEf/2GdH+a1bPl7oR7fuN+FfzUr/aJYBU29gv/foxAQIECBAgQIAAgZ4FBJCet6M3AgQqCeiVAAECBAgQeEJAAHkCyVsIECBAgACBngX0RoBAJQEBpNK29EqAAAECBAgQIECgJ4EdvQggO9B8hAABAgQIECBAgACBfQICyD43nyKwFXBPgAABAgQIECDwhIAA8gSStxAgQIBAzwJ6I0CAAIFKAgJIpW3plQABAgQIECDQk4BeCOwQEEB2oPkIAQIECBAgQIAAAQL7BASQfW7bT7knQIAAAQIECBAgQOAJAQHkCSRvIUCgZwG9ESBAgAABApUEBJBK29IrAQIECBDoSUAvBAgQ2CEggOxA8xECBAgQIECAAAECZwpUPlsAqbw9vRMgQIAAAQIECBAoJiCAFFuYdrcC7gkQIECAAAECBCoJCCCVtqVXAgQI9CSgFwIECBAgsENAANmB5iMECBAgQIAAgTMFnE2gsoAAUnl7eidAgAABAgQIECBQTKB4ACmmrV0CBAgQIECAAAECkwsIIJM/AMYnsFvABwkQIECAAAECOwQEkB1oPkKAAAECBM4UcDYBAgQqCwgglbendwIECBAgQIAAgSMFnNVAQABpgKgEAQK5Auu6LhlXbtc1q2c4f9bMFImIJSLn+uy/9ddMj9a9fq+X2Xdm7e8ztP4+s++InOc6IlL+rra23dbLtM6svZ2jyn2WiQCSJTt6XfMRIECAAAECBAgQ2CEggOxA8xECBAicKeBsAgQIECBQWUAAqbw9vRMgQIAAAQJHCjiLAIEGAgJIA0QlCBAgQIAAAQIECBB4TmBfAHmutncRIECAAAECBAgQIEDgSkAAueJwQ6B/AR0SIECAAAECBCoLCCCVt6d3AgQIEDhSwFkECBAg0EBAAGmAqAQBAgQIECBAgECmgNojCQggI23TLAQIECBAgAABAgQ6FxBAOl/Qtj33BAgQIECAAAECBCoLCCCVt6d3AgSOFHAWAQIECBAg0EBAAGmAqAQBAgQIECCQKaA2AQIjCQggI23TLAQIECBAgAABAgRaCiTUEkASUJUkQIAAAQIECBAgQOC2gABy28WrBLYC7gkQIECAAAECBBoICCANEJUgQIAAgUwBtQkQIEBgJAEBZKRtmoUAAQIECBAg0FJALQIJAgJIKDdmWgAABlVJREFUAqqSBAgQIECAAAECBAjcFhBAbrtsX3VPgAABAgQIECBAgEADAQGkAaISBAhkCqhNgAABAgQIjCQggIy0TbMQIECAAIGWAmoRIEAgQUAASUBVkgABAgQIECBAgMA7AiN/VgC5sd11XRfXtcENJi8lCUTEEpFzZT7XSRx/y0bkePwtnvRPpnVm7SSO9LJMrokjcn5nIuL6oMZ3VfcYEWl/txsTX5WLyOs7Iqf21QCNbyJyeo6Ixp3WLyeA1N/h4BMYjwABAgQIECBAYCQBAWSkbZqFAAECLQXUIkCAAAECCQICSAKqkgQIECBAgACBdwR8lsDIAgLIyNs1GwECBAgQIECAAIHOBDoPIJ1paYcAAQIECBAgQIAAgbcEBJC3+HyYwMACRiNAgAABAgQIJAgIIAmoShIgQIAAgXcEfJYAAQIjCwggI2/XbAQIECBAgAABAq8IeO8BAgLIAciOIECAAAECBAgQIEDgn4AA8s/Bv1sB9wQIECBAgAABAgQSBASQBFQlCRAg8I6AzxIgQIAAgZEFBJCRt2s2AgQIECBA4BUB7yVA4AABAeQAZEcQIECAAAECBAgQIPBP4HYA+fcz/xIgQIAAAQIECBAgQKCpgADSlFMxAu8LqECAAAECBAgQGFlAABl5u2YjQIAAgVcEvJcAAQIEDhAQQA5AdgQBAgQIECBAgMAjAT+bSUAAmWnbZiVAgAABAgQIECBwsoAAcvICtse7J0CAAAECBAgQIDCygAAy8nbNRoDAKwLeS4AAAQIECBwgIIAcgOwIAgQIECBA4JGAnxEgMJOAADLTts1KgAABAgQIECBA4LvACd+XDSARsUS4ImobnPDMT31kRN7zUhF2Xdcl64rIs46oWbviM5LZc9azd6mb2Xdm7Yiaz/bFPOvK9M6qnWVxqZvV86XupX7WFZH3bF96r3aVDSDVoPXbvYAGCRAgQIAAAQIEDhAQQA5AdgQBAgQIPBLwMwIECBCYSUAAmWnbZiVAgAABAgQIfBfwPYETBASQE9AdSYAAAQIECBAgQGBWAQHk3+b9S4AAAQIECBAgQIDAAQICyAHIjiBA4JGAnxEgQIAAAQIzCQggM23brAQIECBA4LuA7wkQIHCCgAByArojCRAgQIAAAQIE5haYeXoBZObtm50AAQIECBAgQIDAwQICyMHgjtsKuCdAgAABAgQIEJhJQACZadtmJUCAwHcB3xMgQIAAgRMEBJAT0B1JgAABAgQIzC1gegIzCwggM2/f7AQIECBAgAABAgQOFjg5gBw8reMIECBAgAABAgQIEDhVQAA5ld/hBE4UcDQBAgQIECBA4AQBAeQEdEcSIECAwNwCpidAgMDMAgLIzNs3OwECBAgQIEBgLgHTdiAggHSwBC0QIECAAAECBAgQmEVAAJll09s53RMgQIAAAQIECBA4QUAAOQHdkQQIzC1gegIECBAgMLOAADLz9s1OgAABAgTmEjAtAQIdCAggHSxBCwQIECBAgAABAgTGFviaLjWArOu6uBic9Qx8Pebtvztrpp7Pba/8VTFr7q8T2n+X1XPluu2VVbwnUPk5qdj7vT20eJ3HtWKmx/VJbe+q9t1W4ataagD5OsZ3BAh8CvhKgAABAgQIEJhZQACZeftmJ0CAwFwCpiVAgACBDgQEkA6WoAUCBAgQIECAwNgCpiPwJSCAfFn4jgABAgQIECBAgACBZAEBJBl4W949AQIECBAgQIAAgZkFBJCZt292AnMJmJYAAQIECBDoQEAA6WAJWiBAgAABAmMLmI4AAQJfAgLIl4XvCBAgQIAAAQIECIwl0OE0AkiHS9ESAQIECBAgQIAAgVEFBJBRN2uurYB7AgQIECBAgACBDgQEkA6WoAUCBAiMLWA6AgQIECDwJSCAfFn4jgABAgQIECAwloBpCHQoIIB0uBQtESBAgAABAgQIEBhVYJYAMur+zEWAAAECBAgQIECglIAAUmpdmiVQUUDPBAgQIECAAIEvAQHky8J3BAgQIEBgLAHTECBAoEMBAaTDpWiJAAECBAgQIECgtoDu7wsIIPdt/IQAAQIECBAgQIAAgcYCAkhjUOW2Au4JECBAgAABAgQIfAkIIF8WviNAgMBYAqYhQIAAAQIdCgggHS5FSwQIECBAgEBtAd0TIHBf4P8AAAD//197aM0AAAAGSURBVAMAI43gJfhyxMYAAAAASUVORK5CYII=</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>okestro_guest</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Okguest!@</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>일일 출석체크</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>교육생 ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>교육생 PW</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>user1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Okestro2026@</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>user2</t>
-  </si>
-  <si>
-    <t>user3</t>
-  </si>
-  <si>
-    <t>user4</t>
-  </si>
-  <si>
-    <t>user5</t>
-  </si>
-  <si>
-    <t>user6</t>
-  </si>
-  <si>
-    <t>user7</t>
-  </si>
-  <si>
-    <t>user8</t>
-  </si>
-  <si>
-    <t>user9</t>
-  </si>
-  <si>
-    <t>user10</t>
-  </si>
-  <si>
-    <t>i</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Okestro2026!</t>
-  </si>
-  <si>
-    <t>CONTRABASS/VIOLA 3.0.5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>접속주소</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VPN ID</t>
-  </si>
-  <si>
-    <t>user ID</t>
-  </si>
-  <si>
-    <t>업무 코드</t>
-  </si>
-  <si>
-    <t>서비스 접속 주소</t>
-  </si>
-  <si>
-    <t>강사</t>
-  </si>
-  <si>
-    <t>user00</t>
-  </si>
-  <si>
-    <t>USER99</t>
-  </si>
-  <si>
-    <t>EDU99</t>
-  </si>
-  <si>
-    <t>STG</t>
-  </si>
-  <si>
-    <t>PRD</t>
-  </si>
-  <si>
-    <t>handson-1</t>
-  </si>
-  <si>
-    <t>user1</t>
-  </si>
-  <si>
-    <t>USER01</t>
-  </si>
-  <si>
-    <t>EDU01</t>
-  </si>
-  <si>
-    <t>handson-2</t>
-  </si>
-  <si>
-    <t>USER02</t>
-  </si>
-  <si>
-    <t>EDU02</t>
-  </si>
-  <si>
-    <t>handson-3</t>
-  </si>
-  <si>
-    <t>USER03</t>
-  </si>
-  <si>
-    <t>EDU03</t>
-  </si>
-  <si>
-    <t>handson-4</t>
-  </si>
-  <si>
-    <t>USER04</t>
-  </si>
-  <si>
-    <t>handson-5</t>
-  </si>
-  <si>
-    <t>USER05</t>
-  </si>
-  <si>
-    <t>EDU05</t>
-  </si>
-  <si>
-    <t>handson-6</t>
-  </si>
-  <si>
-    <t>USER06</t>
-  </si>
-  <si>
-    <t>EDU06</t>
-  </si>
-  <si>
-    <t>handson-7</t>
-  </si>
-  <si>
-    <t>USER07</t>
-  </si>
-  <si>
-    <t>EDU07</t>
-  </si>
-  <si>
-    <t>handson-8</t>
-  </si>
-  <si>
-    <t>USER08</t>
-  </si>
-  <si>
-    <t>EDU08</t>
-  </si>
-  <si>
-    <t>handson-9</t>
-  </si>
-  <si>
-    <t>USER09</t>
-  </si>
-  <si>
-    <t>handson-10</t>
-  </si>
-  <si>
-    <t>EDU04</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31300/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31310/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31301/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31311/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31302/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31312/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31303/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31313/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31304/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31314/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31305/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31315/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31306/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31316/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31307/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31317/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31308/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31318/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31309/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31319/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31320/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>http://10.255.62.49:31321/members</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>edu01</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>edu02</t>
-  </si>
-  <si>
-    <t>edu03</t>
-  </si>
-  <si>
-    <t>edu04</t>
-  </si>
-  <si>
-    <t>edu05</t>
-  </si>
-  <si>
-    <t>edu06</t>
-  </si>
-  <si>
-    <t>edu08</t>
-  </si>
-  <si>
-    <t>Okestro2026!</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>edu07</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CONTRABASS/VIOLA 3.0.4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://edu.console.bf.okestro.cloud/login</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EDU10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>edu10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>edu11</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>user10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>user11</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USER10</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>노트북 번호</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>노트북 1번</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>노트북 2번</t>
-  </si>
-  <si>
-    <t>노트북 3번</t>
-  </si>
-  <si>
-    <t>노트북 4번</t>
-  </si>
-  <si>
-    <t>노트북 5번</t>
-  </si>
-  <si>
-    <t>노트북 6번</t>
-  </si>
-  <si>
-    <t>노트북 7번</t>
-  </si>
-  <si>
-    <t>노트북 8번</t>
-  </si>
-  <si>
-    <t>노트북 9번</t>
-  </si>
-  <si>
-    <t>노트북 10번</t>
-  </si>
-  <si>
-    <t>날짜</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CONTRABASS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:u:/g/personal/ws_choi_okekr_onmicrosoft_com/IQDvfs5bsBxIQI9mz5hSAogxAT1VljI4jPHipTx4Woj0a8Q?e=4STXbE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>다운로드 링크</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[고객사]CONTRABASS 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[파트너사]CONTRABASS 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EDU11</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Git저장소(ID)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Git저장소PW</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgCBIBPxuolZQLyZDp4QQrZmATV-9i46e6T0jsQM4IySD6Q?e=geqmdX</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgBMiVC-RUCOTadlCoEtbrkHAUnfYjbMtLp8HxPN0kwRRYA?e=cxGPtg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[고객사]VIOLA 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgBl5W8IGDwUTIwFI6v1QhpKAVl_Qdeq1lpOLvM8lgK3-Uw?e=pJejqh</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgC6pWckq1-mSKTcy28l6wJPAWSFFsQxH39wxe-7v6r20r8?e=9Jnw5L</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[내부]CONTRABASS 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[내부]VIOLA 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[파트너사]VIOLA 소개 및 기능 교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgDh4vpInDFXQKvW1x5ujldqARgbrFbL5rlHoCsHl3GhRH8?e=B0SOs9</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAi2tO545GUTJDNTdOSm_WYAT7yjij8h810lxQSSeuNXyo?e=bgPkqw</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[내부] 온보딩 제품교육</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgA_IZOLdByoTZ3BxYsPq0TbAYfW-iQugsnPW4SoyythDrk?e=iGX2bh</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>오케스트로 아카데미 VPN계정 목록</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -787,10 +760,50 @@
     <t>Okestro2018!</t>
   </si>
   <si>
+    <t>미들웨어</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>gitlab</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>root</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jenkins</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>argocd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cloud1234!@</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>nexus</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>harbor</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>User</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>stg</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prd</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>user00</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -825,15 +838,7 @@
     <t>user11</t>
   </si>
   <si>
-    <t>stg</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>prd</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[내부] 온보딩 제품교육222</t>
+    <t>Site</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -845,11 +850,47 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Site</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>http://harbor.okestro.cloud/harbor/projects</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">3.0.4 Harbor </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cloud1234</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>harbor.okestro.cloud</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TROMBONE sonarqube</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Cloud1234!@#$</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">  / </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">TROMBONE sonarqube  // </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgD2-Cw1hAmtRLRZS6xQPynlAQSBcVBpAkyIeyOHZ55FjV0?e=99uB1U</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgB9iV0PmZzyRY-OX9_l3D7vAdoSOalS0_nW4EuL1EQk16I?e=dUjOQs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAeSH61MkiqTKogyAAEH0v1AQNWhsstioRHFrdxMBQ7FN8?e=7qWeI5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1677,46 +1718,46 @@
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="41" t="s">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="C4" s="41"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>66</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="42" t="s">
-        <v>68</v>
+        <v>5</v>
       </c>
       <c r="C8" s="42"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="160.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="19" t="s">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.3">
@@ -1748,18 +1789,18 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C3" s="14">
         <v>31300</v>
@@ -1770,7 +1811,7 @@
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C4" s="14">
         <v>31301</v>
@@ -1781,7 +1822,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C5" s="14">
         <v>31302</v>
@@ -1792,7 +1833,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C6" s="14">
         <v>31303</v>
@@ -1803,7 +1844,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C7" s="14">
         <v>31304</v>
@@ -1814,7 +1855,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C8" s="21">
         <v>31305</v>
@@ -1825,7 +1866,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C9" s="21">
         <v>31306</v>
@@ -1836,7 +1877,7 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C10" s="21">
         <v>31307</v>
@@ -1847,7 +1888,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C11" s="21">
         <v>31308</v>
@@ -1858,7 +1899,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C12" s="21">
         <v>31309</v>
@@ -1869,7 +1910,7 @@
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="C13" s="21">
         <v>31320</v>
@@ -1880,7 +1921,7 @@
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="C14" s="21">
         <v>31322</v>
@@ -1897,7 +1938,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F37E8A44-3A61-49CE-B701-EBC3CA86DF07}">
-  <dimension ref="B3:E16"/>
+  <dimension ref="B3:E26"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.125" customWidth="1"/>
@@ -1908,50 +1949,62 @@
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="31" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>61</v>
+        <v>3</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>63</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>30</v>
+        <v>205</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
       <c r="E5" s="20" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="20"/>
+      <c r="B6" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
+      <c r="B7" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>230</v>
+      </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
@@ -2007,6 +2060,16 @@
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
       <c r="E16" s="19"/>
+    </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D25" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D26" t="s">
+        <v>232</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2014,6 +2077,7 @@
     <hyperlink ref="E4" r:id="rId1" xr:uid="{FD717C43-9745-40FD-A3C6-8BB7B59E29A8}"/>
     <hyperlink ref="D4" r:id="rId2" xr:uid="{53E36623-C7F4-4CD8-B277-9E68C5830378}"/>
     <hyperlink ref="E5" r:id="rId3" xr:uid="{9010E554-3EF9-4D6E-9BCE-15890DB2D7A6}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{948E4DB6-DF70-4D82-8F68-DE92E21CBC1C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2031,27 +2095,27 @@
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
       <c r="B2" s="43" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C2" s="43"/>
       <c r="D2" s="43"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="44" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C3" s="45"/>
       <c r="D3" s="45"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -2059,10 +2123,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -2070,10 +2134,10 @@
         <v>2</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -2081,10 +2145,10 @@
         <v>3</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -2092,10 +2156,10 @@
         <v>4</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -2103,10 +2167,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -2114,10 +2178,10 @@
         <v>6</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -2125,10 +2189,10 @@
         <v>7</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
@@ -2136,10 +2200,10 @@
         <v>8</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -2147,10 +2211,10 @@
         <v>9</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
@@ -2158,10 +2222,10 @@
         <v>10</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2186,45 +2250,45 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="9" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>163</v>
+        <v>36</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" s="46" t="s">
-        <v>155</v>
+        <v>40</v>
       </c>
       <c r="C3" s="30" t="s">
-        <v>164</v>
+        <v>41</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="E3" s="52" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="47"/>
       <c r="C4" s="30" t="s">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E4" s="53"/>
       <c r="F4" s="50"/>
@@ -2232,24 +2296,24 @@
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="47"/>
       <c r="C5" s="30" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E5" s="53"/>
       <c r="F5" s="50"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="B6" s="47"/>
       <c r="C6" s="30" t="s">
-        <v>167</v>
+        <v>50</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E6" s="53"/>
       <c r="F6" s="50"/>
@@ -2257,10 +2321,10 @@
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B7" s="47"/>
       <c r="C7" s="30" t="s">
-        <v>168</v>
+        <v>52</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="E7" s="53"/>
       <c r="F7" s="50"/>
@@ -2268,10 +2332,10 @@
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" s="47"/>
       <c r="C8" s="30" t="s">
-        <v>169</v>
+        <v>54</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E8" s="53"/>
       <c r="F8" s="50"/>
@@ -2279,10 +2343,10 @@
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B9" s="47"/>
       <c r="C9" s="30" t="s">
-        <v>170</v>
+        <v>56</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E9" s="53"/>
       <c r="F9" s="50"/>
@@ -2290,10 +2354,10 @@
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" s="47"/>
       <c r="C10" s="30" t="s">
-        <v>171</v>
+        <v>58</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E10" s="53"/>
       <c r="F10" s="50"/>
@@ -2301,10 +2365,10 @@
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11" s="47"/>
       <c r="C11" s="30" t="s">
-        <v>172</v>
+        <v>60</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E11" s="53"/>
       <c r="F11" s="50"/>
@@ -2312,38 +2376,38 @@
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" s="48"/>
       <c r="C12" s="30" t="s">
-        <v>173</v>
+        <v>62</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E12" s="54"/>
       <c r="F12" s="51"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B13" s="55" t="s">
-        <v>84</v>
+        <v>64</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>164</v>
+        <v>41</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="E13" s="49" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F13" s="58" t="s">
-        <v>156</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B14" s="56"/>
       <c r="C14" s="30" t="s">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E14" s="50"/>
       <c r="F14" s="59"/>
@@ -2351,10 +2415,10 @@
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B15" s="56"/>
       <c r="C15" s="30" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E15" s="50"/>
       <c r="F15" s="59"/>
@@ -2362,10 +2426,10 @@
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B16" s="56"/>
       <c r="C16" s="30" t="s">
-        <v>167</v>
+        <v>50</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E16" s="50"/>
       <c r="F16" s="59"/>
@@ -2373,10 +2437,10 @@
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B17" s="56"/>
       <c r="C17" s="30" t="s">
-        <v>168</v>
+        <v>52</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="E17" s="50"/>
       <c r="F17" s="59"/>
@@ -2384,10 +2448,10 @@
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B18" s="56"/>
       <c r="C18" s="30" t="s">
-        <v>169</v>
+        <v>54</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E18" s="50"/>
       <c r="F18" s="59"/>
@@ -2395,10 +2459,10 @@
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B19" s="56"/>
       <c r="C19" s="30" t="s">
-        <v>170</v>
+        <v>56</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E19" s="50"/>
       <c r="F19" s="59"/>
@@ -2406,10 +2470,10 @@
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" s="56"/>
       <c r="C20" s="30" t="s">
-        <v>171</v>
+        <v>58</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E20" s="50"/>
       <c r="F20" s="59"/>
@@ -2417,10 +2481,10 @@
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" s="56"/>
       <c r="C21" s="30" t="s">
-        <v>172</v>
+        <v>60</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E21" s="50"/>
       <c r="F21" s="59"/>
@@ -2428,38 +2492,38 @@
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" s="57"/>
       <c r="C22" s="30" t="s">
-        <v>173</v>
+        <v>62</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="E22" s="51"/>
       <c r="F22" s="60"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="55" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="C23" s="30" t="s">
-        <v>164</v>
+        <v>41</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>146</v>
+        <v>68</v>
       </c>
       <c r="E23" s="49" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="F23" s="58" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" s="56"/>
       <c r="C24" s="30" t="s">
-        <v>165</v>
+        <v>45</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>147</v>
+        <v>71</v>
       </c>
       <c r="E24" s="50"/>
       <c r="F24" s="59"/>
@@ -2467,10 +2531,10 @@
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" s="56"/>
       <c r="C25" s="30" t="s">
-        <v>166</v>
+        <v>47</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>148</v>
+        <v>72</v>
       </c>
       <c r="E25" s="50"/>
       <c r="F25" s="59"/>
@@ -2478,10 +2542,10 @@
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" s="56"/>
       <c r="C26" s="30" t="s">
-        <v>167</v>
+        <v>50</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>149</v>
+        <v>73</v>
       </c>
       <c r="E26" s="50"/>
       <c r="F26" s="59"/>
@@ -2489,10 +2553,10 @@
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" s="56"/>
       <c r="C27" s="30" t="s">
-        <v>168</v>
+        <v>52</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>150</v>
+        <v>74</v>
       </c>
       <c r="E27" s="50"/>
       <c r="F27" s="59"/>
@@ -2500,10 +2564,10 @@
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" s="56"/>
       <c r="C28" s="30" t="s">
-        <v>169</v>
+        <v>54</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>151</v>
+        <v>75</v>
       </c>
       <c r="E28" s="50"/>
       <c r="F28" s="59"/>
@@ -2511,10 +2575,10 @@
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" s="56"/>
       <c r="C29" s="30" t="s">
-        <v>170</v>
+        <v>56</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>154</v>
+        <v>76</v>
       </c>
       <c r="E29" s="50"/>
       <c r="F29" s="59"/>
@@ -2522,10 +2586,10 @@
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" s="56"/>
       <c r="C30" s="30" t="s">
-        <v>171</v>
+        <v>58</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>152</v>
+        <v>77</v>
       </c>
       <c r="E30" s="50"/>
       <c r="F30" s="59"/>
@@ -2533,10 +2597,10 @@
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B31" s="56"/>
       <c r="C31" s="30" t="s">
-        <v>172</v>
+        <v>60</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>158</v>
+        <v>78</v>
       </c>
       <c r="E31" s="50"/>
       <c r="F31" s="59"/>
@@ -2544,10 +2608,10 @@
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" s="57"/>
       <c r="C32" s="30" t="s">
-        <v>173</v>
+        <v>62</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>159</v>
+        <v>79</v>
       </c>
       <c r="E32" s="51"/>
       <c r="F32" s="60"/>
@@ -2604,46 +2668,46 @@
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>182</v>
+        <v>83</v>
       </c>
       <c r="F4" s="37" t="s">
-        <v>183</v>
+        <v>84</v>
       </c>
       <c r="G4" s="65" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H4" s="66"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="61" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="61" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="G5" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="H5" t="s">
         <v>92</v>
-      </c>
-      <c r="E5" s="61" t="s">
-        <v>93</v>
-      </c>
-      <c r="F5" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>94</v>
-      </c>
-      <c r="H5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2653,33 +2717,33 @@
       <c r="E6" s="62"/>
       <c r="F6" s="62"/>
       <c r="G6" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H6" s="27" t="s">
-        <v>125</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="C7" s="63" t="s">
+      <c r="D7" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="E7" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="F7" s="63" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H7" s="27" t="s">
         <v>99</v>
-      </c>
-      <c r="F7" s="63" t="s">
-        <v>29</v>
-      </c>
-      <c r="G7" s="26" t="s">
-        <v>94</v>
-      </c>
-      <c r="H7" s="27" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2689,33 +2753,33 @@
       <c r="E8" s="64"/>
       <c r="F8" s="64"/>
       <c r="G8" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H8" s="27" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="61" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C9" s="61" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="D9" s="61" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E9" s="61" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F9" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G9" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2725,33 +2789,33 @@
       <c r="E10" s="62"/>
       <c r="F10" s="62"/>
       <c r="G10" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H10" s="27" t="s">
-        <v>129</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="63" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C11" s="63" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="D11" s="63" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="E11" s="63" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F11" s="63" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H11" s="27" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2761,33 +2825,33 @@
       <c r="E12" s="64"/>
       <c r="F12" s="64"/>
       <c r="G12" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H12" s="27" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="61" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C13" s="61" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="D13" s="61" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E13" s="61" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="F13" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G13" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H13" s="27" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2797,33 +2861,33 @@
       <c r="E14" s="62"/>
       <c r="F14" s="62"/>
       <c r="G14" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="61" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="C15" s="61" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="D15" s="61" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="E15" s="61" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="F15" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H15" s="27" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2833,33 +2897,33 @@
       <c r="E16" s="62"/>
       <c r="F16" s="62"/>
       <c r="G16" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="61" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C17" s="61" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="D17" s="61" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="E17" s="61" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="F17" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2869,33 +2933,33 @@
       <c r="E18" s="62"/>
       <c r="F18" s="62"/>
       <c r="G18" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H18" s="27" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="63" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="C19" s="63" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="D19" s="63" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="E19" s="63" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="F19" s="63" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G19" s="26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H19" s="27" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2905,33 +2969,33 @@
       <c r="E20" s="64"/>
       <c r="F20" s="64"/>
       <c r="G20" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="61" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="C21" s="61" t="s">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="D21" s="61" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="E21" s="61" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="F21" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G21" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H21" s="27" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2941,33 +3005,33 @@
       <c r="E22" s="62"/>
       <c r="F22" s="62"/>
       <c r="G22" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="63" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="C23" s="63" t="s">
-        <v>160</v>
+        <v>137</v>
       </c>
       <c r="D23" s="63" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="E23" s="63" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="F23" s="63" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G23" s="26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H23" s="27" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2977,33 +3041,33 @@
       <c r="E24" s="64"/>
       <c r="F24" s="64"/>
       <c r="G24" s="26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H24" s="27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="61" t="s">
-        <v>122</v>
+        <v>142</v>
       </c>
       <c r="C25" s="61" t="s">
-        <v>161</v>
+        <v>143</v>
       </c>
       <c r="D25" s="61" t="s">
-        <v>162</v>
+        <v>144</v>
       </c>
       <c r="E25" s="61" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="F25" s="61" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H25" s="27" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3013,10 +3077,10 @@
       <c r="E26" s="62"/>
       <c r="F26" s="62"/>
       <c r="G26" s="25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="H26" s="27" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3112,20 +3176,20 @@
   <dimension ref="B3:D37"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.125" style="35" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" style="35" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.375" customWidth="1"/>
     <col min="4" max="4" width="140.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="33" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>63</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
@@ -3133,10 +3197,10 @@
         <v>46217</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>179</v>
+        <v>150</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>184</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -3144,10 +3208,10 @@
         <v>46218</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>186</v>
+        <v>152</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>185</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -3155,10 +3219,10 @@
         <v>46224</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>187</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -3166,10 +3230,10 @@
         <v>46225</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>191</v>
+        <v>156</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>188</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -3177,10 +3241,10 @@
         <v>46230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>189</v>
+        <v>158</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>192</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -3188,10 +3252,10 @@
         <v>46231</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -3199,10 +3263,10 @@
         <v>46232</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -3210,10 +3274,10 @@
         <v>46232</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>220</v>
+        <v>164</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
@@ -3221,10 +3285,10 @@
         <v>46232</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>220</v>
+        <v>164</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -3232,10 +3296,10 @@
         <v>46231</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>193</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
@@ -3243,42 +3307,52 @@
         <v>46232</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>195</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B15" s="34">
-        <v>46232</v>
+        <v>46245</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>195</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B16" s="34">
-        <v>46232</v>
+        <v>46246</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>220</v>
+        <v>152</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>195</v>
+        <v>233</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B17" s="34"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="19"/>
+      <c r="B17" s="34">
+        <v>46247</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B18" s="34"/>
-      <c r="C18" s="14"/>
+      <c r="B18" s="34">
+        <v>46254</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>165</v>
+      </c>
       <c r="D18" s="19"/>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
@@ -3390,8 +3464,9 @@
     <hyperlink ref="D12" r:id="rId9" xr:uid="{621A8E08-9256-488D-A70A-C5E1B0F691A4}"/>
     <hyperlink ref="D13" r:id="rId10" xr:uid="{AA824B36-87E5-42C8-98E9-2D2001208BCF}"/>
     <hyperlink ref="D14" r:id="rId11" xr:uid="{4470E29F-4FAE-4202-9E25-2704221D7787}"/>
-    <hyperlink ref="D15" r:id="rId12" xr:uid="{91DAAECC-701D-4C77-A047-E0AF9997EE5A}"/>
-    <hyperlink ref="D16" r:id="rId13" xr:uid="{9BE5FAA4-1725-428C-BABE-E69D8B806D1C}"/>
+    <hyperlink ref="D16" r:id="rId12" xr:uid="{E0D720A5-AAC0-4D45-A438-1661E9E19884}"/>
+    <hyperlink ref="D15" r:id="rId13" xr:uid="{364B1836-E2AB-4E20-9CB5-D46DC6CA0FA9}"/>
+    <hyperlink ref="D17" r:id="rId14" xr:uid="{16585DE6-F99F-4F45-AD9B-6D6451BD1173}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3408,18 +3483,18 @@
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="36" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="C2" s="36" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -3445,87 +3520,87 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="9" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>14</v>
+        <v>169</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>2</v>
+        <v>171</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>3</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>16</v>
+        <v>175</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>4</v>
+        <v>176</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>6</v>
+        <v>177</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>22</v>
+        <v>178</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>17</v>
+        <v>179</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>180</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>12</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="127.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>21</v>
+        <v>182</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>18</v>
+        <v>183</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>33</v>
+        <v>184</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="33" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>13</v>
+        <v>185</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>20</v>
+        <v>186</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>9</v>
+        <v>188</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>10</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -3554,7 +3629,7 @@
     <row r="3" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="67" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C4" s="68"/>
       <c r="D4" s="39"/>
@@ -3566,46 +3641,46 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="D6" s="39"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="40" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="D7" s="39"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="40" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D8" s="39"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="40" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D9" s="39"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="40" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D10" s="39"/>
     </row>
@@ -3630,68 +3705,68 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>32</v>
+        <v>200</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>14</v>
+        <v>169</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>24</v>
+        <v>201</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>31</v>
+        <v>202</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>203</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>26</v>
+        <v>204</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>30</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>27</v>
+        <v>206</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>29</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>28</v>
+        <v>207</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>23</v>
+        <v>174</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>30</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update TROMBONE 3.0.5 solution access info with laptop no. 11 (edu12)
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="760" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8084B9A5-E89D-4C59-8459-38273DDA84A6}"/>
+  <xr:revisionPtr revIDLastSave="770" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7045661A-57DC-43C1-B34A-74CC45BB0F57}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="239">
   <si>
     <t>교육장 WiFi 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -891,6 +891,18 @@
   </si>
   <si>
     <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgAeSH61MkiqTKogyAAEH0v1AQNWhsstioRHFrdxMBQ7FN8?e=7qWeI5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>edu12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노트북 11번</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TROMBONE 3.0.5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1404,22 +1416,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1707,6 +1719,33 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="328" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{CBEEE931-E0EC-4364-9B62-A91EDBA26D46}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;704e68df-454b-4727-93fb-2ed39c65f047&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD9A2511-751C-4257-ACD2-7080A9799B54}">
   <dimension ref="B4:C12"/>
@@ -2502,7 +2541,7 @@
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" s="55" t="s">
-        <v>67</v>
+        <v>238</v>
       </c>
       <c r="C23" s="30" t="s">
         <v>41</v>
@@ -2606,22 +2645,26 @@
       <c r="F31" s="59"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="57"/>
+      <c r="B32" s="56"/>
       <c r="C32" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E32" s="51"/>
-      <c r="F32" s="60"/>
+      <c r="E32" s="50"/>
+      <c r="F32" s="59"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="23"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="E33" s="51"/>
+      <c r="F33" s="60"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
@@ -2635,12 +2678,12 @@
     <mergeCell ref="B3:B12"/>
     <mergeCell ref="F3:F12"/>
     <mergeCell ref="E3:E12"/>
-    <mergeCell ref="B23:B32"/>
-    <mergeCell ref="F23:F32"/>
-    <mergeCell ref="E23:E32"/>
     <mergeCell ref="B13:B22"/>
     <mergeCell ref="F13:F22"/>
     <mergeCell ref="E13:E22"/>
+    <mergeCell ref="E23:E33"/>
+    <mergeCell ref="F23:F33"/>
+    <mergeCell ref="B23:B33"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2682,25 +2725,25 @@
       <c r="F4" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="65" t="s">
+      <c r="G4" s="63" t="s">
         <v>85</v>
       </c>
-      <c r="H4" s="66"/>
+      <c r="H4" s="64"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="61" t="s">
+      <c r="B5" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="C5" s="65" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="D5" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="E5" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="61" t="s">
+      <c r="F5" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2711,11 +2754,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="25" t="s">
         <v>93</v>
       </c>
@@ -2724,19 +2767,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="63" t="s">
+      <c r="B7" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="63" t="s">
+      <c r="C7" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="D7" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="63" t="s">
+      <c r="E7" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="63" t="s">
+      <c r="F7" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2747,11 +2790,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="64"/>
-      <c r="C8" s="64"/>
-      <c r="D8" s="64"/>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
       <c r="G8" s="26" t="s">
         <v>93</v>
       </c>
@@ -2760,19 +2803,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="61" t="s">
+      <c r="B9" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="65" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="65" t="s">
         <v>102</v>
       </c>
-      <c r="E9" s="61" t="s">
+      <c r="E9" s="65" t="s">
         <v>103</v>
       </c>
-      <c r="F9" s="61" t="s">
+      <c r="F9" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2783,11 +2826,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
+      <c r="B10" s="66"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
       <c r="G10" s="25" t="s">
         <v>93</v>
       </c>
@@ -2796,19 +2839,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="63" t="s">
+      <c r="B11" s="61" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="63" t="s">
+      <c r="C11" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="63" t="s">
+      <c r="D11" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="E11" s="63" t="s">
+      <c r="E11" s="61" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="63" t="s">
+      <c r="F11" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2819,11 +2862,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="64"/>
-      <c r="C12" s="64"/>
-      <c r="D12" s="64"/>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
       <c r="G12" s="26" t="s">
         <v>93</v>
       </c>
@@ -2832,19 +2875,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="61" t="s">
+      <c r="B13" s="65" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="65" t="s">
         <v>112</v>
       </c>
-      <c r="E13" s="61" t="s">
+      <c r="E13" s="65" t="s">
         <v>113</v>
       </c>
-      <c r="F13" s="61" t="s">
+      <c r="F13" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2855,11 +2898,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="62"/>
-      <c r="C14" s="62"/>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
+      <c r="B14" s="66"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="66"/>
       <c r="G14" s="25" t="s">
         <v>93</v>
       </c>
@@ -2868,19 +2911,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="65" t="s">
         <v>117</v>
       </c>
-      <c r="E15" s="61" t="s">
+      <c r="E15" s="65" t="s">
         <v>118</v>
       </c>
-      <c r="F15" s="61" t="s">
+      <c r="F15" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2891,11 +2934,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
+      <c r="B16" s="66"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="25" t="s">
         <v>93</v>
       </c>
@@ -2904,19 +2947,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="65" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="65" t="s">
         <v>122</v>
       </c>
-      <c r="E17" s="61" t="s">
+      <c r="E17" s="65" t="s">
         <v>123</v>
       </c>
-      <c r="F17" s="61" t="s">
+      <c r="F17" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2927,11 +2970,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
+      <c r="B18" s="66"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
       <c r="G18" s="25" t="s">
         <v>93</v>
       </c>
@@ -2940,19 +2983,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="63" t="s">
+      <c r="B19" s="61" t="s">
         <v>126</v>
       </c>
-      <c r="C19" s="63" t="s">
+      <c r="C19" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="63" t="s">
+      <c r="D19" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="E19" s="63" t="s">
+      <c r="E19" s="61" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="63" t="s">
+      <c r="F19" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -2963,11 +3006,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="64"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="26" t="s">
         <v>93</v>
       </c>
@@ -2976,19 +3019,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="61" t="s">
+      <c r="D21" s="65" t="s">
         <v>132</v>
       </c>
-      <c r="E21" s="61" t="s">
+      <c r="E21" s="65" t="s">
         <v>133</v>
       </c>
-      <c r="F21" s="61" t="s">
+      <c r="F21" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -2999,11 +3042,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="62"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="62"/>
-      <c r="E22" s="62"/>
-      <c r="F22" s="62"/>
+      <c r="B22" s="66"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
       <c r="G22" s="25" t="s">
         <v>93</v>
       </c>
@@ -3012,19 +3055,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="63" t="s">
+      <c r="B23" s="61" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="63" t="s">
+      <c r="C23" s="61" t="s">
         <v>137</v>
       </c>
-      <c r="D23" s="63" t="s">
+      <c r="D23" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="E23" s="63" t="s">
+      <c r="E23" s="61" t="s">
         <v>139</v>
       </c>
-      <c r="F23" s="63" t="s">
+      <c r="F23" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -3035,11 +3078,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="64"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="26" t="s">
         <v>93</v>
       </c>
@@ -3048,19 +3091,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="65" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="65" t="s">
         <v>143</v>
       </c>
-      <c r="D25" s="61" t="s">
+      <c r="D25" s="65" t="s">
         <v>144</v>
       </c>
-      <c r="E25" s="61" t="s">
+      <c r="E25" s="65" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="61" t="s">
+      <c r="F25" s="65" t="s">
         <v>90</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -3071,11 +3114,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
+      <c r="B26" s="66"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
       <c r="G26" s="25" t="s">
         <v>93</v>
       </c>
@@ -3085,40 +3128,16 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -3131,16 +3150,40 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Support laptop no. 11 in VPN and solution access dropdowns
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="770" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7045661A-57DC-43C1-B34A-74CC45BB0F57}"/>
+  <xr:revisionPtr revIDLastSave="778" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{081E9DB3-1133-495C-94FA-5CA5FFE6E50A}"/>
   <bookViews>
-    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="241">
   <si>
     <t>교육장 WiFi 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -903,6 +903,14 @@
   </si>
   <si>
     <t>TROMBONE 3.0.5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>hy.shin</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>nmJjGQLL</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1002,7 +1010,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Freesentation 4 Regular"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="6"/>
@@ -1356,6 +1363,51 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1371,50 +1423,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1426,12 +1439,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1756,10 +1763,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="41"/>
+      <c r="C4" s="56"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1778,10 +1785,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="42"/>
+      <c r="C8" s="57"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -2124,7 +2131,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C90A17B8-D559-4179-9BBE-8680B873B9EB}">
-  <dimension ref="B2:D14"/>
+  <dimension ref="B2:D15"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.125" customWidth="1"/>
@@ -2133,18 +2140,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -2265,6 +2272,17 @@
       </c>
       <c r="D14" s="18" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B15" s="14">
+        <v>11</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -2305,7 +2323,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="41" t="s">
         <v>40</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -2314,117 +2332,117 @@
       <c r="D3" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="52" t="s">
+      <c r="E3" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="F3" s="49" t="s">
+      <c r="F3" s="44" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="47"/>
+      <c r="B4" s="42"/>
       <c r="C4" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="F4" s="50"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="45"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="47"/>
+      <c r="B5" s="42"/>
       <c r="C5" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="53"/>
-      <c r="F5" s="50"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="45"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="47"/>
+      <c r="B6" s="42"/>
       <c r="C6" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="53"/>
-      <c r="F6" s="50"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="45"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="47"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="53"/>
-      <c r="F7" s="50"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="45"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="47"/>
+      <c r="B8" s="42"/>
       <c r="C8" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="53"/>
-      <c r="F8" s="50"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="45"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="47"/>
+      <c r="B9" s="42"/>
       <c r="C9" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="53"/>
-      <c r="F9" s="50"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="45"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="47"/>
+      <c r="B10" s="42"/>
       <c r="C10" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="53"/>
-      <c r="F10" s="50"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="45"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="47"/>
+      <c r="B11" s="42"/>
       <c r="C11" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="53"/>
-      <c r="F11" s="50"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="45"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="48"/>
+      <c r="B12" s="43"/>
       <c r="C12" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="54"/>
-      <c r="F12" s="51"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="46"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="55" t="s">
+      <c r="B13" s="50" t="s">
         <v>64</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -2433,114 +2451,114 @@
       <c r="D13" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="49" t="s">
+      <c r="E13" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="58" t="s">
+      <c r="F13" s="53" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="56"/>
+      <c r="B14" s="51"/>
       <c r="C14" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="50"/>
-      <c r="F14" s="59"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="54"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="56"/>
+      <c r="B15" s="51"/>
       <c r="C15" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="50"/>
-      <c r="F15" s="59"/>
+      <c r="E15" s="45"/>
+      <c r="F15" s="54"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="56"/>
+      <c r="B16" s="51"/>
       <c r="C16" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="50"/>
-      <c r="F16" s="59"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="54"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="56"/>
+      <c r="B17" s="51"/>
       <c r="C17" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="50"/>
-      <c r="F17" s="59"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="54"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="56"/>
+      <c r="B18" s="51"/>
       <c r="C18" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="50"/>
-      <c r="F18" s="59"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="54"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="56"/>
+      <c r="B19" s="51"/>
       <c r="C19" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="50"/>
-      <c r="F19" s="59"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="54"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="56"/>
+      <c r="B20" s="51"/>
       <c r="C20" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="50"/>
-      <c r="F20" s="59"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="54"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="56"/>
+      <c r="B21" s="51"/>
       <c r="C21" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="50"/>
-      <c r="F21" s="59"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="54"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="57"/>
+      <c r="B22" s="52"/>
       <c r="C22" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E22" s="51"/>
-      <c r="F22" s="60"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="55"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="55" t="s">
+      <c r="B23" s="50" t="s">
         <v>238</v>
       </c>
       <c r="C23" s="30" t="s">
@@ -2549,122 +2567,122 @@
       <c r="D23" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="49" t="s">
+      <c r="E23" s="44" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="58" t="s">
+      <c r="F23" s="53" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="56"/>
+      <c r="B24" s="51"/>
       <c r="C24" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="59"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="54"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="56"/>
+      <c r="B25" s="51"/>
       <c r="C25" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="50"/>
-      <c r="F25" s="59"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="54"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="56"/>
+      <c r="B26" s="51"/>
       <c r="C26" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="50"/>
-      <c r="F26" s="59"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="54"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="56"/>
+      <c r="B27" s="51"/>
       <c r="C27" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E27" s="50"/>
-      <c r="F27" s="59"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="54"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="56"/>
+      <c r="B28" s="51"/>
       <c r="C28" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E28" s="50"/>
-      <c r="F28" s="59"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="54"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="56"/>
+      <c r="B29" s="51"/>
       <c r="C29" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E29" s="50"/>
-      <c r="F29" s="59"/>
+      <c r="E29" s="45"/>
+      <c r="F29" s="54"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="56"/>
+      <c r="B30" s="51"/>
       <c r="C30" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="50"/>
-      <c r="F30" s="59"/>
+      <c r="E30" s="45"/>
+      <c r="F30" s="54"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="56"/>
+      <c r="B31" s="51"/>
       <c r="C31" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E31" s="50"/>
-      <c r="F31" s="59"/>
+      <c r="E31" s="45"/>
+      <c r="F31" s="54"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="56"/>
+      <c r="B32" s="51"/>
       <c r="C32" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E32" s="50"/>
-      <c r="F32" s="59"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="54"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="57"/>
+      <c r="B33" s="52"/>
       <c r="C33" s="30" t="s">
         <v>237</v>
       </c>
       <c r="D33" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="E33" s="51"/>
-      <c r="F33" s="60"/>
+      <c r="E33" s="46"/>
+      <c r="F33" s="55"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
@@ -2675,15 +2693,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="E23:E33"/>
+    <mergeCell ref="F23:F33"/>
+    <mergeCell ref="B23:B33"/>
     <mergeCell ref="B3:B12"/>
     <mergeCell ref="F3:F12"/>
     <mergeCell ref="E3:E12"/>
     <mergeCell ref="B13:B22"/>
     <mergeCell ref="F13:F22"/>
     <mergeCell ref="E13:E22"/>
-    <mergeCell ref="E23:E33"/>
-    <mergeCell ref="F23:F33"/>
-    <mergeCell ref="B23:B33"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2725,25 +2743,25 @@
       <c r="F4" s="37" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="63" t="s">
+      <c r="G4" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="H4" s="64"/>
+      <c r="H4" s="66"/>
     </row>
     <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="65" t="s">
+      <c r="B5" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="C5" s="61" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="65" t="s">
+      <c r="D5" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="65" t="s">
+      <c r="E5" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="65" t="s">
+      <c r="F5" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G5" s="25" t="s">
@@ -2754,11 +2772,11 @@
       </c>
     </row>
     <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
       <c r="G6" s="25" t="s">
         <v>93</v>
       </c>
@@ -2767,19 +2785,19 @@
       </c>
     </row>
     <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="63" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="63" t="s">
         <v>90</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2790,11 +2808,11 @@
       </c>
     </row>
     <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
+      <c r="B8" s="64"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="64"/>
+      <c r="F8" s="64"/>
       <c r="G8" s="26" t="s">
         <v>93</v>
       </c>
@@ -2803,19 +2821,19 @@
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="65" t="s">
+      <c r="B9" s="61" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="65" t="s">
+      <c r="C9" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="65" t="s">
+      <c r="D9" s="61" t="s">
         <v>102</v>
       </c>
-      <c r="E9" s="65" t="s">
+      <c r="E9" s="61" t="s">
         <v>103</v>
       </c>
-      <c r="F9" s="65" t="s">
+      <c r="F9" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G9" s="25" t="s">
@@ -2826,11 +2844,11 @@
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="66"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="62"/>
       <c r="G10" s="25" t="s">
         <v>93</v>
       </c>
@@ -2839,19 +2857,19 @@
       </c>
     </row>
     <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="61" t="s">
+      <c r="D11" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="E11" s="61" t="s">
+      <c r="E11" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="61" t="s">
+      <c r="F11" s="63" t="s">
         <v>90</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -2862,11 +2880,11 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
+      <c r="B12" s="64"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="64"/>
+      <c r="F12" s="64"/>
       <c r="G12" s="26" t="s">
         <v>93</v>
       </c>
@@ -2875,19 +2893,19 @@
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="65" t="s">
+      <c r="B13" s="61" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="65" t="s">
+      <c r="C13" s="61" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="65" t="s">
+      <c r="D13" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="E13" s="65" t="s">
+      <c r="E13" s="61" t="s">
         <v>113</v>
       </c>
-      <c r="F13" s="65" t="s">
+      <c r="F13" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G13" s="25" t="s">
@@ -2898,11 +2916,11 @@
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="66"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="62"/>
+      <c r="D14" s="62"/>
+      <c r="E14" s="62"/>
+      <c r="F14" s="62"/>
       <c r="G14" s="25" t="s">
         <v>93</v>
       </c>
@@ -2911,19 +2929,19 @@
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="65" t="s">
+      <c r="B15" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="C15" s="65" t="s">
+      <c r="C15" s="61" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="65" t="s">
+      <c r="D15" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="E15" s="65" t="s">
+      <c r="E15" s="61" t="s">
         <v>118</v>
       </c>
-      <c r="F15" s="65" t="s">
+      <c r="F15" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G15" s="25" t="s">
@@ -2934,11 +2952,11 @@
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="66"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
+      <c r="E16" s="62"/>
+      <c r="F16" s="62"/>
       <c r="G16" s="25" t="s">
         <v>93</v>
       </c>
@@ -2947,19 +2965,19 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="65" t="s">
+      <c r="B17" s="61" t="s">
         <v>121</v>
       </c>
-      <c r="C17" s="65" t="s">
+      <c r="C17" s="61" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="65" t="s">
+      <c r="D17" s="61" t="s">
         <v>122</v>
       </c>
-      <c r="E17" s="65" t="s">
+      <c r="E17" s="61" t="s">
         <v>123</v>
       </c>
-      <c r="F17" s="65" t="s">
+      <c r="F17" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G17" s="25" t="s">
@@ -2970,11 +2988,11 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="66"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
       <c r="G18" s="25" t="s">
         <v>93</v>
       </c>
@@ -2983,19 +3001,19 @@
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="63" t="s">
         <v>126</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="63" t="s">
         <v>127</v>
       </c>
-      <c r="E19" s="61" t="s">
+      <c r="E19" s="63" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="61" t="s">
+      <c r="F19" s="63" t="s">
         <v>90</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -3006,11 +3024,11 @@
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
+      <c r="B20" s="64"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="64"/>
+      <c r="E20" s="64"/>
+      <c r="F20" s="64"/>
       <c r="G20" s="26" t="s">
         <v>93</v>
       </c>
@@ -3019,19 +3037,19 @@
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="65" t="s">
+      <c r="B21" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="65" t="s">
+      <c r="C21" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="65" t="s">
+      <c r="D21" s="61" t="s">
         <v>132</v>
       </c>
-      <c r="E21" s="65" t="s">
+      <c r="E21" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="F21" s="65" t="s">
+      <c r="F21" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G21" s="25" t="s">
@@ -3042,11 +3060,11 @@
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="66"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
+      <c r="B22" s="62"/>
+      <c r="C22" s="62"/>
+      <c r="D22" s="62"/>
+      <c r="E22" s="62"/>
+      <c r="F22" s="62"/>
       <c r="G22" s="25" t="s">
         <v>93</v>
       </c>
@@ -3055,19 +3073,19 @@
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="63" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="63" t="s">
         <v>137</v>
       </c>
-      <c r="D23" s="61" t="s">
+      <c r="D23" s="63" t="s">
         <v>138</v>
       </c>
-      <c r="E23" s="61" t="s">
+      <c r="E23" s="63" t="s">
         <v>139</v>
       </c>
-      <c r="F23" s="61" t="s">
+      <c r="F23" s="63" t="s">
         <v>90</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -3078,11 +3096,11 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="64"/>
+      <c r="E24" s="64"/>
+      <c r="F24" s="64"/>
       <c r="G24" s="26" t="s">
         <v>93</v>
       </c>
@@ -3091,19 +3109,19 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="65" t="s">
+      <c r="B25" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="65" t="s">
+      <c r="C25" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="D25" s="65" t="s">
+      <c r="D25" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="E25" s="65" t="s">
+      <c r="E25" s="61" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="65" t="s">
+      <c r="F25" s="61" t="s">
         <v>90</v>
       </c>
       <c r="G25" s="25" t="s">
@@ -3114,11 +3132,11 @@
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="66"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
+      <c r="D26" s="62"/>
+      <c r="E26" s="62"/>
+      <c r="F26" s="62"/>
       <c r="G26" s="25" t="s">
         <v>93</v>
       </c>
@@ -3128,16 +3146,40 @@
     </row>
   </sheetData>
   <mergeCells count="56">
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -3150,40 +3192,16 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
Sync updated TROMBONE service access info and Excel changes
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="778" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{081E9DB3-1133-495C-94FA-5CA5FFE6E50A}"/>
+  <xr:revisionPtr revIDLastSave="796" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B46B07AA-B222-4582-99F2-803E86EE16C7}"/>
   <bookViews>
-    <workbookView xWindow="-24240" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="234">
   <si>
     <t>교육장 WiFi 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -324,9 +324,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>VPN ID</t>
-  </si>
-  <si>
     <t>user ID</t>
   </si>
   <si>
@@ -374,9 +371,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-1</t>
-  </si>
-  <si>
     <t>user1</t>
   </si>
   <si>
@@ -394,9 +388,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-2</t>
-  </si>
-  <si>
     <t>USER02</t>
   </si>
   <si>
@@ -411,9 +402,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-3</t>
-  </si>
-  <si>
     <t>USER03</t>
   </si>
   <si>
@@ -428,9 +416,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-4</t>
-  </si>
-  <si>
     <t>USER04</t>
   </si>
   <si>
@@ -446,9 +431,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-5</t>
-  </si>
-  <si>
     <t>USER05</t>
   </si>
   <si>
@@ -463,9 +445,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-6</t>
-  </si>
-  <si>
     <t>USER06</t>
   </si>
   <si>
@@ -480,9 +459,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-7</t>
-  </si>
-  <si>
     <t>USER07</t>
   </si>
   <si>
@@ -497,9 +473,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-8</t>
-  </si>
-  <si>
     <t>USER08</t>
   </si>
   <si>
@@ -514,16 +487,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>handson-9</t>
-  </si>
-  <si>
     <t>user10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>USER09</t>
-  </si>
-  <si>
     <t>EDU10</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -534,9 +501,6 @@
   <si>
     <t>http://10.255.62.49:31319/members</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>handson-10</t>
   </si>
   <si>
     <t>user11</t>
@@ -911,6 +875,25 @@
   </si>
   <si>
     <t>nmJjGQLL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>노트북 11번</t>
+  </si>
+  <si>
+    <t>user12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER12</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EDU12</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1010,6 +993,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Freesentation 4 Regular"/>
+      <charset val="129"/>
     </font>
     <font>
       <sz val="6"/>
@@ -1028,7 +1012,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1080,6 +1064,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1253,7 +1243,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1363,6 +1353,48 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1372,15 +1404,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1390,38 +1413,17 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -1429,23 +1431,20 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1763,10 +1762,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="56" t="s">
+      <c r="B4" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="56"/>
+      <c r="C4" s="44"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1785,10 +1784,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="45" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="57"/>
+      <c r="C8" s="45"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -1835,18 +1834,18 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="C3" s="14">
         <v>31300</v>
@@ -1857,7 +1856,7 @@
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="C4" s="14">
         <v>31301</v>
@@ -1868,7 +1867,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
       <c r="C5" s="14">
         <v>31302</v>
@@ -1879,7 +1878,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C6" s="14">
         <v>31303</v>
@@ -1890,7 +1889,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="C7" s="14">
         <v>31304</v>
@@ -1901,7 +1900,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="C8" s="21">
         <v>31305</v>
@@ -1912,7 +1911,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="C9" s="21">
         <v>31306</v>
@@ -1923,7 +1922,7 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="C10" s="21">
         <v>31307</v>
@@ -1934,7 +1933,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="C11" s="21">
         <v>31308</v>
@@ -1945,7 +1944,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="C12" s="21">
         <v>31309</v>
@@ -1967,7 +1966,7 @@
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="C14" s="21">
         <v>31322</v>
@@ -1995,7 +1994,7 @@
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="31" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>1</v>
@@ -2009,47 +2008,47 @@
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="19"/>
       <c r="E5" s="20" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="E7" s="19"/>
     </row>
@@ -2109,12 +2108,12 @@
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
     </row>
     <row r="26" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2140,18 +2139,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -2279,10 +2278,10 @@
         <v>11</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -2323,7 +2322,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="55" t="s">
         <v>40</v>
       </c>
       <c r="C3" s="30" t="s">
@@ -2332,117 +2331,117 @@
       <c r="D3" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="47" t="s">
+      <c r="E3" s="58" t="s">
         <v>43</v>
       </c>
-      <c r="F3" s="44" t="s">
+      <c r="F3" s="46" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="42"/>
+      <c r="B4" s="56"/>
       <c r="C4" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D4" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="F4" s="45"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="47"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="42"/>
+      <c r="B5" s="56"/>
       <c r="C5" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="45"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="47"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="42"/>
+      <c r="B6" s="56"/>
       <c r="C6" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="48"/>
-      <c r="F6" s="45"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="47"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="42"/>
+      <c r="B7" s="56"/>
       <c r="C7" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="45"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="47"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="42"/>
+      <c r="B8" s="56"/>
       <c r="C8" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="E8" s="48"/>
-      <c r="F8" s="45"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="47"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="42"/>
+      <c r="B9" s="56"/>
       <c r="C9" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="45"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="47"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="42"/>
+      <c r="B10" s="56"/>
       <c r="C10" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="45"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="47"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="42"/>
+      <c r="B11" s="56"/>
       <c r="C11" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D11" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="48"/>
-      <c r="F11" s="45"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="47"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="43"/>
+      <c r="B12" s="57"/>
       <c r="C12" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="49"/>
-      <c r="F12" s="46"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="48"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="50" t="s">
+      <c r="B13" s="52" t="s">
         <v>64</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -2451,115 +2450,115 @@
       <c r="D13" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="44" t="s">
+      <c r="E13" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="53" t="s">
+      <c r="F13" s="49" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="51"/>
+      <c r="B14" s="53"/>
       <c r="C14" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D14" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="E14" s="45"/>
-      <c r="F14" s="54"/>
+      <c r="E14" s="47"/>
+      <c r="F14" s="50"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="51"/>
+      <c r="B15" s="53"/>
       <c r="C15" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D15" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="45"/>
-      <c r="F15" s="54"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="50"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="51"/>
+      <c r="B16" s="53"/>
       <c r="C16" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D16" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E16" s="45"/>
-      <c r="F16" s="54"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="50"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="51"/>
+      <c r="B17" s="53"/>
       <c r="C17" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D17" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="45"/>
-      <c r="F17" s="54"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="50"/>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="51"/>
+      <c r="B18" s="53"/>
       <c r="C18" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D18" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="45"/>
-      <c r="F18" s="54"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="50"/>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="51"/>
+      <c r="B19" s="53"/>
       <c r="C19" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D19" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E19" s="45"/>
-      <c r="F19" s="54"/>
+      <c r="E19" s="47"/>
+      <c r="F19" s="50"/>
     </row>
     <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="51"/>
+      <c r="B20" s="53"/>
       <c r="C20" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D20" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="45"/>
-      <c r="F20" s="54"/>
+      <c r="E20" s="47"/>
+      <c r="F20" s="50"/>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="51"/>
+      <c r="B21" s="53"/>
       <c r="C21" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="54"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="50"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="52"/>
+      <c r="B22" s="54"/>
       <c r="C22" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D22" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E22" s="46"/>
-      <c r="F22" s="55"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="51"/>
     </row>
     <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="50" t="s">
-        <v>238</v>
+      <c r="B23" s="52" t="s">
+        <v>226</v>
       </c>
       <c r="C23" s="30" t="s">
         <v>41</v>
@@ -2567,122 +2566,122 @@
       <c r="D23" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="53" t="s">
+      <c r="F23" s="49" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="51"/>
+      <c r="B24" s="53"/>
       <c r="C24" s="30" t="s">
         <v>45</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="E24" s="45"/>
-      <c r="F24" s="54"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="50"/>
     </row>
     <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="51"/>
+      <c r="B25" s="53"/>
       <c r="C25" s="30" t="s">
         <v>47</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="E25" s="45"/>
-      <c r="F25" s="54"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="50"/>
     </row>
     <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="51"/>
+      <c r="B26" s="53"/>
       <c r="C26" s="30" t="s">
         <v>50</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="E26" s="45"/>
-      <c r="F26" s="54"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="50"/>
     </row>
     <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="51"/>
+      <c r="B27" s="53"/>
       <c r="C27" s="30" t="s">
         <v>52</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E27" s="45"/>
-      <c r="F27" s="54"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="50"/>
     </row>
     <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="51"/>
+      <c r="B28" s="53"/>
       <c r="C28" s="30" t="s">
         <v>54</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="E28" s="45"/>
-      <c r="F28" s="54"/>
+      <c r="E28" s="47"/>
+      <c r="F28" s="50"/>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="51"/>
+      <c r="B29" s="53"/>
       <c r="C29" s="30" t="s">
         <v>56</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E29" s="45"/>
-      <c r="F29" s="54"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="50"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="51"/>
+      <c r="B30" s="53"/>
       <c r="C30" s="30" t="s">
         <v>58</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="E30" s="45"/>
-      <c r="F30" s="54"/>
+      <c r="E30" s="47"/>
+      <c r="F30" s="50"/>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="51"/>
+      <c r="B31" s="53"/>
       <c r="C31" s="30" t="s">
         <v>60</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E31" s="45"/>
-      <c r="F31" s="54"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="50"/>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="51"/>
+      <c r="B32" s="53"/>
       <c r="C32" s="30" t="s">
         <v>62</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E32" s="45"/>
-      <c r="F32" s="54"/>
+      <c r="E32" s="47"/>
+      <c r="F32" s="50"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="52"/>
+      <c r="B33" s="54"/>
       <c r="C33" s="30" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="E33" s="46"/>
-      <c r="F33" s="55"/>
+        <v>224</v>
+      </c>
+      <c r="E33" s="48"/>
+      <c r="F33" s="51"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
@@ -2716,9 +2715,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06BC2E8E-44C3-4E0F-92D7-F1091F54A312}">
-  <dimension ref="B3:H26"/>
+  <dimension ref="B3:H28"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="14.25" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="6" width="14.375" customWidth="1"/>
@@ -2729,457 +2729,468 @@
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="D4" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="E4" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="F4" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="G4" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="65" t="s">
+      <c r="H4" s="64"/>
+    </row>
+    <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="H4" s="66"/>
-    </row>
-    <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="61" t="s">
+      <c r="C5" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="61" t="s">
+      <c r="D5" s="65" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="61" t="s">
+      <c r="E5" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="E5" s="61" t="s">
+      <c r="F5" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="F5" s="61" t="s">
+      <c r="G5" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G5" s="25" t="s">
+      <c r="H5" t="s">
         <v>91</v>
       </c>
-      <c r="H5" t="s">
+    </row>
+    <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
+      <c r="G6" s="25" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="62"/>
-      <c r="E6" s="62"/>
-      <c r="F6" s="62"/>
-      <c r="G6" s="25" t="s">
+      <c r="H6" s="27" t="s">
         <v>93</v>
       </c>
-      <c r="H6" s="27" t="s">
+    </row>
+    <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="61" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="63" t="s">
+      <c r="D7" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="C7" s="63" t="s">
+      <c r="E7" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="D7" s="63" t="s">
+      <c r="F7" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="G7" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="E7" s="63" t="s">
+    </row>
+    <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="62"/>
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8" s="27" t="s">
         <v>98</v>
-      </c>
-      <c r="F7" s="63" t="s">
-        <v>90</v>
-      </c>
-      <c r="G7" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H7" s="27" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="64"/>
-      <c r="C8" s="64"/>
-      <c r="D8" s="64"/>
-      <c r="E8" s="64"/>
-      <c r="F8" s="64"/>
-      <c r="G8" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="61" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="65" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="65" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="65" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="27" t="s">
         <v>101</v>
-      </c>
-      <c r="C9" s="61" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="61" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" s="61" t="s">
-        <v>103</v>
-      </c>
-      <c r="F9" s="61" t="s">
-        <v>90</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="62"/>
-      <c r="C10" s="62"/>
-      <c r="D10" s="62"/>
-      <c r="E10" s="62"/>
-      <c r="F10" s="62"/>
+      <c r="C10" s="66"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
       <c r="G10" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H10" s="27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="61" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="61" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="61" t="s">
+        <v>103</v>
+      </c>
+      <c r="E11" s="61" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="27" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="63" t="s">
+    <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="27" t="s">
         <v>106</v>
-      </c>
-      <c r="C11" s="63" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="63" t="s">
-        <v>107</v>
-      </c>
-      <c r="E11" s="63" t="s">
-        <v>108</v>
-      </c>
-      <c r="F11" s="63" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="64"/>
-      <c r="C12" s="64"/>
-      <c r="D12" s="64"/>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64"/>
-      <c r="G12" s="26" t="s">
-        <v>93</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="61" t="s">
-        <v>111</v>
-      </c>
-      <c r="C13" s="61" t="s">
+        <v>50</v>
+      </c>
+      <c r="C13" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="61" t="s">
-        <v>112</v>
-      </c>
-      <c r="E13" s="61" t="s">
-        <v>113</v>
-      </c>
-      <c r="F13" s="61" t="s">
+      <c r="D13" s="65" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="F13" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G13" s="25" t="s">
-        <v>91</v>
-      </c>
       <c r="H13" s="27" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="62"/>
-      <c r="C14" s="62"/>
-      <c r="D14" s="62"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="62"/>
+      <c r="C14" s="66"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="66"/>
       <c r="G14" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H14" s="27" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="61" t="s">
-        <v>116</v>
-      </c>
-      <c r="C15" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="61" t="s">
-        <v>117</v>
-      </c>
-      <c r="E15" s="61" t="s">
-        <v>118</v>
-      </c>
-      <c r="F15" s="61" t="s">
+      <c r="D15" s="65" t="s">
+        <v>111</v>
+      </c>
+      <c r="E15" s="65" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="25" t="s">
-        <v>91</v>
-      </c>
       <c r="H15" s="27" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="62"/>
+      <c r="C16" s="66"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="66"/>
       <c r="G16" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H16" s="27" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="61" t="s">
-        <v>121</v>
-      </c>
-      <c r="C17" s="61" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="61" t="s">
-        <v>122</v>
-      </c>
-      <c r="E17" s="61" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" s="61" t="s">
+      <c r="D17" s="65" t="s">
+        <v>115</v>
+      </c>
+      <c r="E17" s="65" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G17" s="25" t="s">
-        <v>91</v>
-      </c>
       <c r="H17" s="27" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
       <c r="G18" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H18" s="27" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="63" t="s">
-        <v>126</v>
-      </c>
-      <c r="C19" s="63" t="s">
+      <c r="B19" s="61" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="61" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="63" t="s">
-        <v>127</v>
-      </c>
-      <c r="E19" s="63" t="s">
-        <v>128</v>
-      </c>
-      <c r="F19" s="63" t="s">
+      <c r="D19" s="61" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" s="61" t="s">
+        <v>120</v>
+      </c>
+      <c r="F19" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="G19" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="G19" s="26" t="s">
-        <v>91</v>
-      </c>
       <c r="H19" s="27" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="64"/>
-      <c r="C20" s="64"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="62"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
       <c r="G20" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H20" s="27" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="61" t="s">
-        <v>131</v>
-      </c>
-      <c r="C21" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="65" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="61" t="s">
-        <v>132</v>
-      </c>
-      <c r="E21" s="61" t="s">
-        <v>133</v>
-      </c>
-      <c r="F21" s="61" t="s">
+      <c r="D21" s="65" t="s">
+        <v>123</v>
+      </c>
+      <c r="E21" s="65" t="s">
+        <v>124</v>
+      </c>
+      <c r="F21" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G21" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="25" t="s">
-        <v>91</v>
-      </c>
       <c r="H21" s="27" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="62"/>
-      <c r="C22" s="62"/>
-      <c r="D22" s="62"/>
-      <c r="E22" s="62"/>
-      <c r="F22" s="62"/>
+      <c r="C22" s="66"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="66"/>
       <c r="G22" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H22" s="27" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="63" t="s">
-        <v>136</v>
-      </c>
-      <c r="C23" s="63" t="s">
-        <v>137</v>
-      </c>
-      <c r="D23" s="63" t="s">
-        <v>138</v>
-      </c>
-      <c r="E23" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="F23" s="63" t="s">
+      <c r="B23" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="61" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="E23" s="61" t="s">
+        <v>128</v>
+      </c>
+      <c r="F23" s="61" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="G23" s="26" t="s">
-        <v>91</v>
-      </c>
       <c r="H23" s="27" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="64"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="64"/>
-      <c r="F24" s="64"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="62"/>
+      <c r="D24" s="62"/>
+      <c r="E24" s="62"/>
+      <c r="F24" s="62"/>
       <c r="G24" s="26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H24" s="27" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
     </row>
     <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="61" t="s">
-        <v>142</v>
-      </c>
-      <c r="C25" s="61" t="s">
-        <v>143</v>
-      </c>
-      <c r="D25" s="61" t="s">
-        <v>144</v>
-      </c>
-      <c r="E25" s="61" t="s">
-        <v>145</v>
-      </c>
-      <c r="F25" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="65" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="65" t="s">
+        <v>231</v>
+      </c>
+      <c r="E25" s="65" t="s">
+        <v>133</v>
+      </c>
+      <c r="F25" s="65" t="s">
+        <v>89</v>
+      </c>
+      <c r="G25" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="G25" s="25" t="s">
-        <v>91</v>
-      </c>
       <c r="H25" s="27" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="62"/>
-      <c r="C26" s="62"/>
-      <c r="D26" s="62"/>
-      <c r="E26" s="62"/>
-      <c r="F26" s="62"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="66"/>
       <c r="G26" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H26" s="27" t="s">
-        <v>147</v>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B27" s="61" t="s">
+        <v>229</v>
+      </c>
+      <c r="C27" s="69" t="s">
+        <v>230</v>
+      </c>
+      <c r="D27" s="69" t="s">
+        <v>232</v>
+      </c>
+      <c r="E27" s="69" t="s">
+        <v>233</v>
+      </c>
+      <c r="F27" s="69" t="s">
+        <v>89</v>
+      </c>
+      <c r="G27" s="70" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="62"/>
+      <c r="C28" s="71"/>
+      <c r="D28" s="71"/>
+      <c r="E28" s="71"/>
+      <c r="F28" s="71"/>
+      <c r="G28" s="70" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="56">
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
+  <mergeCells count="61">
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -3192,16 +3203,40 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -3244,10 +3279,10 @@
   <sheetData>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="33" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>6</v>
@@ -3258,10 +3293,10 @@
         <v>46217</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -3269,10 +3304,10 @@
         <v>46218</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -3280,10 +3315,10 @@
         <v>46224</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -3291,10 +3326,10 @@
         <v>46225</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -3302,10 +3337,10 @@
         <v>46230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -3313,10 +3348,10 @@
         <v>46231</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -3324,10 +3359,10 @@
         <v>46232</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -3335,10 +3370,10 @@
         <v>46232</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
@@ -3346,10 +3381,10 @@
         <v>46232</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -3357,10 +3392,10 @@
         <v>46231</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
@@ -3368,10 +3403,10 @@
         <v>46232</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
@@ -3379,10 +3414,10 @@
         <v>46245</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
@@ -3390,10 +3425,10 @@
         <v>46246</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
@@ -3401,10 +3436,10 @@
         <v>46247</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
@@ -3412,7 +3447,7 @@
         <v>46254</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="D18" s="19"/>
     </row>
@@ -3547,15 +3582,15 @@
         <v>35</v>
       </c>
       <c r="C2" s="36" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -3584,30 +3619,30 @@
         <v>35</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>44</v>
@@ -3615,19 +3650,19 @@
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="127.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -3635,13 +3670,13 @@
         <v>67</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>70</v>
@@ -3649,19 +3684,19 @@
     </row>
     <row r="6" spans="2:6" ht="33" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -3690,7 +3725,7 @@
     <row r="3" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="67" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="C4" s="68"/>
       <c r="D4" s="39"/>
@@ -3702,7 +3737,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>14</v>
@@ -3711,37 +3746,37 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="40" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="D7" s="39"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="40" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="D8" s="39"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="40" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="D9" s="39"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="40" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="D10" s="39"/>
     </row>
@@ -3766,68 +3801,68 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update practice VPN account passwords from Excel
</commit_message>
<xml_diff>
--- a/솔루션실습 접속정보 관리.xlsx
+++ b/솔루션실습 접속정보 관리.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://okekr-my.sharepoint.com/personal/ws_choi_okekr_onmicrosoft_com/Documents/00.오케스트로 아카데미(아카데미팀 공유폴더)/기획운영 폴더/00. 팀 빌딩/AIDA/ACADEMY Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="796" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B46B07AA-B222-4582-99F2-803E86EE16C7}"/>
+  <xr:revisionPtr revIDLastSave="804" documentId="11_AD4D066CA252ABDACC10481411A76B9749B8DF56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC42C726-24ED-45AD-A22F-B412DF3701BF}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14415" yWindow="-21720" windowWidth="38640" windowHeight="21840" tabRatio="753" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="기본정보" sheetId="5" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="235">
   <si>
     <t>교육장 WiFi 정보</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -111,64 +111,25 @@
     <t>rydbr2o26-1</t>
   </si>
   <si>
-    <t>EB7TPP7wSqpx</t>
-  </si>
-  <si>
     <t>rydbr2o26-2</t>
   </si>
   <si>
-    <t>nMBFCxkWVak3</t>
-  </si>
-  <si>
     <t>rydbr2o26-3</t>
   </si>
   <si>
-    <t>z9rmYSbbkfvv</t>
-  </si>
-  <si>
     <t>rydbr2o26-4</t>
   </si>
   <si>
-    <t>Kb3cK2H1Fy97</t>
-  </si>
-  <si>
     <t>rydbr2o26-5</t>
   </si>
   <si>
-    <t>il1F98mduykO</t>
-  </si>
-  <si>
-    <t>rydbr2o26-6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0EpB9mbdEIQS</t>
-  </si>
-  <si>
     <t>rydbr2o26-7</t>
   </si>
   <si>
-    <t>91DDYymVM7jz</t>
-  </si>
-  <si>
     <t>rydbr2o26-8</t>
   </si>
   <si>
-    <t>Be6WoeM4w13H</t>
-  </si>
-  <si>
     <t>rydbr2o26-9</t>
-  </si>
-  <si>
-    <t>D9C373lsNy6F</t>
-  </si>
-  <si>
-    <t>rydbr2o26-10</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
-    <t>vw1W7i48l47Y</t>
-    <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
     <t>솔루션</t>
@@ -895,6 +856,46 @@
   <si>
     <t>EDU12</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://okekr-my.sharepoint.com/:f:/g/personal/ws_choi_okekr_onmicrosoft_com/IgB8nkzkDBddQrlOhYCI6LdoAVh3p5lvs4py_CDoApsayVI?e=XUSEl6</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>3W7ha1kmFO5R</t>
+  </si>
+  <si>
+    <t>lTBaTjDLflWa</t>
+  </si>
+  <si>
+    <t>kg6gZ3Bt8A4B</t>
+  </si>
+  <si>
+    <t>WBWY7D7eEF1W</t>
+  </si>
+  <si>
+    <t>uOzDBByIZZEt</t>
+  </si>
+  <si>
+    <t>rydbr2o26-6</t>
+  </si>
+  <si>
+    <t>cW7ynDiNUZYT</t>
+  </si>
+  <si>
+    <t>1phE1W3I2enW</t>
+  </si>
+  <si>
+    <t>NozFgNzQVS4o</t>
+  </si>
+  <si>
+    <t>I49DUaV2anrD</t>
+  </si>
+  <si>
+    <t>rydbr2o26-10</t>
+  </si>
+  <si>
+    <t>RKcuymWLiT7B</t>
   </si>
 </sst>
 </file>
@@ -993,7 +994,6 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Freesentation 4 Regular"/>
-      <charset val="129"/>
     </font>
     <font>
       <sz val="6"/>
@@ -1353,6 +1353,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1362,12 +1371,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1419,32 +1422,29 @@
     <xf numFmtId="0" fontId="12" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1762,10 +1762,10 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="44"/>
+      <c r="C4" s="42"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="19" t="s">
@@ -1784,10 +1784,10 @@
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="45"/>
+      <c r="C8" s="43"/>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="19" t="s">
@@ -1834,18 +1834,18 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="C3" s="14">
         <v>31300</v>
@@ -1856,7 +1856,7 @@
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="C4" s="14">
         <v>31301</v>
@@ -1867,7 +1867,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="C5" s="14">
         <v>31302</v>
@@ -1878,7 +1878,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="C6" s="14">
         <v>31303</v>
@@ -1889,7 +1889,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
       <c r="C7" s="14">
         <v>31304</v>
@@ -1900,7 +1900,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
       <c r="C8" s="21">
         <v>31305</v>
@@ -1911,7 +1911,7 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="C9" s="21">
         <v>31306</v>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
       <c r="C10" s="21">
         <v>31307</v>
@@ -1933,7 +1933,7 @@
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
       <c r="C11" s="21">
         <v>31308</v>
@@ -1944,7 +1944,7 @@
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
       <c r="C12" s="21">
         <v>31309</v>
@@ -1955,7 +1955,7 @@
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
-        <v>63</v>
+        <v>51</v>
       </c>
       <c r="C13" s="21">
         <v>31320</v>
@@ -1966,7 +1966,7 @@
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="C14" s="21">
         <v>31322</v>
@@ -1994,7 +1994,7 @@
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" s="31" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="C3" s="31" t="s">
         <v>1</v>
@@ -2008,47 +2008,47 @@
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B5" s="19"/>
       <c r="E5" s="20" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" s="19" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" s="19" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="E7" s="19"/>
     </row>
@@ -2108,12 +2108,12 @@
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D25" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2139,18 +2139,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="42" t="s">
+      <c r="B3" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
@@ -2171,7 +2171,7 @@
         <v>15</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>16</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -2179,10 +2179,10 @@
         <v>2</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>18</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -2190,10 +2190,10 @@
         <v>3</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>20</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -2201,10 +2201,10 @@
         <v>4</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>22</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -2212,10 +2212,10 @@
         <v>5</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>24</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -2223,10 +2223,10 @@
         <v>6</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>25</v>
+        <v>228</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>26</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -2234,10 +2234,10 @@
         <v>7</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>28</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
@@ -2245,10 +2245,10 @@
         <v>8</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>30</v>
+        <v>231</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -2256,10 +2256,10 @@
         <v>9</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>32</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
@@ -2267,10 +2267,10 @@
         <v>10</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>33</v>
+        <v>233</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>34</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
@@ -2278,10 +2278,10 @@
         <v>11</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2306,382 +2306,382 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="59" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="47" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" s="57"/>
+      <c r="C4" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="60"/>
+      <c r="F4" s="48"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B5" s="57"/>
+      <c r="C5" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D5" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="D2" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B3" s="55" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="58" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="46" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B4" s="56"/>
-      <c r="C4" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="E4" s="59"/>
-      <c r="F4" s="47"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B5" s="56"/>
-      <c r="C5" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" s="59"/>
-      <c r="F5" s="47"/>
+      <c r="E5" s="60"/>
+      <c r="F5" s="48"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="57"/>
+      <c r="C6" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="60"/>
+      <c r="F6" s="48"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B7" s="57"/>
+      <c r="C7" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="60"/>
+      <c r="F7" s="48"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B8" s="57"/>
+      <c r="C8" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="60"/>
+      <c r="F8" s="48"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B9" s="57"/>
+      <c r="C9" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="60"/>
+      <c r="F9" s="48"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B10" s="57"/>
+      <c r="C10" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="60"/>
+      <c r="F10" s="48"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B11" s="57"/>
+      <c r="C11" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="56"/>
-      <c r="C6" s="30" t="s">
+      <c r="E11" s="60"/>
+      <c r="F11" s="48"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="58"/>
+      <c r="C12" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D12" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="59"/>
-      <c r="F6" s="47"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B7" s="56"/>
-      <c r="C7" s="30" t="s">
+      <c r="E12" s="61"/>
+      <c r="F12" s="49"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="C13" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="59"/>
-      <c r="F7" s="47"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B8" s="56"/>
-      <c r="C8" s="30" t="s">
+      <c r="F13" s="50" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="59"/>
-      <c r="F8" s="47"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B9" s="56"/>
-      <c r="C9" s="30" t="s">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="54"/>
+      <c r="C14" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="48"/>
+      <c r="F14" s="51"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="54"/>
+      <c r="C15" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="E15" s="48"/>
+      <c r="F15" s="51"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="54"/>
+      <c r="C16" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="E16" s="48"/>
+      <c r="F16" s="51"/>
+    </row>
+    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B17" s="54"/>
+      <c r="C17" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E17" s="48"/>
+      <c r="F17" s="51"/>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B18" s="54"/>
+      <c r="C18" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" s="21" t="s">
+        <v>43</v>
+      </c>
+      <c r="E18" s="48"/>
+      <c r="F18" s="51"/>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B19" s="54"/>
+      <c r="C19" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="48"/>
+      <c r="F19" s="51"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B20" s="54"/>
+      <c r="C20" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="48"/>
+      <c r="F20" s="51"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B21" s="54"/>
+      <c r="C21" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E21" s="48"/>
+      <c r="F21" s="51"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B22" s="55"/>
+      <c r="C22" s="30" t="s">
+        <v>50</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="49"/>
+      <c r="F22" s="52"/>
+    </row>
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B23" s="53" t="s">
+        <v>214</v>
+      </c>
+      <c r="C23" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="E23" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="59"/>
-      <c r="F9" s="47"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B10" s="56"/>
-      <c r="C10" s="30" t="s">
+      <c r="F23" s="50" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="22" t="s">
+    </row>
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B24" s="54"/>
+      <c r="C24" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="D24" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="59"/>
-      <c r="F10" s="47"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B11" s="56"/>
-      <c r="C11" s="30" t="s">
+      <c r="E24" s="48"/>
+      <c r="F24" s="51"/>
+    </row>
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B25" s="54"/>
+      <c r="C25" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="E25" s="48"/>
+      <c r="F25" s="51"/>
+    </row>
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B26" s="54"/>
+      <c r="C26" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="59"/>
-      <c r="F11" s="47"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="57"/>
-      <c r="C12" s="30" t="s">
+      <c r="E26" s="48"/>
+      <c r="F26" s="51"/>
+    </row>
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B27" s="54"/>
+      <c r="C27" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="E27" s="48"/>
+      <c r="F27" s="51"/>
+    </row>
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B28" s="54"/>
+      <c r="C28" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="D28" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="60"/>
-      <c r="F12" s="48"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="52" t="s">
+      <c r="E28" s="48"/>
+      <c r="F28" s="51"/>
+    </row>
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B29" s="54"/>
+      <c r="C29" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" s="46" t="s">
+      <c r="E29" s="48"/>
+      <c r="F29" s="51"/>
+    </row>
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B30" s="54"/>
+      <c r="C30" s="30" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="F13" s="49" t="s">
+      <c r="E30" s="48"/>
+      <c r="F30" s="51"/>
+    </row>
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B31" s="54"/>
+      <c r="C31" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="D31" s="21" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B14" s="53"/>
-      <c r="C14" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="E14" s="47"/>
-      <c r="F14" s="50"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B15" s="53"/>
-      <c r="C15" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" s="47"/>
-      <c r="F15" s="50"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B16" s="53"/>
-      <c r="C16" s="30" t="s">
+      <c r="E31" s="48"/>
+      <c r="F31" s="51"/>
+    </row>
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B32" s="54"/>
+      <c r="C32" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E16" s="47"/>
-      <c r="F16" s="50"/>
-    </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="53"/>
-      <c r="C17" s="30" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="E17" s="47"/>
-      <c r="F17" s="50"/>
-    </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="53"/>
-      <c r="C18" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="E18" s="47"/>
-      <c r="F18" s="50"/>
-    </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="53"/>
-      <c r="C19" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" s="47"/>
-      <c r="F19" s="50"/>
-    </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B20" s="53"/>
-      <c r="C20" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="E20" s="47"/>
-      <c r="F20" s="50"/>
-    </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B21" s="53"/>
-      <c r="C21" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="E21" s="47"/>
-      <c r="F21" s="50"/>
-    </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B22" s="54"/>
-      <c r="C22" s="30" t="s">
-        <v>62</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="E22" s="48"/>
-      <c r="F22" s="51"/>
-    </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B23" s="52" t="s">
-        <v>226</v>
-      </c>
-      <c r="C23" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="E23" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="F23" s="49" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B24" s="53"/>
-      <c r="C24" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="E24" s="47"/>
-      <c r="F24" s="50"/>
-    </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B25" s="53"/>
-      <c r="C25" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E25" s="47"/>
-      <c r="F25" s="50"/>
-    </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B26" s="53"/>
-      <c r="C26" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="D26" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="E26" s="47"/>
-      <c r="F26" s="50"/>
-    </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B27" s="53"/>
-      <c r="C27" s="30" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" s="47"/>
-      <c r="F27" s="50"/>
-    </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B28" s="53"/>
-      <c r="C28" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E28" s="47"/>
-      <c r="F28" s="50"/>
-    </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B29" s="53"/>
-      <c r="C29" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E29" s="47"/>
-      <c r="F29" s="50"/>
-    </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B30" s="53"/>
-      <c r="C30" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="D30" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E30" s="47"/>
-      <c r="F30" s="50"/>
-    </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B31" s="53"/>
-      <c r="C31" s="30" t="s">
-        <v>60</v>
-      </c>
-      <c r="D31" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="E31" s="47"/>
-      <c r="F31" s="50"/>
-    </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B32" s="53"/>
-      <c r="C32" s="30" t="s">
-        <v>62</v>
-      </c>
       <c r="D32" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E32" s="47"/>
-      <c r="F32" s="50"/>
+        <v>67</v>
+      </c>
+      <c r="E32" s="48"/>
+      <c r="F32" s="51"/>
     </row>
     <row r="33" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B33" s="54"/>
+      <c r="B33" s="55"/>
       <c r="C33" s="30" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="E33" s="48"/>
-      <c r="F33" s="51"/>
+        <v>212</v>
+      </c>
+      <c r="E33" s="49"/>
+      <c r="F33" s="52"/>
     </row>
     <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="5"/>
@@ -2729,468 +2729,487 @@
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" s="68" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="69"/>
+    </row>
+    <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="66" t="s">
+        <v>73</v>
+      </c>
+      <c r="C5" s="66" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="66" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="66" t="s">
+        <v>76</v>
+      </c>
+      <c r="F5" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="67"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H6" s="27" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="D7" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="62" t="s">
+        <v>84</v>
+      </c>
+      <c r="F7" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="H7" s="27" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="63"/>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="66" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="66" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="66" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="63"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
+      <c r="E10" s="67"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H10" s="27" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="62" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="D11" s="62" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="F11" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="27" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="63"/>
+      <c r="C12" s="63"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="63"/>
+      <c r="F12" s="63"/>
+      <c r="G12" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F4" s="37" t="s">
-        <v>83</v>
-      </c>
-      <c r="G4" s="63" t="s">
-        <v>84</v>
-      </c>
-      <c r="H4" s="64"/>
-    </row>
-    <row r="5" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="65" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" s="65" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="65" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" s="65" t="s">
-        <v>88</v>
-      </c>
-      <c r="F5" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H6" s="27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="61" t="s">
+      <c r="H12" s="27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="62" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="66" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="66" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" s="66" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="63"/>
+      <c r="C14" s="67"/>
+      <c r="D14" s="67"/>
+      <c r="E14" s="67"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="62" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="61" t="s">
-        <v>94</v>
-      </c>
-      <c r="D7" s="61" t="s">
-        <v>95</v>
-      </c>
-      <c r="E7" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="F7" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="G7" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="27" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="61" t="s">
+      <c r="D15" s="66" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="66" t="s">
+        <v>100</v>
+      </c>
+      <c r="F15" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" s="27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="63"/>
+      <c r="C16" s="67"/>
+      <c r="D16" s="67"/>
+      <c r="E16" s="67"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="27" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="62" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="66" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="66" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H17" s="27" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="63"/>
+      <c r="C18" s="67"/>
+      <c r="D18" s="67"/>
+      <c r="E18" s="67"/>
+      <c r="F18" s="67"/>
+      <c r="G18" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H18" s="27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="62" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="65" t="s">
+      <c r="D19" s="62" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="62" t="s">
+        <v>108</v>
+      </c>
+      <c r="F19" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="H19" s="27" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="63"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="63"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="H20" s="27" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="65" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="65" t="s">
-        <v>100</v>
-      </c>
-      <c r="F9" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G9" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" s="27" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="62"/>
-      <c r="C10" s="66"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="66"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H10" s="27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="61" t="s">
+      <c r="C21" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="D21" s="66" t="s">
+        <v>111</v>
+      </c>
+      <c r="E21" s="66" t="s">
+        <v>112</v>
+      </c>
+      <c r="F21" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H21" s="27" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="63"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="67"/>
+      <c r="E22" s="67"/>
+      <c r="F22" s="67"/>
+      <c r="G22" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H22" s="27" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="61" t="s">
-        <v>103</v>
-      </c>
-      <c r="E11" s="61" t="s">
-        <v>104</v>
-      </c>
-      <c r="F11" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="G11" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" s="27" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="62"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" s="27" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="61" t="s">
+      <c r="C23" s="62" t="s">
+        <v>115</v>
+      </c>
+      <c r="D23" s="62" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" s="62" t="s">
+        <v>116</v>
+      </c>
+      <c r="F23" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G23" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="27" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="63"/>
+      <c r="C24" s="63"/>
+      <c r="D24" s="63"/>
+      <c r="E24" s="63"/>
+      <c r="F24" s="63"/>
+      <c r="G24" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="H24" s="27" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="62" t="s">
         <v>50</v>
       </c>
-      <c r="C13" s="65" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="65" t="s">
-        <v>107</v>
-      </c>
-      <c r="E13" s="65" t="s">
-        <v>108</v>
-      </c>
-      <c r="F13" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H13" s="27" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="62"/>
-      <c r="C14" s="66"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="66"/>
-      <c r="G14" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" s="27" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="61" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="65" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="65" t="s">
-        <v>111</v>
-      </c>
-      <c r="E15" s="65" t="s">
-        <v>112</v>
-      </c>
-      <c r="F15" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="27" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="16" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="62"/>
-      <c r="C16" s="66"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="66"/>
-      <c r="G16" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H16" s="27" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="17" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="61" t="s">
-        <v>54</v>
-      </c>
-      <c r="C17" s="65" t="s">
-        <v>55</v>
-      </c>
-      <c r="D17" s="65" t="s">
-        <v>115</v>
-      </c>
-      <c r="E17" s="65" t="s">
-        <v>116</v>
-      </c>
-      <c r="F17" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G17" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H17" s="27" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="62"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="66"/>
-      <c r="G18" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H18" s="27" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="61" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="61" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="61" t="s">
+      <c r="C25" s="66" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="61" t="s">
-        <v>120</v>
-      </c>
-      <c r="F19" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="G19" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" s="27" t="s">
+      <c r="D25" s="66" t="s">
+        <v>219</v>
+      </c>
+      <c r="E25" s="66" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="62"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="62"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="62"/>
-      <c r="G20" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H20" s="27" t="s">
+      <c r="F25" s="66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G25" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="27" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="21" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="C21" s="65" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="65" t="s">
+    <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="63"/>
+      <c r="C26" s="67"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="67"/>
+      <c r="G26" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="H26" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="E21" s="65" t="s">
-        <v>124</v>
-      </c>
-      <c r="F21" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G21" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="62"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="23" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="61" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="61" t="s">
-        <v>127</v>
-      </c>
-      <c r="D23" s="61" t="s">
-        <v>132</v>
-      </c>
-      <c r="E23" s="61" t="s">
-        <v>128</v>
-      </c>
-      <c r="F23" s="61" t="s">
-        <v>89</v>
-      </c>
-      <c r="G23" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="62"/>
-      <c r="C24" s="62"/>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="62"/>
-      <c r="G24" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" s="27" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="61" t="s">
-        <v>62</v>
-      </c>
-      <c r="C25" s="65" t="s">
-        <v>131</v>
-      </c>
-      <c r="D25" s="65" t="s">
-        <v>231</v>
-      </c>
-      <c r="E25" s="65" t="s">
-        <v>133</v>
-      </c>
-      <c r="F25" s="65" t="s">
-        <v>89</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" s="27" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="62"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="66"/>
-      <c r="G26" s="25" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" s="27" t="s">
-        <v>135</v>
-      </c>
     </row>
     <row r="27" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="61" t="s">
-        <v>229</v>
-      </c>
-      <c r="C27" s="69" t="s">
-        <v>230</v>
-      </c>
-      <c r="D27" s="69" t="s">
-        <v>232</v>
-      </c>
-      <c r="E27" s="69" t="s">
-        <v>233</v>
-      </c>
-      <c r="F27" s="69" t="s">
-        <v>89</v>
-      </c>
-      <c r="G27" s="70" t="s">
-        <v>90</v>
+      <c r="B27" s="62" t="s">
+        <v>217</v>
+      </c>
+      <c r="C27" s="64" t="s">
+        <v>218</v>
+      </c>
+      <c r="D27" s="64" t="s">
+        <v>220</v>
+      </c>
+      <c r="E27" s="64" t="s">
+        <v>221</v>
+      </c>
+      <c r="F27" s="64" t="s">
+        <v>77</v>
+      </c>
+      <c r="G27" s="41" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="62"/>
-      <c r="C28" s="71"/>
-      <c r="D28" s="71"/>
-      <c r="E28" s="71"/>
-      <c r="F28" s="71"/>
-      <c r="G28" s="70" t="s">
-        <v>92</v>
+      <c r="B28" s="63"/>
+      <c r="C28" s="65"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="65"/>
+      <c r="G28" s="41" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="D25:D26"/>
@@ -3203,40 +3222,21 @@
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -3279,10 +3279,10 @@
   <sheetData>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="33" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="D3" s="31" t="s">
         <v>6</v>
@@ -3293,10 +3293,10 @@
         <v>46217</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -3304,10 +3304,10 @@
         <v>46218</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -3315,10 +3315,10 @@
         <v>46224</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -3326,10 +3326,10 @@
         <v>46225</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -3337,10 +3337,10 @@
         <v>46230</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -3348,10 +3348,10 @@
         <v>46231</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -3359,10 +3359,10 @@
         <v>46232</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
@@ -3370,10 +3370,10 @@
         <v>46232</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.3">
@@ -3381,10 +3381,10 @@
         <v>46232</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.3">
@@ -3392,10 +3392,10 @@
         <v>46231</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.3">
@@ -3403,10 +3403,10 @@
         <v>46232</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.3">
@@ -3414,10 +3414,10 @@
         <v>46245</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.3">
@@ -3425,10 +3425,10 @@
         <v>46246</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.3">
@@ -3436,10 +3436,10 @@
         <v>46247</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.3">
@@ -3447,9 +3447,11 @@
         <v>46254</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="D18" s="19"/>
+        <v>141</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>222</v>
+      </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19" s="34"/>
@@ -3563,6 +3565,7 @@
     <hyperlink ref="D16" r:id="rId12" xr:uid="{E0D720A5-AAC0-4D45-A438-1661E9E19884}"/>
     <hyperlink ref="D15" r:id="rId13" xr:uid="{364B1836-E2AB-4E20-9CB5-D46DC6CA0FA9}"/>
     <hyperlink ref="D17" r:id="rId14" xr:uid="{16585DE6-F99F-4F45-AD9B-6D6451BD1173}"/>
+    <hyperlink ref="D18" r:id="rId15" xr:uid="{1EF95B5D-84D8-4D3B-8903-B6637CAA6137}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3579,18 +3582,18 @@
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="36" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C2" s="36" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3616,87 +3619,87 @@
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B2" s="9" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="2:6" ht="127.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="33" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.3">
@@ -3724,10 +3727,10 @@
   <sheetData>
     <row r="3" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:4" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="67" t="s">
-        <v>178</v>
-      </c>
-      <c r="C4" s="68"/>
+      <c r="B4" s="70" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="71"/>
       <c r="D4" s="39"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
@@ -3737,7 +3740,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="16" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="C6" s="17" t="s">
         <v>14</v>
@@ -3746,37 +3749,37 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="40" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="D7" s="39"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" s="40" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="D8" s="39"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B9" s="40" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D9" s="39"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B10" s="40" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="D10" s="39"/>
     </row>
@@ -3801,68 +3804,68 @@
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="13" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" s="6" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>